<commit_message>
Atualização automática: motores (15/07/2026 16:12)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1303,16 +1303,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1328,7 +1320,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1336,30 +1328,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1659,70 +1633,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1763,10 +1737,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1778,7 +1752,7 @@
       <c r="T2" t="s">
         <v>147</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1819,10 +1793,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1869,10 +1843,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1919,10 +1893,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1934,7 +1908,7 @@
       <c r="T5" t="s">
         <v>148</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -1972,10 +1946,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2022,10 +1996,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2037,7 +2011,7 @@
       <c r="T7" t="s">
         <v>149</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2078,10 +2052,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2128,10 +2102,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2143,7 +2117,7 @@
       <c r="T9" t="s">
         <v>150</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2184,10 +2158,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2228,10 +2202,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2243,7 +2217,7 @@
       <c r="T11" t="s">
         <v>151</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46203</v>
       </c>
     </row>
@@ -2281,7 +2255,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2322,10 +2296,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2369,10 +2343,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2384,7 +2358,7 @@
       <c r="T14" t="s">
         <v>152</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2425,10 +2399,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2475,10 +2449,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2490,7 +2464,7 @@
       <c r="T16" t="s">
         <v>153</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2531,10 +2505,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2581,10 +2555,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2596,7 +2570,7 @@
       <c r="T18" t="s">
         <v>154</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2637,10 +2611,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2652,7 +2626,7 @@
       <c r="T19" t="s">
         <v>122</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
       <c r="V19">
@@ -2696,10 +2670,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2711,7 +2685,7 @@
       <c r="T20" t="s">
         <v>155</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2752,10 +2726,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2767,7 +2741,7 @@
       <c r="T21" t="s">
         <v>124</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2808,10 +2782,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2823,7 +2797,7 @@
       <c r="T22" t="s">
         <v>156</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2861,10 +2835,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2873,7 +2847,7 @@
       <c r="S23" t="s">
         <v>146</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -2914,10 +2888,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45925</v>
       </c>
       <c r="R24" t="s">
@@ -2964,10 +2938,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3014,10 +2988,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3029,7 +3003,7 @@
       <c r="T26" t="s">
         <v>157</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3070,10 +3044,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3120,10 +3094,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3170,10 +3144,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3220,10 +3194,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3235,7 +3209,7 @@
       <c r="T30" t="s">
         <v>158</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3276,10 +3250,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46064</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46064</v>
       </c>
       <c r="R31" t="s">
@@ -3326,10 +3300,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3376,10 +3350,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3391,7 +3365,7 @@
       <c r="T33" t="s">
         <v>159</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3432,10 +3406,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3482,10 +3456,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3532,10 +3506,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3582,10 +3556,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3597,7 +3571,7 @@
       <c r="T37" t="s">
         <v>160</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3638,10 +3612,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>45579</v>
       </c>
       <c r="S38" t="s">
@@ -3685,10 +3659,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3732,10 +3706,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3756,22 +3730,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>162</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>163</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>164</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>165</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>166</v>
       </c>
     </row>
@@ -7951,91 +7925,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>226</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>227</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>228</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>229</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>230</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>231</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>232</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>233</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>234</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>235</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>236</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>237</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>238</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>239</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>240</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>241</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>242</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>243</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>244</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>245</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>246</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>247</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>248</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>249</v>
       </c>
     </row>
@@ -8049,13 +8023,13 @@
       <c r="D2" t="s">
         <v>252</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>255</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8073,13 +8047,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8117,13 +8091,13 @@
       <c r="D3" t="s">
         <v>253</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>255</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8141,13 +8115,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8182,13 +8156,13 @@
       <c r="D4" t="s">
         <v>253</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>255</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8206,13 +8180,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8247,13 +8221,13 @@
       <c r="D5" t="s">
         <v>253</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>255</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8271,13 +8245,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8315,13 +8289,13 @@
       <c r="D6" t="s">
         <v>253</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>255</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8339,13 +8313,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8383,7 +8357,7 @@
       <c r="D7" t="s">
         <v>254</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8404,10 +8378,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8445,7 +8419,7 @@
       <c r="D8" t="s">
         <v>254</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8466,10 +8440,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8507,7 +8481,7 @@
       <c r="D9" t="s">
         <v>254</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8528,10 +8502,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8569,13 +8543,13 @@
       <c r="D10" t="s">
         <v>253</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>255</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8593,13 +8567,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8634,13 +8608,13 @@
       <c r="D11" t="s">
         <v>253</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>255</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8658,13 +8632,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8699,13 +8673,13 @@
       <c r="D12" t="s">
         <v>253</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>255</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8723,13 +8697,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8764,13 +8738,13 @@
       <c r="D13" t="s">
         <v>253</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>255</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8788,13 +8762,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8832,13 +8806,13 @@
       <c r="D14" t="s">
         <v>253</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>255</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8856,13 +8830,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -8898,70 +8872,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -8999,10 +8973,10 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9046,10 +9020,10 @@
       <c r="O3" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9093,10 +9067,10 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9140,10 +9114,10 @@
       <c r="O5" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9187,10 +9161,10 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9234,10 +9208,10 @@
       <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9281,10 +9255,10 @@
       <c r="O8" t="s">
         <v>103</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9328,10 +9302,10 @@
       <c r="O9" t="s">
         <v>92</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9375,10 +9349,10 @@
       <c r="O10" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9422,10 +9396,10 @@
       <c r="O11" t="s">
         <v>99</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9469,10 +9443,10 @@
       <c r="O12" t="s">
         <v>82</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9516,10 +9490,10 @@
       <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9563,10 +9537,10 @@
       <c r="O14" t="s">
         <v>100</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9610,7 +9584,7 @@
       <c r="O15" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9651,7 +9625,7 @@
       <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9692,10 +9666,10 @@
       <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9739,10 +9713,10 @@
       <c r="O18" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9786,10 +9760,10 @@
       <c r="O19" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9833,10 +9807,10 @@
       <c r="O20" t="s">
         <v>96</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -9880,10 +9854,10 @@
       <c r="O21" t="s">
         <v>105</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9927,10 +9901,10 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9968,10 +9942,10 @@
       <c r="O23" t="s">
         <v>356</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -9983,7 +9957,7 @@
       <c r="T23" t="s">
         <v>396</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10021,10 +9995,10 @@
       <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10036,7 +10010,7 @@
       <c r="T24" t="s">
         <v>397</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10074,10 +10048,10 @@
       <c r="O25" t="s">
         <v>86</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10089,7 +10063,7 @@
       <c r="T25" t="s">
         <v>398</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10127,10 +10101,10 @@
       <c r="O26" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10142,7 +10116,7 @@
       <c r="T26" t="s">
         <v>399</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10180,10 +10154,10 @@
       <c r="O27" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10195,7 +10169,7 @@
       <c r="T27" t="s">
         <v>400</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10233,10 +10207,10 @@
       <c r="O28" t="s">
         <v>101</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10248,7 +10222,7 @@
       <c r="T28" t="s">
         <v>401</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10286,10 +10260,10 @@
       <c r="O29" t="s">
         <v>98</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10301,7 +10275,7 @@
       <c r="T29" t="s">
         <v>402</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10333,7 +10307,7 @@
       <c r="T30" t="s">
         <v>403</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10365,7 +10339,7 @@
       <c r="T31" t="s">
         <v>404</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10397,7 +10371,7 @@
       <c r="T32" t="s">
         <v>405</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10435,10 +10409,10 @@
       <c r="O33" t="s">
         <v>90</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10450,7 +10424,7 @@
       <c r="T33" t="s">
         <v>384</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10488,16 +10462,16 @@
       <c r="O34" t="s">
         <v>357</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>146</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10529,10 +10503,10 @@
       <c r="O35" t="s">
         <v>87</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10541,7 +10515,7 @@
       <c r="S35" t="s">
         <v>146</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10579,10 +10553,10 @@
       <c r="O36" t="s">
         <v>91</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10591,7 +10565,7 @@
       <c r="S36" t="s">
         <v>146</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10655,10 +10629,10 @@
       <c r="O38" t="s">
         <v>96</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10667,7 +10641,7 @@
       <c r="S38" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10705,10 +10679,10 @@
       <c r="O39" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10720,7 +10694,7 @@
       <c r="T39" t="s">
         <v>406</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10752,10 +10726,10 @@
       <c r="O40" t="s">
         <v>100</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10767,7 +10741,7 @@
       <c r="T40" t="s">
         <v>407</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -10805,10 +10779,10 @@
       <c r="O41" t="s">
         <v>95</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10820,7 +10794,7 @@
       <c r="T41" t="s">
         <v>408</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -10858,10 +10832,10 @@
       <c r="O42" t="s">
         <v>82</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -10873,7 +10847,7 @@
       <c r="T42" t="s">
         <v>409</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -10911,10 +10885,10 @@
       <c r="O43" t="s">
         <v>84</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10926,7 +10900,7 @@
       <c r="T43" t="s">
         <v>410</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -10964,10 +10938,10 @@
       <c r="O44" t="s">
         <v>97</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10979,7 +10953,7 @@
       <c r="T44" t="s">
         <v>411</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11017,10 +10991,10 @@
       <c r="O45" t="s">
         <v>81</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11032,7 +11006,7 @@
       <c r="T45" t="s">
         <v>412</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11070,10 +11044,10 @@
       <c r="O46" t="s">
         <v>88</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11085,7 +11059,7 @@
       <c r="T46" t="s">
         <v>413</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11100,25 +11074,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>162</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>414</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>415</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>416</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>417</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>418</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (16/07/2026 16:04)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -575,7 +575,7 @@
     <t>19.2</t>
   </si>
   <si>
-    <t>2.974628583</t>
+    <t>29.77939946</t>
   </si>
   <si>
     <t>5.1586629</t>
@@ -4906,13 +4906,13 @@
         <v>2729</v>
       </c>
       <c r="C68">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="D68">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E68" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -11302,7 +11302,7 @@
         <v>2832.83</v>
       </c>
       <c r="D11">
-        <v>313.1666667</v>
+        <v>1167.166667</v>
       </c>
       <c r="E11">
         <v>39.70818182</v>
@@ -11311,7 +11311,7 @@
         <v>218.395</v>
       </c>
       <c r="G11">
-        <v>7.886703755</v>
+        <v>29.39360639</v>
       </c>
     </row>
     <row r="12" spans="1:7">

</xml_diff>

<commit_message>
Atualização automática: motores (22/07/2026 12:04)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1312,8 +1312,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1329,7 +1337,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1337,12 +1345,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1642,70 +1668,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1746,10 +1772,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1761,7 +1787,7 @@
       <c r="T2" t="s">
         <v>148</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1802,10 +1828,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1852,10 +1878,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1902,10 +1928,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1917,7 +1943,7 @@
       <c r="T5" t="s">
         <v>149</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -1955,10 +1981,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2005,10 +2031,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2020,7 +2046,7 @@
       <c r="T7" t="s">
         <v>150</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -2061,10 +2087,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2111,10 +2137,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2126,7 +2152,7 @@
       <c r="T9" t="s">
         <v>151</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2167,10 +2193,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2211,10 +2237,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2226,7 +2252,7 @@
       <c r="T11" t="s">
         <v>152</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46203</v>
       </c>
     </row>
@@ -2264,7 +2290,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2305,10 +2331,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2352,10 +2378,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2367,7 +2393,7 @@
       <c r="T14" t="s">
         <v>153</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2408,10 +2434,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2458,10 +2484,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2473,7 +2499,7 @@
       <c r="T16" t="s">
         <v>154</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2514,10 +2540,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2564,10 +2590,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2579,7 +2605,7 @@
       <c r="T18" t="s">
         <v>155</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2620,10 +2646,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2635,7 +2661,7 @@
       <c r="T19" t="s">
         <v>122</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46153</v>
       </c>
       <c r="V19">
@@ -2679,10 +2705,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2694,7 +2720,7 @@
       <c r="T20" t="s">
         <v>156</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2735,10 +2761,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2750,7 +2776,7 @@
       <c r="T21" t="s">
         <v>124</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2791,10 +2817,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2806,7 +2832,7 @@
       <c r="T22" t="s">
         <v>157</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2844,10 +2870,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2856,7 +2882,7 @@
       <c r="S23" t="s">
         <v>146</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -2897,10 +2923,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45925</v>
       </c>
       <c r="R24" t="s">
@@ -2947,10 +2973,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -2997,10 +3023,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3012,7 +3038,7 @@
       <c r="T26" t="s">
         <v>158</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -3053,10 +3079,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3103,10 +3129,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3153,10 +3179,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3203,10 +3229,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3218,7 +3244,7 @@
       <c r="T30" t="s">
         <v>159</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3259,10 +3285,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46064</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46064</v>
       </c>
       <c r="R31" t="s">
@@ -3309,10 +3335,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3359,10 +3385,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3374,7 +3400,7 @@
       <c r="T33" t="s">
         <v>160</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3415,10 +3441,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3465,10 +3491,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3515,10 +3541,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3565,10 +3591,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3580,7 +3606,7 @@
       <c r="T37" t="s">
         <v>161</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3621,10 +3647,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>45579</v>
       </c>
       <c r="S38" t="s">
@@ -3671,10 +3697,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3718,10 +3744,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3742,22 +3768,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>168</v>
       </c>
     </row>
@@ -7971,91 +7997,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>252</v>
       </c>
     </row>
@@ -8069,13 +8095,13 @@
       <c r="D2" t="s">
         <v>255</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>258</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8093,13 +8119,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45491</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <v>45528</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8137,13 +8163,13 @@
       <c r="D3" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>258</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8161,13 +8187,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45628</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>45632</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8202,13 +8228,13 @@
       <c r="D4" t="s">
         <v>256</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8226,13 +8252,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45716</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <v>45722</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="2">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8267,13 +8293,13 @@
       <c r="D5" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8291,13 +8317,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45722</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <v>45782</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8335,13 +8361,13 @@
       <c r="D6" t="s">
         <v>256</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>258</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8359,13 +8385,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45728</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>45734</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8403,7 +8429,7 @@
       <c r="D7" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8424,10 +8450,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45772</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8465,7 +8491,7 @@
       <c r="D8" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8486,10 +8512,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>45762</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="2">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8527,7 +8553,7 @@
       <c r="D9" t="s">
         <v>257</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8548,10 +8574,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45763</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8589,13 +8615,13 @@
       <c r="D10" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="2">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8613,13 +8639,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45754</v>
       </c>
-      <c r="R10" s="1">
+      <c r="R10" s="2">
         <v>45849</v>
       </c>
-      <c r="S10" s="1">
+      <c r="S10" s="2">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8654,13 +8680,13 @@
       <c r="D11" t="s">
         <v>256</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>258</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="2">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8678,13 +8704,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44973</v>
       </c>
-      <c r="R11" s="1">
+      <c r="R11" s="2">
         <v>45687</v>
       </c>
-      <c r="S11" s="1">
+      <c r="S11" s="2">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8719,13 +8745,13 @@
       <c r="D12" t="s">
         <v>256</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>258</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="2">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8743,13 +8769,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45358</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="2">
         <v>45517</v>
       </c>
-      <c r="S12" s="1">
+      <c r="S12" s="2">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8784,13 +8810,13 @@
       <c r="D13" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>258</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="2">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8808,13 +8834,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45572</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="2">
         <v>45572</v>
       </c>
-      <c r="S13" s="1">
+      <c r="S13" s="2">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8852,13 +8878,13 @@
       <c r="D14" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>258</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="2">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8876,13 +8902,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>45736</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="2">
         <v>46101</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="2">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -8918,70 +8944,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9019,10 +9045,10 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9066,10 +9092,10 @@
       <c r="O3" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9113,10 +9139,10 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9160,10 +9186,10 @@
       <c r="O5" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9207,10 +9233,10 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9254,10 +9280,10 @@
       <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9301,10 +9327,10 @@
       <c r="O8" t="s">
         <v>103</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9348,10 +9374,10 @@
       <c r="O9" t="s">
         <v>92</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9395,10 +9421,10 @@
       <c r="O10" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9442,10 +9468,10 @@
       <c r="O11" t="s">
         <v>99</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9489,10 +9515,10 @@
       <c r="O12" t="s">
         <v>82</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9536,10 +9562,10 @@
       <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9583,10 +9609,10 @@
       <c r="O14" t="s">
         <v>100</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9630,7 +9656,7 @@
       <c r="O15" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9671,7 +9697,7 @@
       <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9712,10 +9738,10 @@
       <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9759,10 +9785,10 @@
       <c r="O18" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9806,10 +9832,10 @@
       <c r="O19" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9853,10 +9879,10 @@
       <c r="O20" t="s">
         <v>96</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -9900,10 +9926,10 @@
       <c r="O21" t="s">
         <v>105</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9947,10 +9973,10 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9988,10 +10014,10 @@
       <c r="O23" t="s">
         <v>359</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10003,7 +10029,7 @@
       <c r="T23" t="s">
         <v>399</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -10041,10 +10067,10 @@
       <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10056,7 +10082,7 @@
       <c r="T24" t="s">
         <v>400</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -10094,10 +10120,10 @@
       <c r="O25" t="s">
         <v>86</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10109,7 +10135,7 @@
       <c r="T25" t="s">
         <v>401</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -10147,10 +10173,10 @@
       <c r="O26" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10162,7 +10188,7 @@
       <c r="T26" t="s">
         <v>402</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -10200,10 +10226,10 @@
       <c r="O27" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10215,7 +10241,7 @@
       <c r="T27" t="s">
         <v>403</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -10253,10 +10279,10 @@
       <c r="O28" t="s">
         <v>101</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10268,7 +10294,7 @@
       <c r="T28" t="s">
         <v>404</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -10306,10 +10332,10 @@
       <c r="O29" t="s">
         <v>98</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10321,7 +10347,7 @@
       <c r="T29" t="s">
         <v>405</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -10353,7 +10379,7 @@
       <c r="T30" t="s">
         <v>406</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10385,7 +10411,7 @@
       <c r="T31" t="s">
         <v>407</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10417,7 +10443,7 @@
       <c r="T32" t="s">
         <v>408</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10455,10 +10481,10 @@
       <c r="O33" t="s">
         <v>90</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10470,7 +10496,7 @@
       <c r="T33" t="s">
         <v>387</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -10508,16 +10534,16 @@
       <c r="O34" t="s">
         <v>360</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>146</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -10549,10 +10575,10 @@
       <c r="O35" t="s">
         <v>87</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10561,7 +10587,7 @@
       <c r="S35" t="s">
         <v>146</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -10599,10 +10625,10 @@
       <c r="O36" t="s">
         <v>91</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10611,7 +10637,7 @@
       <c r="S36" t="s">
         <v>146</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -10675,10 +10701,10 @@
       <c r="O38" t="s">
         <v>96</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10687,7 +10713,7 @@
       <c r="S38" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -10725,10 +10751,10 @@
       <c r="O39" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10740,7 +10766,7 @@
       <c r="T39" t="s">
         <v>409</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -10772,10 +10798,10 @@
       <c r="O40" t="s">
         <v>100</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10787,7 +10813,7 @@
       <c r="T40" t="s">
         <v>410</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -10825,10 +10851,10 @@
       <c r="O41" t="s">
         <v>95</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10840,7 +10866,7 @@
       <c r="T41" t="s">
         <v>411</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -10878,10 +10904,10 @@
       <c r="O42" t="s">
         <v>82</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -10893,7 +10919,7 @@
       <c r="T42" t="s">
         <v>412</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -10931,10 +10957,10 @@
       <c r="O43" t="s">
         <v>84</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10946,7 +10972,7 @@
       <c r="T43" t="s">
         <v>413</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -10984,10 +11010,10 @@
       <c r="O44" t="s">
         <v>97</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10999,7 +11025,7 @@
       <c r="T44" t="s">
         <v>414</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -11037,10 +11063,10 @@
       <c r="O45" t="s">
         <v>81</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11052,7 +11078,7 @@
       <c r="T45" t="s">
         <v>415</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -11090,10 +11116,10 @@
       <c r="O46" t="s">
         <v>88</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11105,7 +11131,7 @@
       <c r="T46" t="s">
         <v>416</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -11120,25 +11146,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>421</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (22/07/2026 16:11)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1312,16 +1312,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1337,7 +1329,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1345,30 +1337,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1668,70 +1642,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1772,10 +1746,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1787,7 +1761,7 @@
       <c r="T2" t="s">
         <v>148</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1828,10 +1802,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1878,10 +1852,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1928,10 +1902,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1943,7 +1917,7 @@
       <c r="T5" t="s">
         <v>149</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -1981,10 +1955,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2031,10 +2005,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2046,7 +2020,7 @@
       <c r="T7" t="s">
         <v>150</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2087,10 +2061,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2137,10 +2111,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2152,7 +2126,7 @@
       <c r="T9" t="s">
         <v>151</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2193,10 +2167,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2237,10 +2211,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2252,7 +2226,7 @@
       <c r="T11" t="s">
         <v>152</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46203</v>
       </c>
     </row>
@@ -2290,7 +2264,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2331,10 +2305,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2378,10 +2352,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2393,7 +2367,7 @@
       <c r="T14" t="s">
         <v>153</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2434,10 +2408,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2484,10 +2458,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2499,7 +2473,7 @@
       <c r="T16" t="s">
         <v>154</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2540,10 +2514,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2590,10 +2564,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2605,7 +2579,7 @@
       <c r="T18" t="s">
         <v>155</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2646,10 +2620,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2661,7 +2635,7 @@
       <c r="T19" t="s">
         <v>122</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
       <c r="V19">
@@ -2705,10 +2679,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2720,7 +2694,7 @@
       <c r="T20" t="s">
         <v>156</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2761,10 +2735,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2776,7 +2750,7 @@
       <c r="T21" t="s">
         <v>124</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2817,10 +2791,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2832,7 +2806,7 @@
       <c r="T22" t="s">
         <v>157</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2870,10 +2844,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2882,7 +2856,7 @@
       <c r="S23" t="s">
         <v>146</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -2923,10 +2897,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45925</v>
       </c>
       <c r="R24" t="s">
@@ -2973,10 +2947,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3023,10 +2997,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3038,7 +3012,7 @@
       <c r="T26" t="s">
         <v>158</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3079,10 +3053,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3129,10 +3103,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3179,10 +3153,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3229,10 +3203,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3244,7 +3218,7 @@
       <c r="T30" t="s">
         <v>159</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3285,10 +3259,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46064</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46064</v>
       </c>
       <c r="R31" t="s">
@@ -3335,10 +3309,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3385,10 +3359,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3400,7 +3374,7 @@
       <c r="T33" t="s">
         <v>160</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3441,10 +3415,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3491,10 +3465,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3541,10 +3515,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3591,10 +3565,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3606,7 +3580,7 @@
       <c r="T37" t="s">
         <v>161</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3647,10 +3621,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>45579</v>
       </c>
       <c r="S38" t="s">
@@ -3697,10 +3671,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3744,10 +3718,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3768,22 +3742,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>166</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>167</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>168</v>
       </c>
     </row>
@@ -7997,91 +7971,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>229</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>230</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>231</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>232</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>233</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>234</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>235</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>236</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>237</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>238</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>239</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>240</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>241</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>242</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>243</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>244</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>245</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>246</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>247</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>248</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>249</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>250</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>251</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>252</v>
       </c>
     </row>
@@ -8095,13 +8069,13 @@
       <c r="D2" t="s">
         <v>255</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>258</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8119,13 +8093,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8163,13 +8137,13 @@
       <c r="D3" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>258</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8187,13 +8161,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8228,13 +8202,13 @@
       <c r="D4" t="s">
         <v>256</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8252,13 +8226,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8293,13 +8267,13 @@
       <c r="D5" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8317,13 +8291,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8361,13 +8335,13 @@
       <c r="D6" t="s">
         <v>256</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>258</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8385,13 +8359,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8429,7 +8403,7 @@
       <c r="D7" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8450,10 +8424,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8491,7 +8465,7 @@
       <c r="D8" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8512,10 +8486,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8553,7 +8527,7 @@
       <c r="D9" t="s">
         <v>257</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8574,10 +8548,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8615,13 +8589,13 @@
       <c r="D10" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8639,13 +8613,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8680,13 +8654,13 @@
       <c r="D11" t="s">
         <v>256</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>258</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8704,13 +8678,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8745,13 +8719,13 @@
       <c r="D12" t="s">
         <v>256</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>258</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8769,13 +8743,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8810,13 +8784,13 @@
       <c r="D13" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>258</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8834,13 +8808,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8878,13 +8852,13 @@
       <c r="D14" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>258</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8902,13 +8876,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -8944,70 +8918,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9045,10 +9019,10 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9092,10 +9066,10 @@
       <c r="O3" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9139,10 +9113,10 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9186,10 +9160,10 @@
       <c r="O5" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9233,10 +9207,10 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9280,10 +9254,10 @@
       <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9327,10 +9301,10 @@
       <c r="O8" t="s">
         <v>103</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9374,10 +9348,10 @@
       <c r="O9" t="s">
         <v>92</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9421,10 +9395,10 @@
       <c r="O10" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9468,10 +9442,10 @@
       <c r="O11" t="s">
         <v>99</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9515,10 +9489,10 @@
       <c r="O12" t="s">
         <v>82</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9562,10 +9536,10 @@
       <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9609,10 +9583,10 @@
       <c r="O14" t="s">
         <v>100</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9656,7 +9630,7 @@
       <c r="O15" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9697,7 +9671,7 @@
       <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9738,10 +9712,10 @@
       <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9785,10 +9759,10 @@
       <c r="O18" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9832,10 +9806,10 @@
       <c r="O19" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9879,10 +9853,10 @@
       <c r="O20" t="s">
         <v>96</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -9926,10 +9900,10 @@
       <c r="O21" t="s">
         <v>105</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9973,10 +9947,10 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10014,10 +9988,10 @@
       <c r="O23" t="s">
         <v>359</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10029,7 +10003,7 @@
       <c r="T23" t="s">
         <v>399</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10067,10 +10041,10 @@
       <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10082,7 +10056,7 @@
       <c r="T24" t="s">
         <v>400</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10120,10 +10094,10 @@
       <c r="O25" t="s">
         <v>86</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10135,7 +10109,7 @@
       <c r="T25" t="s">
         <v>401</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10173,10 +10147,10 @@
       <c r="O26" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10188,7 +10162,7 @@
       <c r="T26" t="s">
         <v>402</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10226,10 +10200,10 @@
       <c r="O27" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10241,7 +10215,7 @@
       <c r="T27" t="s">
         <v>403</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10279,10 +10253,10 @@
       <c r="O28" t="s">
         <v>101</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10294,7 +10268,7 @@
       <c r="T28" t="s">
         <v>404</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10332,10 +10306,10 @@
       <c r="O29" t="s">
         <v>98</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10347,7 +10321,7 @@
       <c r="T29" t="s">
         <v>405</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10379,7 +10353,7 @@
       <c r="T30" t="s">
         <v>406</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10411,7 +10385,7 @@
       <c r="T31" t="s">
         <v>407</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10443,7 +10417,7 @@
       <c r="T32" t="s">
         <v>408</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10481,10 +10455,10 @@
       <c r="O33" t="s">
         <v>90</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10496,7 +10470,7 @@
       <c r="T33" t="s">
         <v>387</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10534,16 +10508,16 @@
       <c r="O34" t="s">
         <v>360</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>146</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10575,10 +10549,10 @@
       <c r="O35" t="s">
         <v>87</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10587,7 +10561,7 @@
       <c r="S35" t="s">
         <v>146</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10625,10 +10599,10 @@
       <c r="O36" t="s">
         <v>91</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10637,7 +10611,7 @@
       <c r="S36" t="s">
         <v>146</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10701,10 +10675,10 @@
       <c r="O38" t="s">
         <v>96</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10713,7 +10687,7 @@
       <c r="S38" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10751,10 +10725,10 @@
       <c r="O39" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10766,7 +10740,7 @@
       <c r="T39" t="s">
         <v>409</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10798,10 +10772,10 @@
       <c r="O40" t="s">
         <v>100</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10813,7 +10787,7 @@
       <c r="T40" t="s">
         <v>410</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -10851,10 +10825,10 @@
       <c r="O41" t="s">
         <v>95</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10866,7 +10840,7 @@
       <c r="T41" t="s">
         <v>411</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -10904,10 +10878,10 @@
       <c r="O42" t="s">
         <v>82</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -10919,7 +10893,7 @@
       <c r="T42" t="s">
         <v>412</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -10957,10 +10931,10 @@
       <c r="O43" t="s">
         <v>84</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10972,7 +10946,7 @@
       <c r="T43" t="s">
         <v>413</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -11010,10 +10984,10 @@
       <c r="O44" t="s">
         <v>97</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11025,7 +10999,7 @@
       <c r="T44" t="s">
         <v>414</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11063,10 +11037,10 @@
       <c r="O45" t="s">
         <v>81</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11078,7 +11052,7 @@
       <c r="T45" t="s">
         <v>415</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11116,10 +11090,10 @@
       <c r="O46" t="s">
         <v>88</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11131,7 +11105,7 @@
       <c r="T46" t="s">
         <v>416</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11146,25 +11120,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>417</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>418</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>419</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>420</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>421</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (23/07/2026 11:42)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1312,8 +1312,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1329,7 +1337,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1337,12 +1345,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1642,70 +1668,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1746,10 +1772,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1761,7 +1787,7 @@
       <c r="T2" t="s">
         <v>148</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1802,10 +1828,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1852,10 +1878,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1902,10 +1928,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1917,7 +1943,7 @@
       <c r="T5" t="s">
         <v>149</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -1955,10 +1981,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2005,10 +2031,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2020,7 +2046,7 @@
       <c r="T7" t="s">
         <v>150</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -2061,10 +2087,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2111,10 +2137,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2126,7 +2152,7 @@
       <c r="T9" t="s">
         <v>151</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2167,10 +2193,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2211,10 +2237,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2226,7 +2252,7 @@
       <c r="T11" t="s">
         <v>152</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46203</v>
       </c>
     </row>
@@ -2264,7 +2290,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2305,10 +2331,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2352,10 +2378,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2367,7 +2393,7 @@
       <c r="T14" t="s">
         <v>153</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2408,10 +2434,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2458,10 +2484,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2473,7 +2499,7 @@
       <c r="T16" t="s">
         <v>154</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2514,10 +2540,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2564,10 +2590,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2579,7 +2605,7 @@
       <c r="T18" t="s">
         <v>155</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2620,10 +2646,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2635,7 +2661,7 @@
       <c r="T19" t="s">
         <v>122</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46153</v>
       </c>
       <c r="V19">
@@ -2679,10 +2705,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2694,7 +2720,7 @@
       <c r="T20" t="s">
         <v>156</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2735,10 +2761,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2750,7 +2776,7 @@
       <c r="T21" t="s">
         <v>124</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2791,10 +2817,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2806,7 +2832,7 @@
       <c r="T22" t="s">
         <v>157</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2844,10 +2870,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2856,7 +2882,7 @@
       <c r="S23" t="s">
         <v>146</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -2897,10 +2923,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45925</v>
       </c>
       <c r="R24" t="s">
@@ -2947,10 +2973,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -2997,10 +3023,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3012,7 +3038,7 @@
       <c r="T26" t="s">
         <v>158</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -3053,10 +3079,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3103,10 +3129,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3153,10 +3179,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3203,10 +3229,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3218,7 +3244,7 @@
       <c r="T30" t="s">
         <v>159</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3259,10 +3285,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46064</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46064</v>
       </c>
       <c r="R31" t="s">
@@ -3309,10 +3335,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3359,10 +3385,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3374,7 +3400,7 @@
       <c r="T33" t="s">
         <v>160</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3415,10 +3441,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3465,10 +3491,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3515,10 +3541,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3565,10 +3591,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3580,7 +3606,7 @@
       <c r="T37" t="s">
         <v>161</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3621,10 +3647,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>45579</v>
       </c>
       <c r="S38" t="s">
@@ -3671,10 +3697,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3718,10 +3744,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3742,22 +3768,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>168</v>
       </c>
     </row>
@@ -7971,91 +7997,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>252</v>
       </c>
     </row>
@@ -8069,13 +8095,13 @@
       <c r="D2" t="s">
         <v>255</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>258</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8093,13 +8119,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45491</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <v>45528</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8137,13 +8163,13 @@
       <c r="D3" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>258</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8161,13 +8187,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45628</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>45632</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8202,13 +8228,13 @@
       <c r="D4" t="s">
         <v>256</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8226,13 +8252,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45716</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <v>45722</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="2">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8267,13 +8293,13 @@
       <c r="D5" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8291,13 +8317,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45722</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <v>45782</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8335,13 +8361,13 @@
       <c r="D6" t="s">
         <v>256</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>258</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8359,13 +8385,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45728</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>45734</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8403,7 +8429,7 @@
       <c r="D7" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8424,10 +8450,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45772</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8465,7 +8491,7 @@
       <c r="D8" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8486,10 +8512,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>45762</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="2">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8527,7 +8553,7 @@
       <c r="D9" t="s">
         <v>257</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8548,10 +8574,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45763</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8589,13 +8615,13 @@
       <c r="D10" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="2">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8613,13 +8639,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45754</v>
       </c>
-      <c r="R10" s="1">
+      <c r="R10" s="2">
         <v>45849</v>
       </c>
-      <c r="S10" s="1">
+      <c r="S10" s="2">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8654,13 +8680,13 @@
       <c r="D11" t="s">
         <v>256</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>258</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="2">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8678,13 +8704,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44973</v>
       </c>
-      <c r="R11" s="1">
+      <c r="R11" s="2">
         <v>45687</v>
       </c>
-      <c r="S11" s="1">
+      <c r="S11" s="2">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8719,13 +8745,13 @@
       <c r="D12" t="s">
         <v>256</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>258</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="2">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8743,13 +8769,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45358</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="2">
         <v>45517</v>
       </c>
-      <c r="S12" s="1">
+      <c r="S12" s="2">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8784,13 +8810,13 @@
       <c r="D13" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>258</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="2">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8808,13 +8834,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45572</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="2">
         <v>45572</v>
       </c>
-      <c r="S13" s="1">
+      <c r="S13" s="2">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8852,13 +8878,13 @@
       <c r="D14" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>258</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="2">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8876,13 +8902,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>45736</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="2">
         <v>46101</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="2">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -8918,70 +8944,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9019,10 +9045,10 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9066,10 +9092,10 @@
       <c r="O3" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9113,10 +9139,10 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9160,10 +9186,10 @@
       <c r="O5" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9207,10 +9233,10 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9254,10 +9280,10 @@
       <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9301,10 +9327,10 @@
       <c r="O8" t="s">
         <v>103</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9348,10 +9374,10 @@
       <c r="O9" t="s">
         <v>92</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9395,10 +9421,10 @@
       <c r="O10" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9442,10 +9468,10 @@
       <c r="O11" t="s">
         <v>99</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9489,10 +9515,10 @@
       <c r="O12" t="s">
         <v>82</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9536,10 +9562,10 @@
       <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9583,10 +9609,10 @@
       <c r="O14" t="s">
         <v>100</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9630,7 +9656,7 @@
       <c r="O15" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9671,7 +9697,7 @@
       <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9712,10 +9738,10 @@
       <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9759,10 +9785,10 @@
       <c r="O18" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9806,10 +9832,10 @@
       <c r="O19" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9853,10 +9879,10 @@
       <c r="O20" t="s">
         <v>96</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -9900,10 +9926,10 @@
       <c r="O21" t="s">
         <v>105</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9947,10 +9973,10 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9988,10 +10014,10 @@
       <c r="O23" t="s">
         <v>359</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10003,7 +10029,7 @@
       <c r="T23" t="s">
         <v>399</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -10041,10 +10067,10 @@
       <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10056,7 +10082,7 @@
       <c r="T24" t="s">
         <v>400</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -10094,10 +10120,10 @@
       <c r="O25" t="s">
         <v>86</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10109,7 +10135,7 @@
       <c r="T25" t="s">
         <v>401</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -10147,10 +10173,10 @@
       <c r="O26" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10162,7 +10188,7 @@
       <c r="T26" t="s">
         <v>402</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -10200,10 +10226,10 @@
       <c r="O27" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10215,7 +10241,7 @@
       <c r="T27" t="s">
         <v>403</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -10253,10 +10279,10 @@
       <c r="O28" t="s">
         <v>101</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10268,7 +10294,7 @@
       <c r="T28" t="s">
         <v>404</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -10306,10 +10332,10 @@
       <c r="O29" t="s">
         <v>98</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10321,7 +10347,7 @@
       <c r="T29" t="s">
         <v>405</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -10353,7 +10379,7 @@
       <c r="T30" t="s">
         <v>406</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10385,7 +10411,7 @@
       <c r="T31" t="s">
         <v>407</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10417,7 +10443,7 @@
       <c r="T32" t="s">
         <v>408</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10455,10 +10481,10 @@
       <c r="O33" t="s">
         <v>90</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10470,7 +10496,7 @@
       <c r="T33" t="s">
         <v>387</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -10508,16 +10534,16 @@
       <c r="O34" t="s">
         <v>360</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>146</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -10549,10 +10575,10 @@
       <c r="O35" t="s">
         <v>87</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10561,7 +10587,7 @@
       <c r="S35" t="s">
         <v>146</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -10599,10 +10625,10 @@
       <c r="O36" t="s">
         <v>91</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10611,7 +10637,7 @@
       <c r="S36" t="s">
         <v>146</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -10675,10 +10701,10 @@
       <c r="O38" t="s">
         <v>96</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10687,7 +10713,7 @@
       <c r="S38" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -10725,10 +10751,10 @@
       <c r="O39" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10740,7 +10766,7 @@
       <c r="T39" t="s">
         <v>409</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -10772,10 +10798,10 @@
       <c r="O40" t="s">
         <v>100</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10787,7 +10813,7 @@
       <c r="T40" t="s">
         <v>410</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -10825,10 +10851,10 @@
       <c r="O41" t="s">
         <v>95</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10840,7 +10866,7 @@
       <c r="T41" t="s">
         <v>411</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -10878,10 +10904,10 @@
       <c r="O42" t="s">
         <v>82</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -10893,7 +10919,7 @@
       <c r="T42" t="s">
         <v>412</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -10931,10 +10957,10 @@
       <c r="O43" t="s">
         <v>84</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10946,7 +10972,7 @@
       <c r="T43" t="s">
         <v>413</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -10984,10 +11010,10 @@
       <c r="O44" t="s">
         <v>97</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10999,7 +11025,7 @@
       <c r="T44" t="s">
         <v>414</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -11037,10 +11063,10 @@
       <c r="O45" t="s">
         <v>81</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11052,7 +11078,7 @@
       <c r="T45" t="s">
         <v>415</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -11090,10 +11116,10 @@
       <c r="O46" t="s">
         <v>88</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11105,7 +11131,7 @@
       <c r="T46" t="s">
         <v>416</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -11120,25 +11146,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>421</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (23/07/2026 16:18)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1312,16 +1312,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1337,7 +1329,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1345,30 +1337,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1668,70 +1642,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1772,10 +1746,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1787,7 +1761,7 @@
       <c r="T2" t="s">
         <v>148</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1828,10 +1802,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1878,10 +1852,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1928,10 +1902,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1943,7 +1917,7 @@
       <c r="T5" t="s">
         <v>149</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -1981,10 +1955,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2031,10 +2005,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2046,7 +2020,7 @@
       <c r="T7" t="s">
         <v>150</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2087,10 +2061,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2137,10 +2111,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2152,7 +2126,7 @@
       <c r="T9" t="s">
         <v>151</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2193,10 +2167,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2237,10 +2211,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2252,7 +2226,7 @@
       <c r="T11" t="s">
         <v>152</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46203</v>
       </c>
     </row>
@@ -2290,7 +2264,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2331,10 +2305,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2378,10 +2352,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2393,7 +2367,7 @@
       <c r="T14" t="s">
         <v>153</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2434,10 +2408,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2484,10 +2458,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2499,7 +2473,7 @@
       <c r="T16" t="s">
         <v>154</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2540,10 +2514,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2590,10 +2564,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2605,7 +2579,7 @@
       <c r="T18" t="s">
         <v>155</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2646,10 +2620,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2661,7 +2635,7 @@
       <c r="T19" t="s">
         <v>122</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
       <c r="V19">
@@ -2705,10 +2679,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2720,7 +2694,7 @@
       <c r="T20" t="s">
         <v>156</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2761,10 +2735,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2776,7 +2750,7 @@
       <c r="T21" t="s">
         <v>124</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2817,10 +2791,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2832,7 +2806,7 @@
       <c r="T22" t="s">
         <v>157</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2870,10 +2844,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2882,7 +2856,7 @@
       <c r="S23" t="s">
         <v>146</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -2923,10 +2897,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45925</v>
       </c>
       <c r="R24" t="s">
@@ -2973,10 +2947,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3023,10 +2997,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3038,7 +3012,7 @@
       <c r="T26" t="s">
         <v>158</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3079,10 +3053,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3129,10 +3103,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3179,10 +3153,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3229,10 +3203,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3244,7 +3218,7 @@
       <c r="T30" t="s">
         <v>159</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3285,10 +3259,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46064</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46064</v>
       </c>
       <c r="R31" t="s">
@@ -3335,10 +3309,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3385,10 +3359,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3400,7 +3374,7 @@
       <c r="T33" t="s">
         <v>160</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3441,10 +3415,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3491,10 +3465,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3541,10 +3515,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3591,10 +3565,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3606,7 +3580,7 @@
       <c r="T37" t="s">
         <v>161</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3647,10 +3621,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>45579</v>
       </c>
       <c r="S38" t="s">
@@ -3697,10 +3671,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3744,10 +3718,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3768,22 +3742,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>166</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>167</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>168</v>
       </c>
     </row>
@@ -7997,91 +7971,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>229</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>230</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>231</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>232</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>233</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>234</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>235</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>236</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>237</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>238</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>239</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>240</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>241</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>242</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>243</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>244</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>245</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>246</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>247</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>248</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>249</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>250</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>251</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>252</v>
       </c>
     </row>
@@ -8095,13 +8069,13 @@
       <c r="D2" t="s">
         <v>255</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>258</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8119,13 +8093,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8163,13 +8137,13 @@
       <c r="D3" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>258</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8187,13 +8161,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8228,13 +8202,13 @@
       <c r="D4" t="s">
         <v>256</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8252,13 +8226,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8293,13 +8267,13 @@
       <c r="D5" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8317,13 +8291,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8361,13 +8335,13 @@
       <c r="D6" t="s">
         <v>256</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>258</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8385,13 +8359,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8429,7 +8403,7 @@
       <c r="D7" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8450,10 +8424,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8491,7 +8465,7 @@
       <c r="D8" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8512,10 +8486,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8553,7 +8527,7 @@
       <c r="D9" t="s">
         <v>257</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8574,10 +8548,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8615,13 +8589,13 @@
       <c r="D10" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8639,13 +8613,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8680,13 +8654,13 @@
       <c r="D11" t="s">
         <v>256</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>258</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8704,13 +8678,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8745,13 +8719,13 @@
       <c r="D12" t="s">
         <v>256</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>258</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8769,13 +8743,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8810,13 +8784,13 @@
       <c r="D13" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>258</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8834,13 +8808,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8878,13 +8852,13 @@
       <c r="D14" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>258</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8902,13 +8876,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -8944,70 +8918,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9045,10 +9019,10 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9092,10 +9066,10 @@
       <c r="O3" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9139,10 +9113,10 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9186,10 +9160,10 @@
       <c r="O5" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9233,10 +9207,10 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9280,10 +9254,10 @@
       <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9327,10 +9301,10 @@
       <c r="O8" t="s">
         <v>103</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9374,10 +9348,10 @@
       <c r="O9" t="s">
         <v>92</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9421,10 +9395,10 @@
       <c r="O10" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9468,10 +9442,10 @@
       <c r="O11" t="s">
         <v>99</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9515,10 +9489,10 @@
       <c r="O12" t="s">
         <v>82</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9562,10 +9536,10 @@
       <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9609,10 +9583,10 @@
       <c r="O14" t="s">
         <v>100</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9656,7 +9630,7 @@
       <c r="O15" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9697,7 +9671,7 @@
       <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9738,10 +9712,10 @@
       <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9785,10 +9759,10 @@
       <c r="O18" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9832,10 +9806,10 @@
       <c r="O19" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9879,10 +9853,10 @@
       <c r="O20" t="s">
         <v>96</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -9926,10 +9900,10 @@
       <c r="O21" t="s">
         <v>105</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9973,10 +9947,10 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10014,10 +9988,10 @@
       <c r="O23" t="s">
         <v>359</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10029,7 +10003,7 @@
       <c r="T23" t="s">
         <v>399</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10067,10 +10041,10 @@
       <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10082,7 +10056,7 @@
       <c r="T24" t="s">
         <v>400</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10120,10 +10094,10 @@
       <c r="O25" t="s">
         <v>86</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10135,7 +10109,7 @@
       <c r="T25" t="s">
         <v>401</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10173,10 +10147,10 @@
       <c r="O26" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10188,7 +10162,7 @@
       <c r="T26" t="s">
         <v>402</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10226,10 +10200,10 @@
       <c r="O27" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10241,7 +10215,7 @@
       <c r="T27" t="s">
         <v>403</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10279,10 +10253,10 @@
       <c r="O28" t="s">
         <v>101</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10294,7 +10268,7 @@
       <c r="T28" t="s">
         <v>404</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10332,10 +10306,10 @@
       <c r="O29" t="s">
         <v>98</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10347,7 +10321,7 @@
       <c r="T29" t="s">
         <v>405</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10379,7 +10353,7 @@
       <c r="T30" t="s">
         <v>406</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10411,7 +10385,7 @@
       <c r="T31" t="s">
         <v>407</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10443,7 +10417,7 @@
       <c r="T32" t="s">
         <v>408</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10481,10 +10455,10 @@
       <c r="O33" t="s">
         <v>90</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10496,7 +10470,7 @@
       <c r="T33" t="s">
         <v>387</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10534,16 +10508,16 @@
       <c r="O34" t="s">
         <v>360</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>146</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10575,10 +10549,10 @@
       <c r="O35" t="s">
         <v>87</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10587,7 +10561,7 @@
       <c r="S35" t="s">
         <v>146</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10625,10 +10599,10 @@
       <c r="O36" t="s">
         <v>91</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10637,7 +10611,7 @@
       <c r="S36" t="s">
         <v>146</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10701,10 +10675,10 @@
       <c r="O38" t="s">
         <v>96</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10713,7 +10687,7 @@
       <c r="S38" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10751,10 +10725,10 @@
       <c r="O39" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10766,7 +10740,7 @@
       <c r="T39" t="s">
         <v>409</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10798,10 +10772,10 @@
       <c r="O40" t="s">
         <v>100</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10813,7 +10787,7 @@
       <c r="T40" t="s">
         <v>410</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -10851,10 +10825,10 @@
       <c r="O41" t="s">
         <v>95</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10866,7 +10840,7 @@
       <c r="T41" t="s">
         <v>411</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -10904,10 +10878,10 @@
       <c r="O42" t="s">
         <v>82</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -10919,7 +10893,7 @@
       <c r="T42" t="s">
         <v>412</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -10957,10 +10931,10 @@
       <c r="O43" t="s">
         <v>84</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10972,7 +10946,7 @@
       <c r="T43" t="s">
         <v>413</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -11010,10 +10984,10 @@
       <c r="O44" t="s">
         <v>97</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11025,7 +10999,7 @@
       <c r="T44" t="s">
         <v>414</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11063,10 +11037,10 @@
       <c r="O45" t="s">
         <v>81</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11078,7 +11052,7 @@
       <c r="T45" t="s">
         <v>415</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11116,10 +11090,10 @@
       <c r="O46" t="s">
         <v>88</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11131,7 +11105,7 @@
       <c r="T46" t="s">
         <v>416</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11146,25 +11120,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>417</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>418</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>419</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>420</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>421</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (28/07/2026 21:15)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1445,16 +1445,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1470,7 +1462,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1478,30 +1470,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1801,70 +1775,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1905,10 +1879,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1920,7 +1894,7 @@
       <c r="T2" t="s">
         <v>148</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1961,10 +1935,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -2011,10 +1985,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2061,10 +2035,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2076,7 +2050,7 @@
       <c r="T5" t="s">
         <v>149</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -2114,10 +2088,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2164,10 +2138,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2179,7 +2153,7 @@
       <c r="T7" t="s">
         <v>150</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2220,10 +2194,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2270,10 +2244,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2285,7 +2259,7 @@
       <c r="T9" t="s">
         <v>151</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2326,10 +2300,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2370,10 +2344,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2385,7 +2359,7 @@
       <c r="T11" t="s">
         <v>152</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46203</v>
       </c>
     </row>
@@ -2423,7 +2397,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2464,10 +2438,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2511,10 +2485,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2526,7 +2500,7 @@
       <c r="T14" t="s">
         <v>153</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2567,10 +2541,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2617,10 +2591,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2632,7 +2606,7 @@
       <c r="T16" t="s">
         <v>154</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2673,10 +2647,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2723,10 +2697,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2738,7 +2712,7 @@
       <c r="T18" t="s">
         <v>155</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2779,10 +2753,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2794,7 +2768,7 @@
       <c r="T19" t="s">
         <v>122</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
       <c r="V19">
@@ -2838,10 +2812,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2853,7 +2827,7 @@
       <c r="T20" t="s">
         <v>156</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2894,10 +2868,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2909,7 +2883,7 @@
       <c r="T21" t="s">
         <v>124</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2950,10 +2924,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2965,7 +2939,7 @@
       <c r="T22" t="s">
         <v>157</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -3003,10 +2977,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -3015,7 +2989,7 @@
       <c r="S23" t="s">
         <v>146</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -3056,10 +3030,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45925</v>
       </c>
       <c r="R24" t="s">
@@ -3106,10 +3080,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3156,10 +3130,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3171,7 +3145,7 @@
       <c r="T26" t="s">
         <v>158</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3212,10 +3186,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3262,10 +3236,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3312,10 +3286,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3362,10 +3336,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3377,7 +3351,7 @@
       <c r="T30" t="s">
         <v>159</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3418,10 +3392,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46064</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46064</v>
       </c>
       <c r="R31" t="s">
@@ -3468,10 +3442,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3518,10 +3492,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3533,7 +3507,7 @@
       <c r="T33" t="s">
         <v>160</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3574,10 +3548,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3624,10 +3598,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3674,10 +3648,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3724,10 +3698,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3739,7 +3713,7 @@
       <c r="T37" t="s">
         <v>161</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3780,10 +3754,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>45579</v>
       </c>
       <c r="S38" t="s">
@@ -3830,10 +3804,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3877,10 +3851,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3901,22 +3875,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>165</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>166</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>167</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>168</v>
       </c>
     </row>
@@ -8130,91 +8104,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>229</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>230</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>231</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>232</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>233</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>234</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>235</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>236</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>237</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>238</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>239</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>240</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>241</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>242</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>243</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>244</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>245</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>246</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>247</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>248</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>249</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>250</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>251</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>252</v>
       </c>
     </row>
@@ -8228,13 +8202,13 @@
       <c r="D2" t="s">
         <v>255</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>258</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8252,13 +8226,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8296,13 +8270,13 @@
       <c r="D3" t="s">
         <v>256</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>258</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8320,13 +8294,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8361,13 +8335,13 @@
       <c r="D4" t="s">
         <v>256</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>258</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8385,13 +8359,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8426,13 +8400,13 @@
       <c r="D5" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>258</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8450,13 +8424,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8494,13 +8468,13 @@
       <c r="D6" t="s">
         <v>256</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>258</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8518,13 +8492,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8562,7 +8536,7 @@
       <c r="D7" t="s">
         <v>257</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8583,10 +8557,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8624,7 +8598,7 @@
       <c r="D8" t="s">
         <v>257</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8645,10 +8619,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8686,7 +8660,7 @@
       <c r="D9" t="s">
         <v>257</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8707,10 +8681,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8748,13 +8722,13 @@
       <c r="D10" t="s">
         <v>256</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8772,13 +8746,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8813,13 +8787,13 @@
       <c r="D11" t="s">
         <v>256</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>258</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8837,13 +8811,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8878,13 +8852,13 @@
       <c r="D12" t="s">
         <v>256</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>258</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8902,13 +8876,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8943,13 +8917,13 @@
       <c r="D13" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>258</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8967,13 +8941,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -9011,13 +8985,13 @@
       <c r="D14" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>258</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -9035,13 +9009,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9077,70 +9051,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9178,10 +9152,10 @@
       <c r="O2" t="s">
         <v>102</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9225,10 +9199,10 @@
       <c r="O3" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9272,10 +9246,10 @@
       <c r="O4" t="s">
         <v>97</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9319,10 +9293,10 @@
       <c r="O5" t="s">
         <v>98</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9366,10 +9340,10 @@
       <c r="O6" t="s">
         <v>95</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9413,10 +9387,10 @@
       <c r="O7" t="s">
         <v>83</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9460,10 +9434,10 @@
       <c r="O8" t="s">
         <v>103</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9507,10 +9481,10 @@
       <c r="O9" t="s">
         <v>92</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9554,10 +9528,10 @@
       <c r="O10" t="s">
         <v>89</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9601,10 +9575,10 @@
       <c r="O11" t="s">
         <v>99</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9648,10 +9622,10 @@
       <c r="O12" t="s">
         <v>82</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9695,10 +9669,10 @@
       <c r="O13" t="s">
         <v>80</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9742,10 +9716,10 @@
       <c r="O14" t="s">
         <v>100</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9789,7 +9763,7 @@
       <c r="O15" t="s">
         <v>94</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9830,7 +9804,7 @@
       <c r="O16" t="s">
         <v>90</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9871,10 +9845,10 @@
       <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9918,10 +9892,10 @@
       <c r="O18" t="s">
         <v>91</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9965,10 +9939,10 @@
       <c r="O19" t="s">
         <v>104</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -10012,10 +9986,10 @@
       <c r="O20" t="s">
         <v>96</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10059,10 +10033,10 @@
       <c r="O21" t="s">
         <v>105</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10106,10 +10080,10 @@
       <c r="O22" t="s">
         <v>86</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10147,10 +10121,10 @@
       <c r="O23" t="s">
         <v>359</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10162,7 +10136,7 @@
       <c r="T23" t="s">
         <v>399</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10200,10 +10174,10 @@
       <c r="O24" t="s">
         <v>80</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10215,7 +10189,7 @@
       <c r="T24" t="s">
         <v>400</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10253,10 +10227,10 @@
       <c r="O25" t="s">
         <v>86</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10268,7 +10242,7 @@
       <c r="T25" t="s">
         <v>401</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10306,10 +10280,10 @@
       <c r="O26" t="s">
         <v>100</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10321,7 +10295,7 @@
       <c r="T26" t="s">
         <v>402</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10359,10 +10333,10 @@
       <c r="O27" t="s">
         <v>86</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10374,7 +10348,7 @@
       <c r="T27" t="s">
         <v>403</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10412,10 +10386,10 @@
       <c r="O28" t="s">
         <v>101</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10427,7 +10401,7 @@
       <c r="T28" t="s">
         <v>404</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10465,10 +10439,10 @@
       <c r="O29" t="s">
         <v>98</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10480,7 +10454,7 @@
       <c r="T29" t="s">
         <v>405</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10512,7 +10486,7 @@
       <c r="T30" t="s">
         <v>406</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10544,7 +10518,7 @@
       <c r="T31" t="s">
         <v>407</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10576,7 +10550,7 @@
       <c r="T32" t="s">
         <v>408</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10614,10 +10588,10 @@
       <c r="O33" t="s">
         <v>90</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10629,7 +10603,7 @@
       <c r="T33" t="s">
         <v>387</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10667,16 +10641,16 @@
       <c r="O34" t="s">
         <v>360</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>146</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10708,10 +10682,10 @@
       <c r="O35" t="s">
         <v>87</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10720,7 +10694,7 @@
       <c r="S35" t="s">
         <v>146</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10758,10 +10732,10 @@
       <c r="O36" t="s">
         <v>91</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10770,7 +10744,7 @@
       <c r="S36" t="s">
         <v>146</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10834,10 +10808,10 @@
       <c r="O38" t="s">
         <v>96</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10846,7 +10820,7 @@
       <c r="S38" t="s">
         <v>146</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10884,10 +10858,10 @@
       <c r="O39" t="s">
         <v>103</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10899,7 +10873,7 @@
       <c r="T39" t="s">
         <v>409</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10931,10 +10905,10 @@
       <c r="O40" t="s">
         <v>100</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10946,7 +10920,7 @@
       <c r="T40" t="s">
         <v>410</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -10984,10 +10958,10 @@
       <c r="O41" t="s">
         <v>95</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10999,7 +10973,7 @@
       <c r="T41" t="s">
         <v>411</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -11037,10 +11011,10 @@
       <c r="O42" t="s">
         <v>82</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11052,7 +11026,7 @@
       <c r="T42" t="s">
         <v>412</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -11090,10 +11064,10 @@
       <c r="O43" t="s">
         <v>84</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11105,7 +11079,7 @@
       <c r="T43" t="s">
         <v>413</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -11143,10 +11117,10 @@
       <c r="O44" t="s">
         <v>97</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11158,7 +11132,7 @@
       <c r="T44" t="s">
         <v>414</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11196,10 +11170,10 @@
       <c r="O45" t="s">
         <v>81</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11211,7 +11185,7 @@
       <c r="T45" t="s">
         <v>415</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11249,10 +11223,10 @@
       <c r="O46" t="s">
         <v>88</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11264,7 +11238,7 @@
       <c r="T46" t="s">
         <v>416</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11279,25 +11253,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>417</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>418</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>419</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>420</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>421</v>
       </c>
     </row>
@@ -11983,22 +11957,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>422</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>423</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>424</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>425</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>426</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>427</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (13/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -687,8 +687,7 @@
 Motor já está no GLOG-CO</t>
   </si>
   <si>
-    <t>sem at
-Possui AT de 200H, porém foi encontrada  uma trinca e o housing será recolhido.</t>
+    <t>Possui AT 313000000812 de 200H, porém foi encontrada  uma trinca e o housing será recolhido.</t>
   </si>
   <si>
     <t>Fez o 1° HSI COM 1941H, O PROX SERÁ COM 3441.
@@ -4288,10 +4287,10 @@
         <v>2741</v>
       </c>
       <c r="C25">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D25">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E25" t="s">
         <v>172</v>
@@ -11326,7 +11325,7 @@
         <v>3886.67</v>
       </c>
       <c r="D5">
-        <v>113.3333333</v>
+        <v>313.3333333</v>
       </c>
       <c r="E5">
         <v>55.52851064</v>
@@ -11335,7 +11334,7 @@
         <v>260.984</v>
       </c>
       <c r="G5">
-        <v>2.040993573</v>
+        <v>5.642746937</v>
       </c>
     </row>
     <row r="6" spans="1:7">

</xml_diff>

<commit_message>
Atualização automática: motores (18/08/2026 12:33)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1427,8 +1427,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1444,7 +1452,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1452,12 +1460,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1757,70 +1783,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1861,10 +1887,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1876,7 +1902,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1917,10 +1943,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1967,10 +1993,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2014,10 +2040,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2029,7 +2055,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -2070,10 +2096,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2120,10 +2146,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2135,7 +2161,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -2176,10 +2202,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2226,10 +2252,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2241,7 +2267,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2282,10 +2308,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2323,10 +2349,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2338,7 +2364,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46227</v>
       </c>
     </row>
@@ -2376,7 +2402,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2417,10 +2443,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2467,10 +2493,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2482,7 +2508,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2523,10 +2549,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2573,10 +2599,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2588,7 +2614,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2629,10 +2655,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2679,10 +2705,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2694,7 +2720,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2735,10 +2761,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2750,7 +2776,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46153</v>
       </c>
     </row>
@@ -2791,10 +2817,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2806,7 +2832,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2847,10 +2873,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2862,7 +2888,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2903,10 +2929,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2918,7 +2944,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2956,10 +2982,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2968,7 +2994,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -3009,10 +3035,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3021,7 +3047,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -3062,10 +3088,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3112,10 +3138,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3127,7 +3153,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -3168,10 +3194,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3218,10 +3244,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3268,10 +3294,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3318,10 +3344,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3333,7 +3359,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3374,10 +3400,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46220</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3424,10 +3450,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3474,10 +3500,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3489,7 +3515,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3530,10 +3556,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3580,10 +3606,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3630,10 +3656,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3680,10 +3706,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3695,7 +3721,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3736,10 +3762,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3748,7 +3774,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>45351</v>
       </c>
     </row>
@@ -3789,10 +3815,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3836,10 +3862,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3860,22 +3886,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8086,91 +8112,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>255</v>
       </c>
     </row>
@@ -8184,13 +8210,13 @@
       <c r="D2" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>261</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8208,13 +8234,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45491</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <v>45528</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8252,13 +8278,13 @@
       <c r="D3" t="s">
         <v>259</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>261</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8276,13 +8302,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45628</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>45632</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8317,13 +8343,13 @@
       <c r="D4" t="s">
         <v>259</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>261</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8341,13 +8367,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45716</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <v>45722</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="2">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8382,13 +8408,13 @@
       <c r="D5" t="s">
         <v>259</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>261</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8406,13 +8432,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45722</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <v>45782</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8450,13 +8476,13 @@
       <c r="D6" t="s">
         <v>259</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>261</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8474,13 +8500,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45728</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>45734</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8518,7 +8544,7 @@
       <c r="D7" t="s">
         <v>260</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8539,10 +8565,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45772</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8580,7 +8606,7 @@
       <c r="D8" t="s">
         <v>260</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8601,10 +8627,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>45762</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="2">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8642,7 +8668,7 @@
       <c r="D9" t="s">
         <v>260</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8663,10 +8689,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45763</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8704,13 +8730,13 @@
       <c r="D10" t="s">
         <v>259</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>261</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="2">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8728,13 +8754,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45754</v>
       </c>
-      <c r="R10" s="1">
+      <c r="R10" s="2">
         <v>45849</v>
       </c>
-      <c r="S10" s="1">
+      <c r="S10" s="2">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8769,13 +8795,13 @@
       <c r="D11" t="s">
         <v>259</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>261</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="2">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8793,13 +8819,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44973</v>
       </c>
-      <c r="R11" s="1">
+      <c r="R11" s="2">
         <v>45687</v>
       </c>
-      <c r="S11" s="1">
+      <c r="S11" s="2">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8834,13 +8860,13 @@
       <c r="D12" t="s">
         <v>259</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>261</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="2">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8858,13 +8884,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45358</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="2">
         <v>45517</v>
       </c>
-      <c r="S12" s="1">
+      <c r="S12" s="2">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8899,13 +8925,13 @@
       <c r="D13" t="s">
         <v>259</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>261</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="2">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8923,13 +8949,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45572</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="2">
         <v>45572</v>
       </c>
-      <c r="S13" s="1">
+      <c r="S13" s="2">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8967,13 +8993,13 @@
       <c r="D14" t="s">
         <v>259</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>261</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="2">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8991,13 +9017,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>45736</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="2">
         <v>46101</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="2">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9033,70 +9059,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9134,10 +9160,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9181,10 +9207,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9228,10 +9254,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9275,10 +9301,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9322,10 +9348,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9369,10 +9395,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9416,10 +9442,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9463,10 +9489,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9510,10 +9536,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9557,10 +9583,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9604,10 +9630,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9651,10 +9677,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9698,10 +9724,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9745,7 +9771,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9786,7 +9812,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9827,10 +9853,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9874,10 +9900,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9921,10 +9947,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9968,10 +9994,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10015,10 +10041,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10062,10 +10088,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10103,10 +10129,10 @@
       <c r="O23" t="s">
         <v>354</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10118,7 +10144,7 @@
       <c r="T23" t="s">
         <v>394</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -10156,10 +10182,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10171,7 +10197,7 @@
       <c r="T24" t="s">
         <v>395</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -10209,10 +10235,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10224,7 +10250,7 @@
       <c r="T25" t="s">
         <v>396</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -10262,10 +10288,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10277,7 +10303,7 @@
       <c r="T26" t="s">
         <v>397</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -10315,10 +10341,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10330,7 +10356,7 @@
       <c r="T27" t="s">
         <v>398</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -10368,10 +10394,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10383,7 +10409,7 @@
       <c r="T28" t="s">
         <v>399</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -10421,10 +10447,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10436,7 +10462,7 @@
       <c r="T29" t="s">
         <v>400</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -10468,7 +10494,7 @@
       <c r="T30" t="s">
         <v>401</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10500,7 +10526,7 @@
       <c r="T31" t="s">
         <v>402</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10532,7 +10558,7 @@
       <c r="T32" t="s">
         <v>403</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10570,10 +10596,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10585,7 +10611,7 @@
       <c r="T33" t="s">
         <v>382</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -10623,16 +10649,16 @@
       <c r="O34" t="s">
         <v>355</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -10664,10 +10690,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10676,7 +10702,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -10714,10 +10740,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10726,7 +10752,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -10790,10 +10816,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10802,7 +10828,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -10840,10 +10866,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10855,7 +10881,7 @@
       <c r="T39" t="s">
         <v>404</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -10887,10 +10913,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10902,7 +10928,7 @@
       <c r="T40" t="s">
         <v>405</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -10940,10 +10966,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10955,7 +10981,7 @@
       <c r="T41" t="s">
         <v>406</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -10993,10 +11019,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11008,7 +11034,7 @@
       <c r="T42" t="s">
         <v>407</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -11046,10 +11072,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11061,7 +11087,7 @@
       <c r="T43" t="s">
         <v>408</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -11099,10 +11125,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11114,7 +11140,7 @@
       <c r="T44" t="s">
         <v>409</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -11152,10 +11178,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11167,7 +11193,7 @@
       <c r="T45" t="s">
         <v>410</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -11205,10 +11231,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11220,7 +11246,7 @@
       <c r="T46" t="s">
         <v>411</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -11235,25 +11261,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>416</v>
       </c>
     </row>
@@ -11927,22 +11953,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>422</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (18/08/2026 12:41)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1427,16 +1427,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1452,7 +1444,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1460,30 +1452,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1783,70 +1757,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1887,10 +1861,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1902,7 +1876,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1943,10 +1917,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1993,10 +1967,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2040,10 +2014,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2055,7 +2029,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -2096,10 +2070,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2146,10 +2120,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2161,7 +2135,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2202,10 +2176,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2252,10 +2226,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2267,7 +2241,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2308,10 +2282,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2349,10 +2323,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2364,7 +2338,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46227</v>
       </c>
     </row>
@@ -2402,7 +2376,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2443,10 +2417,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2493,10 +2467,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2508,7 +2482,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2549,10 +2523,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2599,10 +2573,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2614,7 +2588,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2655,10 +2629,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2705,10 +2679,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2720,7 +2694,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2761,10 +2735,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2776,7 +2750,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
     </row>
@@ -2817,10 +2791,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2832,7 +2806,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2873,10 +2847,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2888,7 +2862,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2929,10 +2903,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2944,7 +2918,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2982,10 +2956,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2994,7 +2968,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -3035,10 +3009,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3047,7 +3021,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -3088,10 +3062,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3138,10 +3112,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3153,7 +3127,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3194,10 +3168,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3244,10 +3218,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3294,10 +3268,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3344,10 +3318,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3359,7 +3333,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3400,10 +3374,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46220</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3450,10 +3424,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3500,10 +3474,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3515,7 +3489,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3556,10 +3530,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3606,10 +3580,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3656,10 +3630,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3706,10 +3680,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3721,7 +3695,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3762,10 +3736,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3774,7 +3748,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>45351</v>
       </c>
     </row>
@@ -3815,10 +3789,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3862,10 +3836,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3886,22 +3860,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8112,91 +8086,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>233</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>234</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>235</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>236</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>237</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>238</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>239</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>240</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>241</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>242</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>243</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>244</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>245</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>246</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>247</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>248</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>249</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>250</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>251</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>252</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>253</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>254</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>255</v>
       </c>
     </row>
@@ -8210,13 +8184,13 @@
       <c r="D2" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>261</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8234,13 +8208,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8278,13 +8252,13 @@
       <c r="D3" t="s">
         <v>259</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>261</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8302,13 +8276,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8343,13 +8317,13 @@
       <c r="D4" t="s">
         <v>259</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>261</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8367,13 +8341,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8408,13 +8382,13 @@
       <c r="D5" t="s">
         <v>259</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>261</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8432,13 +8406,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8476,13 +8450,13 @@
       <c r="D6" t="s">
         <v>259</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>261</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8500,13 +8474,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8544,7 +8518,7 @@
       <c r="D7" t="s">
         <v>260</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8565,10 +8539,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8606,7 +8580,7 @@
       <c r="D8" t="s">
         <v>260</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8627,10 +8601,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8668,7 +8642,7 @@
       <c r="D9" t="s">
         <v>260</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8689,10 +8663,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8730,13 +8704,13 @@
       <c r="D10" t="s">
         <v>259</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>261</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8754,13 +8728,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8795,13 +8769,13 @@
       <c r="D11" t="s">
         <v>259</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>261</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8819,13 +8793,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8860,13 +8834,13 @@
       <c r="D12" t="s">
         <v>259</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>261</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8884,13 +8858,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8925,13 +8899,13 @@
       <c r="D13" t="s">
         <v>259</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>261</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8949,13 +8923,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8993,13 +8967,13 @@
       <c r="D14" t="s">
         <v>259</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>261</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -9017,13 +8991,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9059,70 +9033,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9160,10 +9134,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9207,10 +9181,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9254,10 +9228,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9301,10 +9275,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9348,10 +9322,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9395,10 +9369,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9442,10 +9416,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9489,10 +9463,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9536,10 +9510,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9583,10 +9557,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9630,10 +9604,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9677,10 +9651,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9724,10 +9698,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9771,7 +9745,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9812,7 +9786,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9853,10 +9827,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9900,10 +9874,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9947,10 +9921,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9994,10 +9968,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10041,10 +10015,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10088,10 +10062,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10129,10 +10103,10 @@
       <c r="O23" t="s">
         <v>354</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10144,7 +10118,7 @@
       <c r="T23" t="s">
         <v>394</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10182,10 +10156,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10197,7 +10171,7 @@
       <c r="T24" t="s">
         <v>395</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10235,10 +10209,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10250,7 +10224,7 @@
       <c r="T25" t="s">
         <v>396</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10288,10 +10262,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10303,7 +10277,7 @@
       <c r="T26" t="s">
         <v>397</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10341,10 +10315,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10356,7 +10330,7 @@
       <c r="T27" t="s">
         <v>398</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10394,10 +10368,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10409,7 +10383,7 @@
       <c r="T28" t="s">
         <v>399</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10447,10 +10421,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10462,7 +10436,7 @@
       <c r="T29" t="s">
         <v>400</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10494,7 +10468,7 @@
       <c r="T30" t="s">
         <v>401</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10526,7 +10500,7 @@
       <c r="T31" t="s">
         <v>402</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10558,7 +10532,7 @@
       <c r="T32" t="s">
         <v>403</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10596,10 +10570,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10611,7 +10585,7 @@
       <c r="T33" t="s">
         <v>382</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10649,16 +10623,16 @@
       <c r="O34" t="s">
         <v>355</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10690,10 +10664,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10702,7 +10676,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10740,10 +10714,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10752,7 +10726,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10816,10 +10790,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10828,7 +10802,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10866,10 +10840,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10881,7 +10855,7 @@
       <c r="T39" t="s">
         <v>404</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10913,10 +10887,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10928,7 +10902,7 @@
       <c r="T40" t="s">
         <v>405</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -10966,10 +10940,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10981,7 +10955,7 @@
       <c r="T41" t="s">
         <v>406</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -11019,10 +10993,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11034,7 +11008,7 @@
       <c r="T42" t="s">
         <v>407</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -11072,10 +11046,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11087,7 +11061,7 @@
       <c r="T43" t="s">
         <v>408</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -11125,10 +11099,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11140,7 +11114,7 @@
       <c r="T44" t="s">
         <v>409</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11178,10 +11152,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11193,7 +11167,7 @@
       <c r="T45" t="s">
         <v>410</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11231,10 +11205,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11246,7 +11220,7 @@
       <c r="T46" t="s">
         <v>411</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11261,25 +11235,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>412</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>413</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>414</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>415</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>416</v>
       </c>
     </row>
@@ -11953,22 +11927,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>417</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>418</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>419</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>420</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>421</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>422</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (19/08/2026 12:41)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -537,39 +537,39 @@
     <t>1.0</t>
   </si>
   <si>
+    <t>NÃO HÁ AT</t>
+  </si>
+  <si>
     <t>TBO</t>
   </si>
   <si>
     <t>X</t>
   </si>
   <si>
-    <t>NÃO HÁ AT</t>
+    <t>17.3</t>
+  </si>
+  <si>
+    <t>16.0</t>
+  </si>
+  <si>
+    <t>HSI</t>
+  </si>
+  <si>
+    <t>16.3</t>
+  </si>
+  <si>
+    <t>34.2</t>
+  </si>
+  <si>
+    <t>22.0</t>
+  </si>
+  <si>
+    <t>27.1</t>
   </si>
   <si>
     <t>vazamento de oleo pelo flange</t>
   </si>
   <si>
-    <t>17.3</t>
-  </si>
-  <si>
-    <t>16.0</t>
-  </si>
-  <si>
-    <t>HSI</t>
-  </si>
-  <si>
-    <t>16.3</t>
-  </si>
-  <si>
-    <t>34.2</t>
-  </si>
-  <si>
-    <t>22.0</t>
-  </si>
-  <si>
-    <t>27.1</t>
-  </si>
-  <si>
     <t>HÁ AT</t>
   </si>
   <si>
@@ -591,34 +591,34 @@
     <t>2.726773384</t>
   </si>
   <si>
+    <t>57.1</t>
+  </si>
+  <si>
+    <t>47.0</t>
+  </si>
+  <si>
+    <t>4.906536528</t>
+  </si>
+  <si>
+    <t>#N/A</t>
+  </si>
+  <si>
+    <t>Rachadura na CT DISK, vai recolher</t>
+  </si>
+  <si>
+    <t>19.2</t>
+  </si>
+  <si>
+    <t>MOTOR EM HSI NO OPERADOR, 17/07/2026</t>
+  </si>
+  <si>
     <t>28.1</t>
   </si>
   <si>
     <t>27.0</t>
   </si>
   <si>
-    <t>9.574774775</t>
-  </si>
-  <si>
-    <t>#N/A</t>
-  </si>
-  <si>
-    <t>Rachadura na CT DISK, vai recolher</t>
-  </si>
-  <si>
-    <t>19.2</t>
-  </si>
-  <si>
-    <t>MOTOR EM HSI NO OPERADOR, 17/07/2026</t>
-  </si>
-  <si>
-    <t>57.1</t>
-  </si>
-  <si>
-    <t>47.0</t>
-  </si>
-  <si>
-    <t>4.906536528</t>
+    <t>12.68828829</t>
   </si>
   <si>
     <t>6.081238361</t>
@@ -660,7 +660,7 @@
     <t>17.63967357</t>
   </si>
   <si>
-    <t>22.94847203</t>
+    <t>22.95015112</t>
   </si>
   <si>
     <t>Motor novo, não atingiu performance (CAIXA DE ACESSÓRIOS PESADA) 27/05</t>
@@ -669,25 +669,19 @@
     <t>recolhido 23/04. adiantou o tbo</t>
   </si>
   <si>
-    <t>54.82962963</t>
+    <t>54.9</t>
   </si>
   <si>
     <t>30.17519472</t>
   </si>
   <si>
-    <t>AT 313000000805 extensão até 4200h TBO</t>
+    <t>AT 386000001002  500H
+Motor já está no GLOG-CO</t>
   </si>
   <si>
     <t>AT 313000000695
 4450H
 Motor substituto já em MN</t>
-  </si>
-  <si>
-    <t>AT 386000001002  500H
-Motor já está no GLOG-CO</t>
-  </si>
-  <si>
-    <t>Possui AT 313000000812 de 200H, porém foi encontrada  uma trinca e o housing será recolhido.</t>
   </si>
   <si>
     <t>Fez o 1° HSI COM 1941H, O PROX SERÁ COM 3441.
@@ -696,7 +690,13 @@
 motor POSSUI TSO DE 2.941:00H, RESTANDO 500:15H . vai casar exatamente com o HSI 3.441,25</t>
   </si>
   <si>
+    <t>AT 313000000805 extensão até 4200h TBO</t>
+  </si>
+  <si>
     <t>AT 685000002046, CONCEDEU MAIS 400H</t>
+  </si>
+  <si>
+    <t>Possui AT 313000000812 de 200H, porém foi encontrada  uma trinca e o housing será recolhido.</t>
   </si>
   <si>
     <t>PREVISÃO PARA O PRÓXIMO HSI COM 4665:30 TSO
@@ -2364,6 +2364,9 @@
       <c r="J12" t="s">
         <v>81</v>
       </c>
+      <c r="K12">
+        <v>100</v>
+      </c>
       <c r="L12">
         <v>7592.92</v>
       </c>
@@ -2404,6 +2407,9 @@
       </c>
       <c r="J13" t="s">
         <v>81</v>
+      </c>
+      <c r="K13">
+        <v>100</v>
       </c>
       <c r="L13">
         <v>4526.42</v>
@@ -3881,10 +3887,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B2">
-        <v>2736</v>
+        <v>2743</v>
       </c>
       <c r="C2">
         <v>2025</v>
@@ -3898,10 +3904,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B3">
-        <v>2736</v>
+        <v>2743</v>
       </c>
       <c r="C3">
         <v>2025</v>
@@ -3915,10 +3921,10 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B4">
-        <v>2736</v>
+        <v>2743</v>
       </c>
       <c r="C4">
         <v>2025</v>
@@ -3932,39 +3938,39 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B5">
-        <v>2736</v>
+        <v>2743</v>
       </c>
       <c r="C5">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
         <v>172</v>
       </c>
-      <c r="F5" t="s">
-        <v>218</v>
-      </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" t="b">
-        <v>0</v>
+        <v>74</v>
+      </c>
+      <c r="B6">
+        <v>2743</v>
       </c>
       <c r="C6">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
         <v>173</v>
+      </c>
+      <c r="F6" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -3978,10 +3984,10 @@
         <v>2025</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -3995,10 +4001,10 @@
         <v>2025</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -4012,10 +4018,10 @@
         <v>2025</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -4029,10 +4035,10 @@
         <v>2025</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -4046,7 +4052,7 @@
         <v>2025</v>
       </c>
       <c r="D11">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E11" t="s">
         <v>174</v>
@@ -4060,47 +4066,47 @@
         <v>0</v>
       </c>
       <c r="C12">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D12">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E12" t="s">
         <v>172</v>
       </c>
-      <c r="F12" t="s">
-        <v>219</v>
-      </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13">
-        <v>2743</v>
+        <v>61</v>
+      </c>
+      <c r="B13" t="b">
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E13" t="s">
-        <v>171</v>
+        <v>173</v>
+      </c>
+      <c r="F13" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="B14">
-        <v>2743</v>
+        <v>2740</v>
       </c>
       <c r="C14">
         <v>2025</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" t="s">
         <v>171</v>
@@ -4108,16 +4114,16 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="B15">
-        <v>2743</v>
+        <v>2740</v>
       </c>
       <c r="C15">
         <v>2025</v>
       </c>
       <c r="D15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" t="s">
         <v>171</v>
@@ -4125,104 +4131,104 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="B16">
-        <v>2743</v>
+        <v>2740</v>
       </c>
       <c r="C16">
         <v>2025</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="B17">
-        <v>2743</v>
+        <v>2740</v>
       </c>
       <c r="C17">
         <v>2026</v>
       </c>
       <c r="D17">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E17" t="s">
-        <v>172</v>
-      </c>
-      <c r="F17" t="s">
-        <v>220</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="B18">
-        <v>2741</v>
+        <v>2740</v>
       </c>
       <c r="C18">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E18" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="B19">
-        <v>2741</v>
+        <v>2740</v>
       </c>
       <c r="C19">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>173</v>
+        <v>177</v>
+      </c>
+      <c r="F19" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="B20">
-        <v>2741</v>
+        <v>2740</v>
       </c>
       <c r="C20">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D20">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="B21">
-        <v>2741</v>
+        <v>2740</v>
       </c>
       <c r="C21">
-        <v>2025</v>
+        <v>2028</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E21" t="s">
         <v>173</v>
@@ -4230,220 +4236,217 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B22">
-        <v>2741</v>
+        <v>2709</v>
       </c>
       <c r="C22">
         <v>2025</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E22" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B23">
-        <v>2741</v>
+        <v>2709</v>
       </c>
       <c r="C23">
         <v>2025</v>
       </c>
       <c r="D23">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B24">
-        <v>2741</v>
+        <v>2709</v>
       </c>
       <c r="C24">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D24">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B25">
-        <v>2741</v>
+        <v>2709</v>
       </c>
       <c r="C25">
-        <v>2027</v>
+        <v>2025</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E25" t="s">
         <v>172</v>
       </c>
-      <c r="F25" t="s">
-        <v>221</v>
-      </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B26">
-        <v>2740</v>
+        <v>2709</v>
       </c>
       <c r="C26">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B27">
-        <v>2740</v>
+        <v>2709</v>
       </c>
       <c r="C27">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E27" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B28">
-        <v>2740</v>
+        <v>2709</v>
       </c>
       <c r="C28">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D28">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B29">
-        <v>2740</v>
+        <v>2709</v>
       </c>
       <c r="C29">
         <v>2026</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="B30">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="C30">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D30">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="B31">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="C31">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D31">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>178</v>
-      </c>
-      <c r="F31" t="s">
-        <v>222</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="B32">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="C32">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E32" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="B33">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="C33">
-        <v>2028</v>
+        <v>2026</v>
       </c>
       <c r="D33">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>172</v>
+        <v>173</v>
+      </c>
+      <c r="F33" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B34">
-        <v>2709</v>
+        <v>2722</v>
       </c>
       <c r="C34">
         <v>2025</v>
@@ -4457,10 +4460,10 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B35">
-        <v>2709</v>
+        <v>2722</v>
       </c>
       <c r="C35">
         <v>2025</v>
@@ -4474,10 +4477,10 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B36">
-        <v>2709</v>
+        <v>2722</v>
       </c>
       <c r="C36">
         <v>2025</v>
@@ -4491,10 +4494,10 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B37">
-        <v>2709</v>
+        <v>2722</v>
       </c>
       <c r="C37">
         <v>2025</v>
@@ -4503,160 +4506,163 @@
         <v>10</v>
       </c>
       <c r="E37" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B38">
-        <v>2709</v>
+        <v>2722</v>
       </c>
       <c r="C38">
         <v>2026</v>
       </c>
       <c r="D38">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>180</v>
+        <v>173</v>
+      </c>
+      <c r="F38" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B39">
-        <v>2709</v>
+        <v>2741</v>
       </c>
       <c r="C39">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E39" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B40">
-        <v>2709</v>
+        <v>2741</v>
       </c>
       <c r="C40">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D40">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="E40" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B41">
-        <v>2709</v>
+        <v>2741</v>
       </c>
       <c r="C41">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D41">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E41" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B42">
-        <v>2722</v>
+        <v>2741</v>
       </c>
       <c r="C42">
         <v>2025</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E42" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B43">
-        <v>2722</v>
+        <v>2741</v>
       </c>
       <c r="C43">
         <v>2025</v>
       </c>
       <c r="D43">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E43" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B44">
-        <v>2722</v>
+        <v>2741</v>
       </c>
       <c r="C44">
         <v>2025</v>
       </c>
       <c r="D44">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E44" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B45">
-        <v>2722</v>
+        <v>2741</v>
       </c>
       <c r="C45">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D45">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E45" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B46">
-        <v>2722</v>
+        <v>2741</v>
       </c>
       <c r="C46">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D46">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F46" t="s">
         <v>223</v>
@@ -4832,7 +4838,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -4900,7 +4906,7 @@
         <v>3</v>
       </c>
       <c r="E60" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F60" t="s">
         <v>225</v>
@@ -4920,7 +4926,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -5022,15 +5028,15 @@
         <v>3</v>
       </c>
       <c r="E67" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B68">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C68">
         <v>2025</v>
@@ -5039,15 +5045,15 @@
         <v>1</v>
       </c>
       <c r="E68" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B69">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C69">
         <v>2025</v>
@@ -5056,15 +5062,15 @@
         <v>2</v>
       </c>
       <c r="E69" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B70">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C70">
         <v>2025</v>
@@ -5073,126 +5079,126 @@
         <v>3</v>
       </c>
       <c r="E70" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B71">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C71">
         <v>2025</v>
       </c>
       <c r="D71">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E71" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B72">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C72">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D72">
         <v>5</v>
       </c>
       <c r="E72" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B73">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C73">
         <v>2026</v>
       </c>
       <c r="D73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E73" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B74">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C74">
         <v>2026</v>
       </c>
       <c r="D74">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E74" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B75">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C75">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="D75">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E75" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>46</v>
-      </c>
-      <c r="B76">
-        <v>2742</v>
+        <v>64</v>
+      </c>
+      <c r="B76" t="b">
+        <v>0</v>
       </c>
       <c r="C76">
-        <v>2027</v>
+        <v>2025</v>
       </c>
       <c r="D76">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E76" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>46</v>
-      </c>
-      <c r="B77">
-        <v>2742</v>
+        <v>64</v>
+      </c>
+      <c r="B77" t="b">
+        <v>0</v>
       </c>
       <c r="C77">
-        <v>2029</v>
+        <v>2025</v>
       </c>
       <c r="D77">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E77" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -5206,7 +5212,7 @@
         <v>2025</v>
       </c>
       <c r="D78">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E78" t="s">
         <v>171</v>
@@ -5223,10 +5229,10 @@
         <v>2025</v>
       </c>
       <c r="D79">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E79" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -5240,10 +5246,10 @@
         <v>2025</v>
       </c>
       <c r="D80">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E80" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -5254,13 +5260,13 @@
         <v>0</v>
       </c>
       <c r="C81">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D81">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E81" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -5271,47 +5277,47 @@
         <v>0</v>
       </c>
       <c r="C82">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D82">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E82" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B83" t="b">
         <v>0</v>
       </c>
       <c r="C83">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D83">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E83" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="B84" t="b">
         <v>0</v>
       </c>
       <c r="C84">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D84">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E84" t="s">
-        <v>194</v>
+        <v>171</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -5325,7 +5331,7 @@
         <v>2025</v>
       </c>
       <c r="D85">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E85" t="s">
         <v>171</v>
@@ -5342,10 +5348,10 @@
         <v>2025</v>
       </c>
       <c r="D86">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E86" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -5356,13 +5362,13 @@
         <v>0</v>
       </c>
       <c r="C87">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D87">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E87" t="s">
-        <v>171</v>
+        <v>195</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -5373,13 +5379,16 @@
         <v>0</v>
       </c>
       <c r="C88">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D88">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E88" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="F88" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -5393,10 +5402,10 @@
         <v>2026</v>
       </c>
       <c r="D89">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E89" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -5410,183 +5419,180 @@
         <v>2026</v>
       </c>
       <c r="D90">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E90" t="s">
-        <v>178</v>
-      </c>
-      <c r="F90" t="s">
-        <v>226</v>
+        <v>196</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" t="s">
-        <v>78</v>
-      </c>
-      <c r="B91" t="b">
-        <v>0</v>
+        <v>46</v>
+      </c>
+      <c r="B91">
+        <v>2742</v>
       </c>
       <c r="C91">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D91">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E91" t="s">
-        <v>193</v>
+        <v>174</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" t="s">
-        <v>78</v>
-      </c>
-      <c r="B92" t="b">
-        <v>0</v>
+        <v>46</v>
+      </c>
+      <c r="B92">
+        <v>2742</v>
       </c>
       <c r="C92">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D92">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E92" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B93">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C93">
         <v>2025</v>
       </c>
       <c r="D93">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E93" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B94">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C94">
         <v>2025</v>
       </c>
       <c r="D94">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E94" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B95">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C95">
         <v>2025</v>
       </c>
       <c r="D95">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E95" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B96">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C96">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D96">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E96" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
     </row>
     <row r="97" spans="1:5">
       <c r="A97" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B97">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C97">
         <v>2026</v>
       </c>
       <c r="D97">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E97" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="98" spans="1:5">
       <c r="A98" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B98">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C98">
         <v>2026</v>
       </c>
       <c r="D98">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E98" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="99" spans="1:5">
       <c r="A99" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B99">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C99">
-        <v>2026</v>
+        <v>2028</v>
       </c>
       <c r="D99">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E99" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
     </row>
     <row r="100" spans="1:5">
       <c r="A100" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B100">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C100">
-        <v>2027</v>
+        <v>2029</v>
       </c>
       <c r="D100">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E100" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -5654,7 +5660,7 @@
         <v>5</v>
       </c>
       <c r="E104" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -5671,7 +5677,7 @@
         <v>8</v>
       </c>
       <c r="E105" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -5688,7 +5694,7 @@
         <v>10</v>
       </c>
       <c r="E106" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -5722,7 +5728,7 @@
         <v>7</v>
       </c>
       <c r="E108" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -5790,7 +5796,7 @@
         <v>4</v>
       </c>
       <c r="E112" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -5807,7 +5813,7 @@
         <v>5</v>
       </c>
       <c r="E113" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -5824,7 +5830,7 @@
         <v>10</v>
       </c>
       <c r="E114" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -5858,7 +5864,7 @@
         <v>2</v>
       </c>
       <c r="E116" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -5926,7 +5932,7 @@
         <v>10</v>
       </c>
       <c r="E120" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -5994,7 +6000,7 @@
         <v>1</v>
       </c>
       <c r="E124" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -6011,7 +6017,7 @@
         <v>4</v>
       </c>
       <c r="E125" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -6028,7 +6034,7 @@
         <v>1</v>
       </c>
       <c r="E126" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -6045,7 +6051,7 @@
         <v>2</v>
       </c>
       <c r="E127" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -6062,7 +6068,7 @@
         <v>3</v>
       </c>
       <c r="E128" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -6079,7 +6085,7 @@
         <v>4</v>
       </c>
       <c r="E129" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -6096,7 +6102,7 @@
         <v>5</v>
       </c>
       <c r="E130" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -6147,7 +6153,7 @@
         <v>6</v>
       </c>
       <c r="E133" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -6269,7 +6275,7 @@
         <v>9</v>
       </c>
       <c r="E140" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F140" t="s">
         <v>228</v>
@@ -6289,7 +6295,7 @@
         <v>2</v>
       </c>
       <c r="E141" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -6306,7 +6312,7 @@
         <v>1</v>
       </c>
       <c r="E142" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -6323,7 +6329,7 @@
         <v>2</v>
       </c>
       <c r="E143" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -6340,7 +6346,7 @@
         <v>3</v>
       </c>
       <c r="E144" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -6357,7 +6363,7 @@
         <v>4</v>
       </c>
       <c r="E145" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -6374,7 +6380,7 @@
         <v>5</v>
       </c>
       <c r="E146" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -6391,7 +6397,7 @@
         <v>10</v>
       </c>
       <c r="E147" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -6425,7 +6431,7 @@
         <v>8</v>
       </c>
       <c r="E149" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -6493,7 +6499,7 @@
         <v>10</v>
       </c>
       <c r="E153" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -6561,7 +6567,7 @@
         <v>6</v>
       </c>
       <c r="E157" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -6578,7 +6584,7 @@
         <v>1</v>
       </c>
       <c r="E158" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -6595,7 +6601,7 @@
         <v>2</v>
       </c>
       <c r="E159" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -6612,7 +6618,7 @@
         <v>3</v>
       </c>
       <c r="E160" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -6629,7 +6635,7 @@
         <v>4</v>
       </c>
       <c r="E161" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -6646,7 +6652,7 @@
         <v>5</v>
       </c>
       <c r="E162" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -6680,7 +6686,7 @@
         <v>12</v>
       </c>
       <c r="E164" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -6697,7 +6703,7 @@
         <v>1</v>
       </c>
       <c r="E165" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -6731,7 +6737,7 @@
         <v>1</v>
       </c>
       <c r="E167" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -6748,7 +6754,7 @@
         <v>2</v>
       </c>
       <c r="E168" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -6765,7 +6771,7 @@
         <v>3</v>
       </c>
       <c r="E169" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -6782,7 +6788,7 @@
         <v>4</v>
       </c>
       <c r="E170" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -6799,7 +6805,7 @@
         <v>5</v>
       </c>
       <c r="E171" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -6816,7 +6822,7 @@
         <v>1</v>
       </c>
       <c r="E172" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -6833,7 +6839,7 @@
         <v>2</v>
       </c>
       <c r="E173" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -6850,7 +6856,7 @@
         <v>3</v>
       </c>
       <c r="E174" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -6867,7 +6873,7 @@
         <v>4</v>
       </c>
       <c r="E175" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -6884,7 +6890,7 @@
         <v>5</v>
       </c>
       <c r="E176" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="177" spans="1:6">
@@ -6952,7 +6958,7 @@
         <v>8</v>
       </c>
       <c r="E180" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F180" t="s">
         <v>229</v>
@@ -7006,7 +7012,7 @@
         <v>1</v>
       </c>
       <c r="E183" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="184" spans="1:6">
@@ -7023,7 +7029,7 @@
         <v>2</v>
       </c>
       <c r="E184" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="185" spans="1:6">
@@ -7040,7 +7046,7 @@
         <v>3</v>
       </c>
       <c r="E185" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="186" spans="1:6">
@@ -7057,7 +7063,7 @@
         <v>4</v>
       </c>
       <c r="E186" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="187" spans="1:6">
@@ -7074,7 +7080,7 @@
         <v>5</v>
       </c>
       <c r="E187" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="188" spans="1:6">
@@ -7108,7 +7114,7 @@
         <v>3</v>
       </c>
       <c r="E189" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="190" spans="1:6">
@@ -7125,7 +7131,7 @@
         <v>1</v>
       </c>
       <c r="E190" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="191" spans="1:6">
@@ -7142,7 +7148,7 @@
         <v>2</v>
       </c>
       <c r="E191" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="192" spans="1:6">
@@ -7159,7 +7165,7 @@
         <v>3</v>
       </c>
       <c r="E192" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="193" spans="1:6">
@@ -7176,7 +7182,7 @@
         <v>4</v>
       </c>
       <c r="E193" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="194" spans="1:6">
@@ -7193,7 +7199,7 @@
         <v>5</v>
       </c>
       <c r="E194" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="195" spans="1:6">
@@ -7210,7 +7216,7 @@
         <v>1</v>
       </c>
       <c r="E195" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="196" spans="1:6">
@@ -7227,7 +7233,7 @@
         <v>2</v>
       </c>
       <c r="E196" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="197" spans="1:6">
@@ -7244,7 +7250,7 @@
         <v>3</v>
       </c>
       <c r="E197" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="198" spans="1:6">
@@ -7261,7 +7267,7 @@
         <v>4</v>
       </c>
       <c r="E198" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="199" spans="1:6">
@@ -7278,7 +7284,7 @@
         <v>5</v>
       </c>
       <c r="E199" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="200" spans="1:6">
@@ -7295,7 +7301,7 @@
         <v>8</v>
       </c>
       <c r="E200" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F200" t="s">
         <v>230</v>
@@ -7332,7 +7338,7 @@
         <v>1</v>
       </c>
       <c r="E202" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F202" t="s">
         <v>230</v>
@@ -7454,7 +7460,7 @@
         <v>8</v>
       </c>
       <c r="E209" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="210" spans="1:6">
@@ -7471,7 +7477,7 @@
         <v>9</v>
       </c>
       <c r="E210" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="211" spans="1:6">
@@ -7556,7 +7562,7 @@
         <v>2</v>
       </c>
       <c r="E215" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="216" spans="1:6">
@@ -7590,7 +7596,7 @@
         <v>8</v>
       </c>
       <c r="E217" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F217" t="s">
         <v>231</v>
@@ -7610,7 +7616,7 @@
         <v>9</v>
       </c>
       <c r="E218" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F218" t="s">
         <v>231</v>
@@ -7630,7 +7636,7 @@
         <v>1</v>
       </c>
       <c r="E219" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="220" spans="1:6">
@@ -7647,7 +7653,7 @@
         <v>2</v>
       </c>
       <c r="E220" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="221" spans="1:6">
@@ -7664,7 +7670,7 @@
         <v>3</v>
       </c>
       <c r="E221" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="222" spans="1:6">
@@ -7681,7 +7687,7 @@
         <v>4</v>
       </c>
       <c r="E222" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="223" spans="1:6">
@@ -7698,7 +7704,7 @@
         <v>5</v>
       </c>
       <c r="E223" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="224" spans="1:6">
@@ -7715,7 +7721,7 @@
         <v>1</v>
       </c>
       <c r="E224" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -7732,7 +7738,7 @@
         <v>2</v>
       </c>
       <c r="E225" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -7749,7 +7755,7 @@
         <v>3</v>
       </c>
       <c r="E226" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -7766,7 +7772,7 @@
         <v>4</v>
       </c>
       <c r="E227" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -7783,7 +7789,7 @@
         <v>5</v>
       </c>
       <c r="E228" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -7800,7 +7806,7 @@
         <v>10</v>
       </c>
       <c r="E229" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -7834,7 +7840,7 @@
         <v>10</v>
       </c>
       <c r="E231" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -7851,7 +7857,7 @@
         <v>1</v>
       </c>
       <c r="E232" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -7868,7 +7874,7 @@
         <v>2</v>
       </c>
       <c r="E233" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -7885,7 +7891,7 @@
         <v>3</v>
       </c>
       <c r="E234" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -7902,7 +7908,7 @@
         <v>4</v>
       </c>
       <c r="E235" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -7919,7 +7925,7 @@
         <v>5</v>
       </c>
       <c r="E236" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -7987,7 +7993,7 @@
         <v>10</v>
       </c>
       <c r="E240" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -8004,7 +8010,7 @@
         <v>1</v>
       </c>
       <c r="E241" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -8021,7 +8027,7 @@
         <v>2</v>
       </c>
       <c r="E242" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -8038,7 +8044,7 @@
         <v>3</v>
       </c>
       <c r="E243" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="244" spans="1:5">
@@ -8055,7 +8061,7 @@
         <v>4</v>
       </c>
       <c r="E244" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -8072,7 +8078,7 @@
         <v>5</v>
       </c>
       <c r="E245" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -11259,25 +11265,25 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B2">
-        <v>2736</v>
+        <v>2743</v>
       </c>
       <c r="C2">
-        <v>3992.33</v>
+        <v>4412.92</v>
       </c>
       <c r="D2">
-        <v>207.6666667</v>
+        <v>87.08333333</v>
       </c>
       <c r="E2">
-        <v>55.52851064</v>
+        <v>95.14042553</v>
       </c>
       <c r="F2">
-        <v>260.984</v>
+        <v>447.16</v>
       </c>
       <c r="G2">
-        <v>3.739820576</v>
+        <v>0.9153136834</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -11293,62 +11299,62 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="B4">
-        <v>2743</v>
+        <v>2740</v>
       </c>
       <c r="C4">
-        <v>4412.92</v>
+        <v>3301.75</v>
       </c>
       <c r="D4">
-        <v>87.08333333</v>
+        <v>139.25</v>
       </c>
       <c r="E4">
-        <v>95.14042553</v>
+        <v>55.52851064</v>
       </c>
       <c r="F4">
-        <v>447.16</v>
+        <v>260.984</v>
       </c>
       <c r="G4">
-        <v>0.9153136834</v>
+        <v>2.50772078</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B5">
-        <v>2741</v>
+        <v>2709</v>
       </c>
       <c r="C5">
-        <v>3886.67</v>
+        <v>2755.25</v>
       </c>
       <c r="D5">
-        <v>313.3333333</v>
+        <v>147.75</v>
       </c>
       <c r="E5">
-        <v>55.52851064</v>
+        <v>51.37446809</v>
       </c>
       <c r="F5">
-        <v>260.984</v>
+        <v>241.46</v>
       </c>
       <c r="G5">
-        <v>5.642746937</v>
+        <v>2.875942185</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="B6">
-        <v>2740</v>
+        <v>2736</v>
       </c>
       <c r="C6">
-        <v>3301.75</v>
+        <v>3992.33</v>
       </c>
       <c r="D6">
-        <v>139.25</v>
+        <v>207.6666667</v>
       </c>
       <c r="E6">
         <v>55.52851064</v>
@@ -11357,53 +11363,53 @@
         <v>260.984</v>
       </c>
       <c r="G6">
-        <v>2.50772078</v>
+        <v>3.739820576</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B7">
-        <v>2709</v>
+        <v>2722</v>
       </c>
       <c r="C7">
-        <v>2755.25</v>
+        <v>4158.42</v>
       </c>
       <c r="D7">
-        <v>147.75</v>
+        <v>241.5833333</v>
       </c>
       <c r="E7">
-        <v>51.37446809</v>
+        <v>59.24680851</v>
       </c>
       <c r="F7">
-        <v>241.46</v>
+        <v>278.46</v>
       </c>
       <c r="G7">
-        <v>2.875942185</v>
+        <v>4.077575475</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B8">
-        <v>2722</v>
+        <v>2741</v>
       </c>
       <c r="C8">
-        <v>4158.42</v>
+        <v>3886.67</v>
       </c>
       <c r="D8">
-        <v>241.5833333</v>
+        <v>313.3333333</v>
       </c>
       <c r="E8">
-        <v>59.24680851</v>
+        <v>55.52851064</v>
       </c>
       <c r="F8">
-        <v>278.46</v>
+        <v>260.984</v>
       </c>
       <c r="G8">
-        <v>4.077575475</v>
+        <v>5.642746937</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -11477,25 +11483,25 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B12">
-        <v>2742</v>
+        <v>2739</v>
       </c>
       <c r="C12">
-        <v>790.42</v>
+        <v>1250.58</v>
       </c>
       <c r="D12">
-        <v>709.5833333</v>
+        <v>249.4166667</v>
       </c>
       <c r="E12">
-        <v>56.75531915</v>
+        <v>17.77163121</v>
       </c>
       <c r="F12">
-        <v>266.75</v>
+        <v>83.52666667</v>
       </c>
       <c r="G12">
-        <v>12.50249922</v>
+        <v>14.03453987</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -11522,25 +11528,25 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="B15">
-        <v>2739</v>
+        <v>2742</v>
       </c>
       <c r="C15">
-        <v>1250.58</v>
+        <v>790.42</v>
       </c>
       <c r="D15">
-        <v>249.4166667</v>
+        <v>853.5833333</v>
       </c>
       <c r="E15">
-        <v>17.77163121</v>
+        <v>56.75531915</v>
       </c>
       <c r="F15">
-        <v>83.52666667</v>
+        <v>266.75</v>
       </c>
       <c r="G15">
-        <v>14.03453987</v>
+        <v>15.03970634</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -11707,8 +11713,11 @@
       <c r="B24">
         <v>2738</v>
       </c>
+      <c r="C24">
+        <v>100</v>
+      </c>
       <c r="D24">
-        <v>1399.916667</v>
+        <v>1400</v>
       </c>
       <c r="E24">
         <v>55.52851064</v>
@@ -11717,7 +11726,7 @@
         <v>260.984</v>
       </c>
       <c r="G24">
-        <v>25.21077282</v>
+        <v>25.21227355</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -11768,8 +11777,11 @@
       <c r="B29">
         <v>2727</v>
       </c>
+      <c r="C29">
+        <v>100</v>
+      </c>
       <c r="D29">
-        <v>1398.416667</v>
+        <v>1400</v>
       </c>
       <c r="E29">
         <v>35.05319149</v>
@@ -11778,7 +11790,7 @@
         <v>164.75</v>
       </c>
       <c r="G29">
-        <v>39.89413252</v>
+        <v>39.93930197</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -11913,7 +11925,7 @@
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: motores (19/08/2026 13:09)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1427,8 +1427,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1444,7 +1452,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1452,12 +1460,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1757,70 +1783,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1861,10 +1887,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1876,7 +1902,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1917,10 +1943,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1967,10 +1993,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2014,10 +2040,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2029,7 +2055,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -2070,10 +2096,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2120,10 +2146,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2135,7 +2161,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -2176,10 +2202,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2226,10 +2252,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2241,7 +2267,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2282,10 +2308,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2323,10 +2349,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2338,7 +2364,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46227</v>
       </c>
     </row>
@@ -2379,7 +2405,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2423,10 +2449,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2473,10 +2499,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2488,7 +2514,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2529,10 +2555,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2579,10 +2605,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2594,7 +2620,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2635,10 +2661,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2685,10 +2711,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2700,7 +2726,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2741,10 +2767,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2756,7 +2782,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46153</v>
       </c>
     </row>
@@ -2797,10 +2823,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2812,7 +2838,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2853,10 +2879,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2868,7 +2894,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2909,10 +2935,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2924,7 +2950,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2962,10 +2988,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2974,7 +3000,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -3015,10 +3041,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3027,7 +3053,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -3068,10 +3094,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3118,10 +3144,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3133,7 +3159,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -3174,10 +3200,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3224,10 +3250,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3274,10 +3300,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3324,10 +3350,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3339,7 +3365,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3380,10 +3406,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46220</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3430,10 +3456,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3480,10 +3506,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3495,7 +3521,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3536,10 +3562,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3586,10 +3612,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3636,10 +3662,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3686,10 +3712,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3701,7 +3727,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3742,10 +3768,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3754,7 +3780,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>45351</v>
       </c>
     </row>
@@ -3795,10 +3821,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3842,10 +3868,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3866,22 +3892,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8092,91 +8118,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>255</v>
       </c>
     </row>
@@ -8190,13 +8216,13 @@
       <c r="D2" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>261</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8214,13 +8240,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45491</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <v>45528</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8258,13 +8284,13 @@
       <c r="D3" t="s">
         <v>259</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>261</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8282,13 +8308,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45628</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>45632</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8323,13 +8349,13 @@
       <c r="D4" t="s">
         <v>259</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>261</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8347,13 +8373,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45716</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <v>45722</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="2">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8388,13 +8414,13 @@
       <c r="D5" t="s">
         <v>259</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>261</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8412,13 +8438,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45722</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <v>45782</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8456,13 +8482,13 @@
       <c r="D6" t="s">
         <v>259</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>261</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8480,13 +8506,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45728</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>45734</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8524,7 +8550,7 @@
       <c r="D7" t="s">
         <v>260</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8545,10 +8571,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45772</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8586,7 +8612,7 @@
       <c r="D8" t="s">
         <v>260</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8607,10 +8633,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>45762</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="2">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8648,7 +8674,7 @@
       <c r="D9" t="s">
         <v>260</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8669,10 +8695,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45763</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8710,13 +8736,13 @@
       <c r="D10" t="s">
         <v>259</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>261</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="2">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8734,13 +8760,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45754</v>
       </c>
-      <c r="R10" s="1">
+      <c r="R10" s="2">
         <v>45849</v>
       </c>
-      <c r="S10" s="1">
+      <c r="S10" s="2">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8775,13 +8801,13 @@
       <c r="D11" t="s">
         <v>259</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>261</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="2">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8799,13 +8825,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44973</v>
       </c>
-      <c r="R11" s="1">
+      <c r="R11" s="2">
         <v>45687</v>
       </c>
-      <c r="S11" s="1">
+      <c r="S11" s="2">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8840,13 +8866,13 @@
       <c r="D12" t="s">
         <v>259</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>261</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="2">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8864,13 +8890,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45358</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="2">
         <v>45517</v>
       </c>
-      <c r="S12" s="1">
+      <c r="S12" s="2">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8905,13 +8931,13 @@
       <c r="D13" t="s">
         <v>259</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>261</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="2">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8929,13 +8955,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45572</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="2">
         <v>45572</v>
       </c>
-      <c r="S13" s="1">
+      <c r="S13" s="2">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -8973,13 +8999,13 @@
       <c r="D14" t="s">
         <v>259</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>261</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="2">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -8997,13 +9023,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>45736</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="2">
         <v>46101</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="2">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9039,70 +9065,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9140,10 +9166,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9187,10 +9213,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9234,10 +9260,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9281,10 +9307,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9328,10 +9354,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9375,10 +9401,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9422,10 +9448,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9469,10 +9495,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9516,10 +9542,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9563,10 +9589,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9610,10 +9636,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9657,10 +9683,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9704,10 +9730,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9751,7 +9777,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9792,7 +9818,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9833,10 +9859,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9880,10 +9906,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9927,10 +9953,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -9974,10 +10000,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10021,10 +10047,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10068,10 +10094,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10109,10 +10135,10 @@
       <c r="O23" t="s">
         <v>354</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10124,7 +10150,7 @@
       <c r="T23" t="s">
         <v>394</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -10162,10 +10188,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10177,7 +10203,7 @@
       <c r="T24" t="s">
         <v>395</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -10215,10 +10241,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10230,7 +10256,7 @@
       <c r="T25" t="s">
         <v>396</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -10268,10 +10294,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10283,7 +10309,7 @@
       <c r="T26" t="s">
         <v>397</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -10321,10 +10347,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10336,7 +10362,7 @@
       <c r="T27" t="s">
         <v>398</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -10374,10 +10400,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10389,7 +10415,7 @@
       <c r="T28" t="s">
         <v>399</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -10427,10 +10453,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10442,7 +10468,7 @@
       <c r="T29" t="s">
         <v>400</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -10474,7 +10500,7 @@
       <c r="T30" t="s">
         <v>401</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10506,7 +10532,7 @@
       <c r="T31" t="s">
         <v>402</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10538,7 +10564,7 @@
       <c r="T32" t="s">
         <v>403</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10576,10 +10602,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10591,7 +10617,7 @@
       <c r="T33" t="s">
         <v>382</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -10629,16 +10655,16 @@
       <c r="O34" t="s">
         <v>355</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -10670,10 +10696,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10682,7 +10708,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -10720,10 +10746,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10732,7 +10758,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -10796,10 +10822,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10808,7 +10834,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -10846,10 +10872,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10861,7 +10887,7 @@
       <c r="T39" t="s">
         <v>404</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -10893,10 +10919,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10908,7 +10934,7 @@
       <c r="T40" t="s">
         <v>405</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -10946,10 +10972,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -10961,7 +10987,7 @@
       <c r="T41" t="s">
         <v>406</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -10999,10 +11025,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11014,7 +11040,7 @@
       <c r="T42" t="s">
         <v>407</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -11052,10 +11078,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11067,7 +11093,7 @@
       <c r="T43" t="s">
         <v>408</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -11105,10 +11131,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11120,7 +11146,7 @@
       <c r="T44" t="s">
         <v>409</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -11158,10 +11184,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11173,7 +11199,7 @@
       <c r="T45" t="s">
         <v>410</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -11211,10 +11237,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11226,7 +11252,7 @@
       <c r="T46" t="s">
         <v>411</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -11241,25 +11267,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>416</v>
       </c>
     </row>
@@ -11939,22 +11965,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>422</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (21/08/2026 09:08)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1433,8 +1433,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1450,7 +1458,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1458,12 +1466,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1763,70 +1789,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1867,10 +1893,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1882,7 +1908,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1923,10 +1949,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1973,10 +1999,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2020,10 +2046,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2035,7 +2061,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -2076,10 +2102,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2126,10 +2152,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2141,7 +2167,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -2182,10 +2208,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2232,10 +2258,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2247,7 +2273,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2288,10 +2314,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2329,10 +2355,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2344,7 +2370,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46227</v>
       </c>
     </row>
@@ -2385,7 +2411,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2429,10 +2455,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2479,10 +2505,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2494,7 +2520,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2535,10 +2561,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2585,10 +2611,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2600,7 +2626,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2641,10 +2667,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2691,10 +2717,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2706,7 +2732,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2747,10 +2773,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2762,7 +2788,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46153</v>
       </c>
     </row>
@@ -2803,10 +2829,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2818,7 +2844,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2859,10 +2885,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2874,7 +2900,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2915,10 +2941,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2930,7 +2956,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2968,10 +2994,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2980,7 +3006,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -3021,10 +3047,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3033,7 +3059,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -3074,10 +3100,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3124,10 +3150,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3139,7 +3165,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -3180,10 +3206,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3230,10 +3256,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3280,10 +3306,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3330,10 +3356,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3345,7 +3371,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3386,10 +3412,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46220</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3436,10 +3462,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3486,10 +3512,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3501,7 +3527,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3542,10 +3568,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3592,10 +3618,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3642,10 +3668,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3692,10 +3718,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3707,7 +3733,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3748,10 +3774,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3760,7 +3786,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>45351</v>
       </c>
     </row>
@@ -3801,10 +3827,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3848,10 +3874,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3872,22 +3898,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8132,91 +8158,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>257</v>
       </c>
     </row>
@@ -8230,13 +8256,13 @@
       <c r="D2" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>263</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8254,13 +8280,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45491</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <v>45528</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8298,13 +8324,13 @@
       <c r="D3" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>263</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8322,13 +8348,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45628</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>45632</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8363,13 +8389,13 @@
       <c r="D4" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>263</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8387,13 +8413,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45716</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <v>45722</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="2">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8428,13 +8454,13 @@
       <c r="D5" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>263</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8452,13 +8478,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45722</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <v>45782</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8496,13 +8522,13 @@
       <c r="D6" t="s">
         <v>261</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8520,13 +8546,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45728</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>45734</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8564,7 +8590,7 @@
       <c r="D7" t="s">
         <v>262</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8585,10 +8611,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45772</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8626,7 +8652,7 @@
       <c r="D8" t="s">
         <v>262</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8647,10 +8673,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>45762</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="2">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8688,7 +8714,7 @@
       <c r="D9" t="s">
         <v>262</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8709,10 +8735,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45763</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8750,13 +8776,13 @@
       <c r="D10" t="s">
         <v>261</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>263</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="2">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8774,13 +8800,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45754</v>
       </c>
-      <c r="R10" s="1">
+      <c r="R10" s="2">
         <v>45849</v>
       </c>
-      <c r="S10" s="1">
+      <c r="S10" s="2">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8815,13 +8841,13 @@
       <c r="D11" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>263</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="2">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8839,13 +8865,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44973</v>
       </c>
-      <c r="R11" s="1">
+      <c r="R11" s="2">
         <v>45687</v>
       </c>
-      <c r="S11" s="1">
+      <c r="S11" s="2">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8880,13 +8906,13 @@
       <c r="D12" t="s">
         <v>261</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>263</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="2">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8904,13 +8930,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45358</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="2">
         <v>45517</v>
       </c>
-      <c r="S12" s="1">
+      <c r="S12" s="2">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8945,13 +8971,13 @@
       <c r="D13" t="s">
         <v>261</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>263</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="2">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8969,13 +8995,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45572</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="2">
         <v>45572</v>
       </c>
-      <c r="S13" s="1">
+      <c r="S13" s="2">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -9013,13 +9039,13 @@
       <c r="D14" t="s">
         <v>261</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>263</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="2">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -9037,13 +9063,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>45736</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="2">
         <v>46101</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="2">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9079,70 +9105,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9180,10 +9206,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9227,10 +9253,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9274,10 +9300,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9321,10 +9347,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9368,10 +9394,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9415,10 +9441,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9462,10 +9488,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9509,10 +9535,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9556,10 +9582,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9603,10 +9629,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9650,10 +9676,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9697,10 +9723,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9744,10 +9770,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9791,7 +9817,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9832,7 +9858,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9873,10 +9899,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9920,10 +9946,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9967,10 +9993,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -10014,10 +10040,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10061,10 +10087,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10108,10 +10134,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10149,10 +10175,10 @@
       <c r="O23" t="s">
         <v>356</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10164,7 +10190,7 @@
       <c r="T23" t="s">
         <v>396</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -10202,10 +10228,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10217,7 +10243,7 @@
       <c r="T24" t="s">
         <v>397</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -10255,10 +10281,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10270,7 +10296,7 @@
       <c r="T25" t="s">
         <v>398</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -10308,10 +10334,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10323,7 +10349,7 @@
       <c r="T26" t="s">
         <v>399</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -10361,10 +10387,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10376,7 +10402,7 @@
       <c r="T27" t="s">
         <v>400</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -10414,10 +10440,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10429,7 +10455,7 @@
       <c r="T28" t="s">
         <v>401</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -10467,10 +10493,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10482,7 +10508,7 @@
       <c r="T29" t="s">
         <v>402</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -10514,7 +10540,7 @@
       <c r="T30" t="s">
         <v>403</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10546,7 +10572,7 @@
       <c r="T31" t="s">
         <v>404</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10578,7 +10604,7 @@
       <c r="T32" t="s">
         <v>405</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10616,10 +10642,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10631,7 +10657,7 @@
       <c r="T33" t="s">
         <v>384</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -10669,16 +10695,16 @@
       <c r="O34" t="s">
         <v>357</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -10710,10 +10736,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10722,7 +10748,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -10760,10 +10786,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10772,7 +10798,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -10836,10 +10862,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10848,7 +10874,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -10886,10 +10912,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10901,7 +10927,7 @@
       <c r="T39" t="s">
         <v>406</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -10933,10 +10959,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10948,7 +10974,7 @@
       <c r="T40" t="s">
         <v>407</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -10986,10 +11012,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -11001,7 +11027,7 @@
       <c r="T41" t="s">
         <v>408</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -11039,10 +11065,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11054,7 +11080,7 @@
       <c r="T42" t="s">
         <v>409</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -11092,10 +11118,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11107,7 +11133,7 @@
       <c r="T43" t="s">
         <v>410</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -11145,10 +11171,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11160,7 +11186,7 @@
       <c r="T44" t="s">
         <v>411</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -11198,10 +11224,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11213,7 +11239,7 @@
       <c r="T45" t="s">
         <v>412</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -11251,10 +11277,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11266,7 +11292,7 @@
       <c r="T46" t="s">
         <v>413</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -11281,25 +11307,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>418</v>
       </c>
     </row>
@@ -11979,22 +12005,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>424</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (21/08/2026 10:53)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1433,16 +1433,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1458,7 +1450,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1466,30 +1458,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1789,70 +1763,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1893,10 +1867,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1908,7 +1882,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1949,10 +1923,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1999,10 +1973,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2046,10 +2020,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2061,7 +2035,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -2102,10 +2076,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2152,10 +2126,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2167,7 +2141,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2208,10 +2182,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2258,10 +2232,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2273,7 +2247,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2314,10 +2288,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2355,10 +2329,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2370,7 +2344,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46227</v>
       </c>
     </row>
@@ -2411,7 +2385,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2455,10 +2429,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2505,10 +2479,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2520,7 +2494,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2561,10 +2535,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2611,10 +2585,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2626,7 +2600,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2667,10 +2641,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2717,10 +2691,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2732,7 +2706,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2773,10 +2747,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2788,7 +2762,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
     </row>
@@ -2829,10 +2803,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2844,7 +2818,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2885,10 +2859,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2900,7 +2874,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2941,10 +2915,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2956,7 +2930,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2994,10 +2968,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -3006,7 +2980,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -3047,10 +3021,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3059,7 +3033,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -3100,10 +3074,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3150,10 +3124,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3165,7 +3139,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3206,10 +3180,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3256,10 +3230,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3306,10 +3280,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3356,10 +3330,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3371,7 +3345,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3412,10 +3386,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46220</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3462,10 +3436,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3512,10 +3486,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3527,7 +3501,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3568,10 +3542,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3618,10 +3592,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3668,10 +3642,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3718,10 +3692,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3733,7 +3707,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3774,10 +3748,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3786,7 +3760,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>45351</v>
       </c>
     </row>
@@ -3827,10 +3801,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3874,10 +3848,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3898,22 +3872,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8158,91 +8132,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>235</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>236</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>237</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>238</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>239</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>240</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>241</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>242</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>243</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>244</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>245</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>246</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>247</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>248</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>249</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>250</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>251</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>252</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>253</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>254</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>255</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>256</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>257</v>
       </c>
     </row>
@@ -8256,13 +8230,13 @@
       <c r="D2" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>263</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8280,13 +8254,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8324,13 +8298,13 @@
       <c r="D3" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>263</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8348,13 +8322,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8389,13 +8363,13 @@
       <c r="D4" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>263</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8413,13 +8387,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8454,13 +8428,13 @@
       <c r="D5" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>263</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8478,13 +8452,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8522,13 +8496,13 @@
       <c r="D6" t="s">
         <v>261</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8546,13 +8520,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8590,7 +8564,7 @@
       <c r="D7" t="s">
         <v>262</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8611,10 +8585,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8652,7 +8626,7 @@
       <c r="D8" t="s">
         <v>262</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8673,10 +8647,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8714,7 +8688,7 @@
       <c r="D9" t="s">
         <v>262</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8735,10 +8709,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8776,13 +8750,13 @@
       <c r="D10" t="s">
         <v>261</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>263</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8800,13 +8774,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8841,13 +8815,13 @@
       <c r="D11" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>263</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8865,13 +8839,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8906,13 +8880,13 @@
       <c r="D12" t="s">
         <v>261</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>263</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8930,13 +8904,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8971,13 +8945,13 @@
       <c r="D13" t="s">
         <v>261</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>263</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8995,13 +8969,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -9039,13 +9013,13 @@
       <c r="D14" t="s">
         <v>261</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>263</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -9063,13 +9037,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9105,70 +9079,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9206,10 +9180,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9253,10 +9227,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9300,10 +9274,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9347,10 +9321,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9394,10 +9368,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9441,10 +9415,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9488,10 +9462,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9535,10 +9509,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9582,10 +9556,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9629,10 +9603,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9676,10 +9650,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9723,10 +9697,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9770,10 +9744,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9817,7 +9791,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9858,7 +9832,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9899,10 +9873,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9946,10 +9920,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9993,10 +9967,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -10040,10 +10014,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10087,10 +10061,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10134,10 +10108,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10175,10 +10149,10 @@
       <c r="O23" t="s">
         <v>356</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10190,7 +10164,7 @@
       <c r="T23" t="s">
         <v>396</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10228,10 +10202,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10243,7 +10217,7 @@
       <c r="T24" t="s">
         <v>397</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10281,10 +10255,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10296,7 +10270,7 @@
       <c r="T25" t="s">
         <v>398</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10334,10 +10308,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10349,7 +10323,7 @@
       <c r="T26" t="s">
         <v>399</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10387,10 +10361,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10402,7 +10376,7 @@
       <c r="T27" t="s">
         <v>400</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10440,10 +10414,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10455,7 +10429,7 @@
       <c r="T28" t="s">
         <v>401</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10493,10 +10467,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10508,7 +10482,7 @@
       <c r="T29" t="s">
         <v>402</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10540,7 +10514,7 @@
       <c r="T30" t="s">
         <v>403</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10572,7 +10546,7 @@
       <c r="T31" t="s">
         <v>404</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10604,7 +10578,7 @@
       <c r="T32" t="s">
         <v>405</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10642,10 +10616,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10657,7 +10631,7 @@
       <c r="T33" t="s">
         <v>384</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10695,16 +10669,16 @@
       <c r="O34" t="s">
         <v>357</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10736,10 +10710,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10748,7 +10722,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10786,10 +10760,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10798,7 +10772,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10862,10 +10836,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10874,7 +10848,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10912,10 +10886,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10927,7 +10901,7 @@
       <c r="T39" t="s">
         <v>406</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10959,10 +10933,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10974,7 +10948,7 @@
       <c r="T40" t="s">
         <v>407</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -11012,10 +10986,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -11027,7 +11001,7 @@
       <c r="T41" t="s">
         <v>408</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -11065,10 +11039,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11080,7 +11054,7 @@
       <c r="T42" t="s">
         <v>409</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -11118,10 +11092,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11133,7 +11107,7 @@
       <c r="T43" t="s">
         <v>410</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -11171,10 +11145,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11186,7 +11160,7 @@
       <c r="T44" t="s">
         <v>411</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11224,10 +11198,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11239,7 +11213,7 @@
       <c r="T45" t="s">
         <v>412</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11277,10 +11251,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11292,7 +11266,7 @@
       <c r="T46" t="s">
         <v>413</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11307,25 +11281,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>414</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>415</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>416</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>417</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>418</v>
       </c>
     </row>
@@ -12005,22 +11979,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>419</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>420</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>421</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>422</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>423</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>424</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (25/08/2026 08:32)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1433,8 +1433,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1450,7 +1458,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1458,12 +1466,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1763,70 +1789,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1867,10 +1893,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1882,7 +1908,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1923,10 +1949,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1973,10 +1999,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2020,10 +2046,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2035,7 +2061,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -2076,10 +2102,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2126,10 +2152,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2141,7 +2167,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -2182,10 +2208,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2232,10 +2258,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2247,7 +2273,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2288,10 +2314,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2329,10 +2355,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2344,7 +2370,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46227</v>
       </c>
     </row>
@@ -2385,7 +2411,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2429,10 +2455,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2479,10 +2505,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2494,7 +2520,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2535,10 +2561,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2585,10 +2611,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2600,7 +2626,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2641,10 +2667,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2691,10 +2717,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2706,7 +2732,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2747,10 +2773,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2762,7 +2788,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46153</v>
       </c>
     </row>
@@ -2803,10 +2829,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2818,7 +2844,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2859,10 +2885,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2874,7 +2900,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2915,10 +2941,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2930,7 +2956,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2968,10 +2994,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2980,7 +3006,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -3021,10 +3047,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3033,7 +3059,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>46220</v>
       </c>
     </row>
@@ -3074,10 +3100,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3124,10 +3150,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3139,7 +3165,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -3180,10 +3206,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3230,10 +3256,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3280,10 +3306,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3330,10 +3356,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3345,7 +3371,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3386,10 +3412,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46220</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3436,10 +3462,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3486,10 +3512,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3501,7 +3527,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3542,10 +3568,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3592,10 +3618,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3642,10 +3668,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3692,10 +3718,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3707,7 +3733,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3748,10 +3774,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3760,7 +3786,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>45351</v>
       </c>
     </row>
@@ -3801,10 +3827,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3848,10 +3874,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3872,22 +3898,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8132,91 +8158,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>257</v>
       </c>
     </row>
@@ -8230,13 +8256,13 @@
       <c r="D2" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>263</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8254,13 +8280,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45491</v>
       </c>
-      <c r="R2" s="1">
+      <c r="R2" s="2">
         <v>45528</v>
       </c>
-      <c r="S2" s="1">
+      <c r="S2" s="2">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8298,13 +8324,13 @@
       <c r="D3" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>263</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8322,13 +8348,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45628</v>
       </c>
-      <c r="R3" s="1">
+      <c r="R3" s="2">
         <v>45632</v>
       </c>
-      <c r="S3" s="1">
+      <c r="S3" s="2">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8363,13 +8389,13 @@
       <c r="D4" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>263</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="2">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8387,13 +8413,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45716</v>
       </c>
-      <c r="R4" s="1">
+      <c r="R4" s="2">
         <v>45722</v>
       </c>
-      <c r="S4" s="1">
+      <c r="S4" s="2">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8428,13 +8454,13 @@
       <c r="D5" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>263</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5" s="2">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8452,13 +8478,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45722</v>
       </c>
-      <c r="R5" s="1">
+      <c r="R5" s="2">
         <v>45782</v>
       </c>
-      <c r="S5" s="1">
+      <c r="S5" s="2">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8496,13 +8522,13 @@
       <c r="D6" t="s">
         <v>261</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6" s="2">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8520,13 +8546,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45728</v>
       </c>
-      <c r="R6" s="1">
+      <c r="R6" s="2">
         <v>45734</v>
       </c>
-      <c r="S6" s="1">
+      <c r="S6" s="2">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8564,7 +8590,7 @@
       <c r="D7" t="s">
         <v>262</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8585,10 +8611,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45772</v>
       </c>
-      <c r="R7" s="1">
+      <c r="R7" s="2">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8626,7 +8652,7 @@
       <c r="D8" t="s">
         <v>262</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8647,10 +8673,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>45762</v>
       </c>
-      <c r="R8" s="1">
+      <c r="R8" s="2">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8688,7 +8714,7 @@
       <c r="D9" t="s">
         <v>262</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8709,10 +8735,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45763</v>
       </c>
-      <c r="R9" s="1">
+      <c r="R9" s="2">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8750,13 +8776,13 @@
       <c r="D10" t="s">
         <v>261</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>263</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10" s="2">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8774,13 +8800,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45754</v>
       </c>
-      <c r="R10" s="1">
+      <c r="R10" s="2">
         <v>45849</v>
       </c>
-      <c r="S10" s="1">
+      <c r="S10" s="2">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8815,13 +8841,13 @@
       <c r="D11" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>263</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11" s="2">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8839,13 +8865,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44973</v>
       </c>
-      <c r="R11" s="1">
+      <c r="R11" s="2">
         <v>45687</v>
       </c>
-      <c r="S11" s="1">
+      <c r="S11" s="2">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8880,13 +8906,13 @@
       <c r="D12" t="s">
         <v>261</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>263</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12" s="2">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8904,13 +8930,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45358</v>
       </c>
-      <c r="R12" s="1">
+      <c r="R12" s="2">
         <v>45517</v>
       </c>
-      <c r="S12" s="1">
+      <c r="S12" s="2">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8945,13 +8971,13 @@
       <c r="D13" t="s">
         <v>261</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>263</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13" s="2">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8969,13 +8995,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45572</v>
       </c>
-      <c r="R13" s="1">
+      <c r="R13" s="2">
         <v>45572</v>
       </c>
-      <c r="S13" s="1">
+      <c r="S13" s="2">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -9013,13 +9039,13 @@
       <c r="D14" t="s">
         <v>261</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>263</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="2">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -9037,13 +9063,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>45736</v>
       </c>
-      <c r="R14" s="1">
+      <c r="R14" s="2">
         <v>46101</v>
       </c>
-      <c r="S14" s="1">
+      <c r="S14" s="2">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9079,70 +9105,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9180,10 +9206,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9227,10 +9253,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9274,10 +9300,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9321,10 +9347,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9368,10 +9394,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9415,10 +9441,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9462,10 +9488,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9509,10 +9535,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9556,10 +9582,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9603,10 +9629,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9650,10 +9676,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9697,10 +9723,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9744,10 +9770,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9791,7 +9817,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9832,7 +9858,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9873,10 +9899,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9920,10 +9946,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9967,10 +9993,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -10014,10 +10040,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10061,10 +10087,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10108,10 +10134,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10149,10 +10175,10 @@
       <c r="O23" t="s">
         <v>356</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10164,7 +10190,7 @@
       <c r="T23" t="s">
         <v>396</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -10202,10 +10228,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10217,7 +10243,7 @@
       <c r="T24" t="s">
         <v>397</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -10255,10 +10281,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10270,7 +10296,7 @@
       <c r="T25" t="s">
         <v>398</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -10308,10 +10334,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10323,7 +10349,7 @@
       <c r="T26" t="s">
         <v>399</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -10361,10 +10387,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10376,7 +10402,7 @@
       <c r="T27" t="s">
         <v>400</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -10414,10 +10440,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10429,7 +10455,7 @@
       <c r="T28" t="s">
         <v>401</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -10467,10 +10493,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10482,7 +10508,7 @@
       <c r="T29" t="s">
         <v>402</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -10514,7 +10540,7 @@
       <c r="T30" t="s">
         <v>403</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10546,7 +10572,7 @@
       <c r="T31" t="s">
         <v>404</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10578,7 +10604,7 @@
       <c r="T32" t="s">
         <v>405</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -10616,10 +10642,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10631,7 +10657,7 @@
       <c r="T33" t="s">
         <v>384</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -10669,16 +10695,16 @@
       <c r="O34" t="s">
         <v>357</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -10710,10 +10736,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10722,7 +10748,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -10760,10 +10786,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10772,7 +10798,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -10836,10 +10862,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10848,7 +10874,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -10886,10 +10912,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10901,7 +10927,7 @@
       <c r="T39" t="s">
         <v>406</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -10933,10 +10959,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10948,7 +10974,7 @@
       <c r="T40" t="s">
         <v>407</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -10986,10 +11012,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -11001,7 +11027,7 @@
       <c r="T41" t="s">
         <v>408</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -11039,10 +11065,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11054,7 +11080,7 @@
       <c r="T42" t="s">
         <v>409</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -11092,10 +11118,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11107,7 +11133,7 @@
       <c r="T43" t="s">
         <v>410</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -11145,10 +11171,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11160,7 +11186,7 @@
       <c r="T44" t="s">
         <v>411</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -11198,10 +11224,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11213,7 +11239,7 @@
       <c r="T45" t="s">
         <v>412</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -11251,10 +11277,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11266,7 +11292,7 @@
       <c r="T46" t="s">
         <v>413</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -11281,25 +11307,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>418</v>
       </c>
     </row>
@@ -11979,22 +12005,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>424</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (25/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1433,16 +1433,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1458,7 +1450,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1466,30 +1458,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1789,70 +1763,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1893,10 +1867,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1908,7 +1882,7 @@
       <c r="T2" t="s">
         <v>150</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1949,10 +1923,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1999,10 +1973,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -2046,10 +2020,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -2061,7 +2035,7 @@
       <c r="T5" t="s">
         <v>151</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -2102,10 +2076,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -2152,10 +2126,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -2167,7 +2141,7 @@
       <c r="T7" t="s">
         <v>152</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2208,10 +2182,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2258,10 +2232,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2273,7 +2247,7 @@
       <c r="T9" t="s">
         <v>153</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2314,10 +2288,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2355,10 +2329,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2370,7 +2344,7 @@
       <c r="T11" t="s">
         <v>154</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46227</v>
       </c>
     </row>
@@ -2411,7 +2385,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2455,10 +2429,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2505,10 +2479,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2520,7 +2494,7 @@
       <c r="T14" t="s">
         <v>155</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2561,10 +2535,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2611,10 +2585,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2626,7 +2600,7 @@
       <c r="T16" t="s">
         <v>156</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2667,10 +2641,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2717,10 +2691,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2732,7 +2706,7 @@
       <c r="T18" t="s">
         <v>157</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2773,10 +2747,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2788,7 +2762,7 @@
       <c r="T19" t="s">
         <v>124</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46153</v>
       </c>
     </row>
@@ -2829,10 +2803,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2844,7 +2818,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2885,10 +2859,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2900,7 +2874,7 @@
       <c r="T21" t="s">
         <v>126</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2941,10 +2915,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2956,7 +2930,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2994,10 +2968,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -3006,7 +2980,7 @@
       <c r="S23" t="s">
         <v>149</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -3047,10 +3021,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -3059,7 +3033,7 @@
       <c r="S24" t="s">
         <v>149</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>46220</v>
       </c>
     </row>
@@ -3100,10 +3074,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -3150,10 +3124,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -3165,7 +3139,7 @@
       <c r="T26" t="s">
         <v>160</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3206,10 +3180,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3256,10 +3230,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3306,10 +3280,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3356,10 +3330,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3371,7 +3345,7 @@
       <c r="T30" t="s">
         <v>161</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3412,10 +3386,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46220</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46220</v>
       </c>
       <c r="R31" t="s">
@@ -3462,10 +3436,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3512,10 +3486,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3527,7 +3501,7 @@
       <c r="T33" t="s">
         <v>162</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3568,10 +3542,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>44910</v>
       </c>
       <c r="R34" t="s">
@@ -3618,10 +3592,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3668,10 +3642,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3718,10 +3692,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3733,7 +3707,7 @@
       <c r="T37" t="s">
         <v>163</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3774,10 +3748,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3786,7 +3760,7 @@
       <c r="T38" t="s">
         <v>164</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>45351</v>
       </c>
     </row>
@@ -3827,10 +3801,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3874,10 +3848,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3898,22 +3872,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>169</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>170</v>
       </c>
     </row>
@@ -8158,91 +8132,91 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:29">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>234</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>235</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>236</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>237</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>238</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>239</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>240</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>241</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>242</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>243</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>244</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>245</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>246</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>247</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>248</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>249</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>250</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>251</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>252</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>253</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>254</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>255</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" t="s">
         <v>256</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" t="s">
         <v>257</v>
       </c>
     </row>
@@ -8256,13 +8230,13 @@
       <c r="D2" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45686</v>
       </c>
       <c r="F2" t="s">
         <v>263</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="1">
         <v>45492</v>
       </c>
       <c r="H2" t="s">
@@ -8280,13 +8254,13 @@
       <c r="P2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45491</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="1">
         <v>45528</v>
       </c>
-      <c r="S2" s="2">
+      <c r="S2" s="1">
         <v>45492</v>
       </c>
       <c r="U2" t="s">
@@ -8324,13 +8298,13 @@
       <c r="D3" t="s">
         <v>261</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45728</v>
       </c>
       <c r="F3" t="s">
         <v>263</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>45631</v>
       </c>
       <c r="H3" t="s">
@@ -8348,13 +8322,13 @@
       <c r="P3">
         <v>1</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45628</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="1">
         <v>45632</v>
       </c>
-      <c r="S3" s="2">
+      <c r="S3" s="1">
         <v>45631</v>
       </c>
       <c r="U3" t="s">
@@ -8389,13 +8363,13 @@
       <c r="D4" t="s">
         <v>261</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45716</v>
       </c>
       <c r="F4" t="s">
         <v>263</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="1">
         <v>45716</v>
       </c>
       <c r="H4" t="s">
@@ -8413,13 +8387,13 @@
       <c r="P4">
         <v>1</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45716</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="1">
         <v>45722</v>
       </c>
-      <c r="S4" s="2">
+      <c r="S4" s="1">
         <v>45716</v>
       </c>
       <c r="U4" t="s">
@@ -8454,13 +8428,13 @@
       <c r="D5" t="s">
         <v>261</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45728</v>
       </c>
       <c r="F5" t="s">
         <v>263</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>45728</v>
       </c>
       <c r="H5" t="s">
@@ -8478,13 +8452,13 @@
       <c r="P5">
         <v>1</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45722</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="1">
         <v>45782</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="1">
         <v>45728</v>
       </c>
       <c r="U5" t="s">
@@ -8522,13 +8496,13 @@
       <c r="D6" t="s">
         <v>261</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45755</v>
       </c>
       <c r="F6" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="1">
         <v>45755</v>
       </c>
       <c r="H6" t="s">
@@ -8546,13 +8520,13 @@
       <c r="P6">
         <v>1</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45728</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="1">
         <v>45734</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="1">
         <v>45755</v>
       </c>
       <c r="U6" t="s">
@@ -8590,7 +8564,7 @@
       <c r="D7" t="s">
         <v>262</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45772</v>
       </c>
       <c r="F7" t="s">
@@ -8611,10 +8585,10 @@
       <c r="P7">
         <v>1</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45772</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="1">
         <v>45775</v>
       </c>
       <c r="U7" t="s">
@@ -8652,7 +8626,7 @@
       <c r="D8" t="s">
         <v>262</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45762</v>
       </c>
       <c r="F8" t="s">
@@ -8673,10 +8647,10 @@
       <c r="P8">
         <v>1</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>45762</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="1">
         <v>45770</v>
       </c>
       <c r="U8" t="s">
@@ -8714,7 +8688,7 @@
       <c r="D9" t="s">
         <v>262</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45763</v>
       </c>
       <c r="F9" t="s">
@@ -8735,10 +8709,10 @@
       <c r="P9">
         <v>1</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45763</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="1">
         <v>45777</v>
       </c>
       <c r="U9" t="s">
@@ -8776,13 +8750,13 @@
       <c r="D10" t="s">
         <v>261</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45755</v>
       </c>
       <c r="F10" t="s">
         <v>263</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="1">
         <v>45755</v>
       </c>
       <c r="H10" t="s">
@@ -8800,13 +8774,13 @@
       <c r="P10">
         <v>1</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45754</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="1">
         <v>45849</v>
       </c>
-      <c r="S10" s="2">
+      <c r="S10" s="1">
         <v>45754</v>
       </c>
       <c r="U10" t="s">
@@ -8841,13 +8815,13 @@
       <c r="D11" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>44973</v>
       </c>
       <c r="F11" t="s">
         <v>263</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>44973</v>
       </c>
       <c r="H11" t="s">
@@ -8865,13 +8839,13 @@
       <c r="P11">
         <v>1</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44973</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="1">
         <v>45687</v>
       </c>
-      <c r="S11" s="2">
+      <c r="S11" s="1">
         <v>44973</v>
       </c>
       <c r="U11" t="s">
@@ -8906,13 +8880,13 @@
       <c r="D12" t="s">
         <v>261</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>45358</v>
       </c>
       <c r="F12" t="s">
         <v>263</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="1">
         <v>45358</v>
       </c>
       <c r="H12" t="s">
@@ -8930,13 +8904,13 @@
       <c r="P12">
         <v>1</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45358</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="1">
         <v>45517</v>
       </c>
-      <c r="S12" s="2">
+      <c r="S12" s="1">
         <v>45358</v>
       </c>
       <c r="U12" t="s">
@@ -8971,13 +8945,13 @@
       <c r="D13" t="s">
         <v>261</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>45573</v>
       </c>
       <c r="F13" t="s">
         <v>263</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="1">
         <v>45573</v>
       </c>
       <c r="H13" t="s">
@@ -8995,13 +8969,13 @@
       <c r="P13">
         <v>1</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45572</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="1">
         <v>45572</v>
       </c>
-      <c r="S13" s="2">
+      <c r="S13" s="1">
         <v>45573</v>
       </c>
       <c r="U13" t="s">
@@ -9039,13 +9013,13 @@
       <c r="D14" t="s">
         <v>261</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>45747</v>
       </c>
       <c r="F14" t="s">
         <v>263</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="1">
         <v>45747</v>
       </c>
       <c r="H14" t="s">
@@ -9063,13 +9037,13 @@
       <c r="P14">
         <v>1</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>45736</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="1">
         <v>46101</v>
       </c>
-      <c r="S14" s="2">
+      <c r="S14" s="1">
         <v>45747</v>
       </c>
       <c r="U14" t="s">
@@ -9105,70 +9079,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -9206,10 +9180,10 @@
       <c r="O2" t="s">
         <v>104</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -9253,10 +9227,10 @@
       <c r="O3" t="s">
         <v>83</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -9300,10 +9274,10 @@
       <c r="O4" t="s">
         <v>99</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -9347,10 +9321,10 @@
       <c r="O5" t="s">
         <v>100</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -9394,10 +9368,10 @@
       <c r="O6" t="s">
         <v>97</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -9441,10 +9415,10 @@
       <c r="O7" t="s">
         <v>85</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -9488,10 +9462,10 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -9535,10 +9509,10 @@
       <c r="O9" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -9582,10 +9556,10 @@
       <c r="O10" t="s">
         <v>91</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -9629,10 +9603,10 @@
       <c r="O11" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -9676,10 +9650,10 @@
       <c r="O12" t="s">
         <v>84</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -9723,10 +9697,10 @@
       <c r="O13" t="s">
         <v>82</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -9770,10 +9744,10 @@
       <c r="O14" t="s">
         <v>102</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -9817,7 +9791,7 @@
       <c r="O15" t="s">
         <v>96</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -9858,7 +9832,7 @@
       <c r="O16" t="s">
         <v>92</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -9899,10 +9873,10 @@
       <c r="O17" t="s">
         <v>95</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -9946,10 +9920,10 @@
       <c r="O18" t="s">
         <v>93</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -9993,10 +9967,10 @@
       <c r="O19" t="s">
         <v>106</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -10040,10 +10014,10 @@
       <c r="O20" t="s">
         <v>98</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -10087,10 +10061,10 @@
       <c r="O21" t="s">
         <v>107</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -10134,10 +10108,10 @@
       <c r="O22" t="s">
         <v>88</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -10175,10 +10149,10 @@
       <c r="O23" t="s">
         <v>356</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -10190,7 +10164,7 @@
       <c r="T23" t="s">
         <v>396</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -10228,10 +10202,10 @@
       <c r="O24" t="s">
         <v>82</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -10243,7 +10217,7 @@
       <c r="T24" t="s">
         <v>397</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -10281,10 +10255,10 @@
       <c r="O25" t="s">
         <v>88</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -10296,7 +10270,7 @@
       <c r="T25" t="s">
         <v>398</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -10334,10 +10308,10 @@
       <c r="O26" t="s">
         <v>102</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -10349,7 +10323,7 @@
       <c r="T26" t="s">
         <v>399</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -10387,10 +10361,10 @@
       <c r="O27" t="s">
         <v>88</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -10402,7 +10376,7 @@
       <c r="T27" t="s">
         <v>400</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -10440,10 +10414,10 @@
       <c r="O28" t="s">
         <v>103</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -10455,7 +10429,7 @@
       <c r="T28" t="s">
         <v>401</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -10493,10 +10467,10 @@
       <c r="O29" t="s">
         <v>100</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -10508,7 +10482,7 @@
       <c r="T29" t="s">
         <v>402</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -10540,7 +10514,7 @@
       <c r="T30" t="s">
         <v>403</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10572,7 +10546,7 @@
       <c r="T31" t="s">
         <v>404</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10604,7 +10578,7 @@
       <c r="T32" t="s">
         <v>405</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -10642,10 +10616,10 @@
       <c r="O33" t="s">
         <v>92</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -10657,7 +10631,7 @@
       <c r="T33" t="s">
         <v>384</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -10695,16 +10669,16 @@
       <c r="O34" t="s">
         <v>357</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>149</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -10736,10 +10710,10 @@
       <c r="O35" t="s">
         <v>89</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -10748,7 +10722,7 @@
       <c r="S35" t="s">
         <v>149</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -10786,10 +10760,10 @@
       <c r="O36" t="s">
         <v>93</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -10798,7 +10772,7 @@
       <c r="S36" t="s">
         <v>149</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -10862,10 +10836,10 @@
       <c r="O38" t="s">
         <v>98</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -10874,7 +10848,7 @@
       <c r="S38" t="s">
         <v>149</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -10912,10 +10886,10 @@
       <c r="O39" t="s">
         <v>105</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -10927,7 +10901,7 @@
       <c r="T39" t="s">
         <v>406</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -10959,10 +10933,10 @@
       <c r="O40" t="s">
         <v>102</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -10974,7 +10948,7 @@
       <c r="T40" t="s">
         <v>407</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -11012,10 +10986,10 @@
       <c r="O41" t="s">
         <v>97</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -11027,7 +11001,7 @@
       <c r="T41" t="s">
         <v>408</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -11065,10 +11039,10 @@
       <c r="O42" t="s">
         <v>84</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -11080,7 +11054,7 @@
       <c r="T42" t="s">
         <v>409</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -11118,10 +11092,10 @@
       <c r="O43" t="s">
         <v>86</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -11133,7 +11107,7 @@
       <c r="T43" t="s">
         <v>410</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -11171,10 +11145,10 @@
       <c r="O44" t="s">
         <v>99</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -11186,7 +11160,7 @@
       <c r="T44" t="s">
         <v>411</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -11224,10 +11198,10 @@
       <c r="O45" t="s">
         <v>83</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -11239,7 +11213,7 @@
       <c r="T45" t="s">
         <v>412</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -11277,10 +11251,10 @@
       <c r="O46" t="s">
         <v>90</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -11292,7 +11266,7 @@
       <c r="T46" t="s">
         <v>413</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -11307,25 +11281,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>166</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>414</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>415</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>416</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>417</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>418</v>
       </c>
     </row>
@@ -12005,22 +11979,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>419</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>420</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>421</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>422</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>423</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>424</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (03/09/2026 13:44)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1237,8 +1237,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1254,7 +1262,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1262,12 +1270,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1567,70 +1593,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1671,10 +1697,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1686,7 +1712,7 @@
       <c r="T2" t="s">
         <v>149</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1727,10 +1753,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1777,10 +1803,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1827,10 +1853,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1842,7 +1868,7 @@
       <c r="T5" t="s">
         <v>150</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -1883,10 +1909,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -1933,10 +1959,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -1948,7 +1974,7 @@
       <c r="T7" t="s">
         <v>151</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -1989,10 +2015,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2039,10 +2065,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2054,7 +2080,7 @@
       <c r="T9" t="s">
         <v>152</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2095,10 +2121,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2139,10 +2165,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2154,7 +2180,7 @@
       <c r="T11" t="s">
         <v>153</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46227</v>
       </c>
     </row>
@@ -2195,7 +2221,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2239,10 +2265,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2289,10 +2315,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2304,7 +2330,7 @@
       <c r="T14" t="s">
         <v>154</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2345,10 +2371,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2395,10 +2421,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2410,7 +2436,7 @@
       <c r="T16" t="s">
         <v>155</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2451,10 +2477,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2501,10 +2527,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2516,7 +2542,7 @@
       <c r="T18" t="s">
         <v>156</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2557,10 +2583,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2572,7 +2598,7 @@
       <c r="T19" t="s">
         <v>157</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46258</v>
       </c>
     </row>
@@ -2613,10 +2639,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2628,7 +2654,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2669,10 +2695,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2684,7 +2710,7 @@
       <c r="T21" t="s">
         <v>125</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2722,10 +2748,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2737,7 +2763,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2775,10 +2801,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2787,7 +2813,7 @@
       <c r="S23" t="s">
         <v>148</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -2828,10 +2854,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -2843,7 +2869,7 @@
       <c r="T24" t="s">
         <v>160</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>46253</v>
       </c>
     </row>
@@ -2884,10 +2910,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -2934,10 +2960,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -2949,7 +2975,7 @@
       <c r="T26" t="s">
         <v>161</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -2990,10 +3016,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3040,10 +3066,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3090,10 +3116,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3140,10 +3166,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3155,7 +3181,7 @@
       <c r="T30" t="s">
         <v>162</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3196,10 +3222,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46220</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46253</v>
       </c>
       <c r="R31" t="s">
@@ -3211,7 +3237,7 @@
       <c r="T31" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46252</v>
       </c>
     </row>
@@ -3252,10 +3278,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3302,10 +3328,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3317,7 +3343,7 @@
       <c r="T33" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3358,10 +3384,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>46258</v>
       </c>
       <c r="R34" t="s">
@@ -3373,7 +3399,7 @@
       <c r="T34" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>46258</v>
       </c>
     </row>
@@ -3414,10 +3440,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3464,10 +3490,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3514,10 +3540,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3529,7 +3555,7 @@
       <c r="T37" t="s">
         <v>166</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3570,10 +3596,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3582,7 +3608,7 @@
       <c r="T38" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>45351</v>
       </c>
     </row>
@@ -3623,10 +3649,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3670,10 +3696,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3694,22 +3720,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>173</v>
       </c>
     </row>
@@ -7957,70 +7983,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -8058,10 +8084,10 @@
       <c r="O2" t="s">
         <v>103</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -8105,10 +8131,10 @@
       <c r="O3" t="s">
         <v>82</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -8152,10 +8178,10 @@
       <c r="O4" t="s">
         <v>98</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -8199,10 +8225,10 @@
       <c r="O5" t="s">
         <v>99</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -8246,10 +8272,10 @@
       <c r="O6" t="s">
         <v>96</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -8293,10 +8319,10 @@
       <c r="O7" t="s">
         <v>84</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -8340,10 +8366,10 @@
       <c r="O8" t="s">
         <v>104</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -8387,10 +8413,10 @@
       <c r="O9" t="s">
         <v>93</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -8434,10 +8460,10 @@
       <c r="O10" t="s">
         <v>90</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -8481,10 +8507,10 @@
       <c r="O11" t="s">
         <v>100</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -8528,10 +8554,10 @@
       <c r="O12" t="s">
         <v>83</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -8575,10 +8601,10 @@
       <c r="O13" t="s">
         <v>81</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -8622,10 +8648,10 @@
       <c r="O14" t="s">
         <v>101</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -8669,7 +8695,7 @@
       <c r="O15" t="s">
         <v>95</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -8710,7 +8736,7 @@
       <c r="O16" t="s">
         <v>91</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -8751,10 +8777,10 @@
       <c r="O17" t="s">
         <v>94</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -8798,10 +8824,10 @@
       <c r="O18" t="s">
         <v>92</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -8845,10 +8871,10 @@
       <c r="O19" t="s">
         <v>105</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -8892,10 +8918,10 @@
       <c r="O20" t="s">
         <v>97</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -8939,10 +8965,10 @@
       <c r="O21" t="s">
         <v>106</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -8986,10 +9012,10 @@
       <c r="O22" t="s">
         <v>87</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9027,10 +9053,10 @@
       <c r="O23" t="s">
         <v>291</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -9042,7 +9068,7 @@
       <c r="T23" t="s">
         <v>331</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -9080,10 +9106,10 @@
       <c r="O24" t="s">
         <v>81</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -9095,7 +9121,7 @@
       <c r="T24" t="s">
         <v>332</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -9133,10 +9159,10 @@
       <c r="O25" t="s">
         <v>87</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -9148,7 +9174,7 @@
       <c r="T25" t="s">
         <v>333</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -9186,10 +9212,10 @@
       <c r="O26" t="s">
         <v>101</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -9201,7 +9227,7 @@
       <c r="T26" t="s">
         <v>334</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -9239,10 +9265,10 @@
       <c r="O27" t="s">
         <v>87</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -9254,7 +9280,7 @@
       <c r="T27" t="s">
         <v>335</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -9292,10 +9318,10 @@
       <c r="O28" t="s">
         <v>102</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -9307,7 +9333,7 @@
       <c r="T28" t="s">
         <v>336</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -9345,10 +9371,10 @@
       <c r="O29" t="s">
         <v>99</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -9360,7 +9386,7 @@
       <c r="T29" t="s">
         <v>337</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -9392,7 +9418,7 @@
       <c r="T30" t="s">
         <v>338</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -9424,7 +9450,7 @@
       <c r="T31" t="s">
         <v>339</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -9456,7 +9482,7 @@
       <c r="T32" t="s">
         <v>340</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -9494,10 +9520,10 @@
       <c r="O33" t="s">
         <v>91</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -9509,7 +9535,7 @@
       <c r="T33" t="s">
         <v>319</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -9547,16 +9573,16 @@
       <c r="O34" t="s">
         <v>292</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>148</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -9588,10 +9614,10 @@
       <c r="O35" t="s">
         <v>88</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -9600,7 +9626,7 @@
       <c r="S35" t="s">
         <v>148</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -9638,10 +9664,10 @@
       <c r="O36" t="s">
         <v>92</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -9650,7 +9676,7 @@
       <c r="S36" t="s">
         <v>148</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -9714,10 +9740,10 @@
       <c r="O38" t="s">
         <v>97</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -9726,7 +9752,7 @@
       <c r="S38" t="s">
         <v>148</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -9764,10 +9790,10 @@
       <c r="O39" t="s">
         <v>104</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -9779,7 +9805,7 @@
       <c r="T39" t="s">
         <v>341</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -9811,10 +9837,10 @@
       <c r="O40" t="s">
         <v>101</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -9826,7 +9852,7 @@
       <c r="T40" t="s">
         <v>342</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -9864,10 +9890,10 @@
       <c r="O41" t="s">
         <v>96</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -9879,7 +9905,7 @@
       <c r="T41" t="s">
         <v>343</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -9917,10 +9943,10 @@
       <c r="O42" t="s">
         <v>83</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -9932,7 +9958,7 @@
       <c r="T42" t="s">
         <v>344</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -9970,10 +9996,10 @@
       <c r="O43" t="s">
         <v>85</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -9985,7 +10011,7 @@
       <c r="T43" t="s">
         <v>345</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -10023,10 +10049,10 @@
       <c r="O44" t="s">
         <v>98</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10038,7 +10064,7 @@
       <c r="T44" t="s">
         <v>346</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -10076,10 +10102,10 @@
       <c r="O45" t="s">
         <v>82</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -10091,7 +10117,7 @@
       <c r="T45" t="s">
         <v>347</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -10129,10 +10155,10 @@
       <c r="O46" t="s">
         <v>89</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -10144,7 +10170,7 @@
       <c r="T46" t="s">
         <v>348</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -10159,25 +10185,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>353</v>
       </c>
     </row>
@@ -10839,22 +10865,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>359</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (04/09/2026 11:56)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1237,16 +1237,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1262,7 +1254,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1270,30 +1262,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1593,70 +1567,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1697,10 +1671,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1712,7 +1686,7 @@
       <c r="T2" t="s">
         <v>149</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1753,10 +1727,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1803,10 +1777,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1853,10 +1827,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1868,7 +1842,7 @@
       <c r="T5" t="s">
         <v>150</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -1909,10 +1883,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -1959,10 +1933,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -1974,7 +1948,7 @@
       <c r="T7" t="s">
         <v>151</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2015,10 +1989,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2065,10 +2039,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2080,7 +2054,7 @@
       <c r="T9" t="s">
         <v>152</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2121,10 +2095,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2165,10 +2139,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2180,7 +2154,7 @@
       <c r="T11" t="s">
         <v>153</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46227</v>
       </c>
     </row>
@@ -2221,7 +2195,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2265,10 +2239,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2315,10 +2289,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2330,7 +2304,7 @@
       <c r="T14" t="s">
         <v>154</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2371,10 +2345,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2421,10 +2395,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2436,7 +2410,7 @@
       <c r="T16" t="s">
         <v>155</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2477,10 +2451,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2527,10 +2501,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2542,7 +2516,7 @@
       <c r="T18" t="s">
         <v>156</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2583,10 +2557,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2598,7 +2572,7 @@
       <c r="T19" t="s">
         <v>157</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46258</v>
       </c>
     </row>
@@ -2639,10 +2613,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2654,7 +2628,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2695,10 +2669,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2710,7 +2684,7 @@
       <c r="T21" t="s">
         <v>125</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2748,10 +2722,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2763,7 +2737,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2801,10 +2775,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2813,7 +2787,7 @@
       <c r="S23" t="s">
         <v>148</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -2854,10 +2828,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -2869,7 +2843,7 @@
       <c r="T24" t="s">
         <v>160</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>46253</v>
       </c>
     </row>
@@ -2910,10 +2884,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -2960,10 +2934,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -2975,7 +2949,7 @@
       <c r="T26" t="s">
         <v>161</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3016,10 +2990,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3066,10 +3040,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3116,10 +3090,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3166,10 +3140,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3181,7 +3155,7 @@
       <c r="T30" t="s">
         <v>162</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3222,10 +3196,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46220</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46253</v>
       </c>
       <c r="R31" t="s">
@@ -3237,7 +3211,7 @@
       <c r="T31" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46252</v>
       </c>
     </row>
@@ -3278,10 +3252,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3328,10 +3302,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3343,7 +3317,7 @@
       <c r="T33" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3384,10 +3358,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>46258</v>
       </c>
       <c r="R34" t="s">
@@ -3399,7 +3373,7 @@
       <c r="T34" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>46258</v>
       </c>
     </row>
@@ -3440,10 +3414,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3490,10 +3464,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3540,10 +3514,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3555,7 +3529,7 @@
       <c r="T37" t="s">
         <v>166</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3596,10 +3570,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3608,7 +3582,7 @@
       <c r="T38" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>45351</v>
       </c>
     </row>
@@ -3649,10 +3623,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3696,10 +3670,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3720,22 +3694,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>170</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>171</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>172</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>173</v>
       </c>
     </row>
@@ -7983,70 +7957,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -8084,10 +8058,10 @@
       <c r="O2" t="s">
         <v>103</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -8131,10 +8105,10 @@
       <c r="O3" t="s">
         <v>82</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -8178,10 +8152,10 @@
       <c r="O4" t="s">
         <v>98</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -8225,10 +8199,10 @@
       <c r="O5" t="s">
         <v>99</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -8272,10 +8246,10 @@
       <c r="O6" t="s">
         <v>96</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -8319,10 +8293,10 @@
       <c r="O7" t="s">
         <v>84</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -8366,10 +8340,10 @@
       <c r="O8" t="s">
         <v>104</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -8413,10 +8387,10 @@
       <c r="O9" t="s">
         <v>93</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -8460,10 +8434,10 @@
       <c r="O10" t="s">
         <v>90</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -8507,10 +8481,10 @@
       <c r="O11" t="s">
         <v>100</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -8554,10 +8528,10 @@
       <c r="O12" t="s">
         <v>83</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -8601,10 +8575,10 @@
       <c r="O13" t="s">
         <v>81</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -8648,10 +8622,10 @@
       <c r="O14" t="s">
         <v>101</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -8695,7 +8669,7 @@
       <c r="O15" t="s">
         <v>95</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -8736,7 +8710,7 @@
       <c r="O16" t="s">
         <v>91</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -8777,10 +8751,10 @@
       <c r="O17" t="s">
         <v>94</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -8824,10 +8798,10 @@
       <c r="O18" t="s">
         <v>92</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -8871,10 +8845,10 @@
       <c r="O19" t="s">
         <v>105</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -8918,10 +8892,10 @@
       <c r="O20" t="s">
         <v>97</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -8965,10 +8939,10 @@
       <c r="O21" t="s">
         <v>106</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9012,10 +8986,10 @@
       <c r="O22" t="s">
         <v>87</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9053,10 +9027,10 @@
       <c r="O23" t="s">
         <v>291</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -9068,7 +9042,7 @@
       <c r="T23" t="s">
         <v>331</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -9106,10 +9080,10 @@
       <c r="O24" t="s">
         <v>81</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -9121,7 +9095,7 @@
       <c r="T24" t="s">
         <v>332</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -9159,10 +9133,10 @@
       <c r="O25" t="s">
         <v>87</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -9174,7 +9148,7 @@
       <c r="T25" t="s">
         <v>333</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -9212,10 +9186,10 @@
       <c r="O26" t="s">
         <v>101</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -9227,7 +9201,7 @@
       <c r="T26" t="s">
         <v>334</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -9265,10 +9239,10 @@
       <c r="O27" t="s">
         <v>87</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -9280,7 +9254,7 @@
       <c r="T27" t="s">
         <v>335</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -9318,10 +9292,10 @@
       <c r="O28" t="s">
         <v>102</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -9333,7 +9307,7 @@
       <c r="T28" t="s">
         <v>336</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -9371,10 +9345,10 @@
       <c r="O29" t="s">
         <v>99</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -9386,7 +9360,7 @@
       <c r="T29" t="s">
         <v>337</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -9418,7 +9392,7 @@
       <c r="T30" t="s">
         <v>338</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -9450,7 +9424,7 @@
       <c r="T31" t="s">
         <v>339</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -9482,7 +9456,7 @@
       <c r="T32" t="s">
         <v>340</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -9520,10 +9494,10 @@
       <c r="O33" t="s">
         <v>91</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -9535,7 +9509,7 @@
       <c r="T33" t="s">
         <v>319</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -9573,16 +9547,16 @@
       <c r="O34" t="s">
         <v>292</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>148</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -9614,10 +9588,10 @@
       <c r="O35" t="s">
         <v>88</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -9626,7 +9600,7 @@
       <c r="S35" t="s">
         <v>148</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -9664,10 +9638,10 @@
       <c r="O36" t="s">
         <v>92</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -9676,7 +9650,7 @@
       <c r="S36" t="s">
         <v>148</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -9740,10 +9714,10 @@
       <c r="O38" t="s">
         <v>97</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -9752,7 +9726,7 @@
       <c r="S38" t="s">
         <v>148</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -9790,10 +9764,10 @@
       <c r="O39" t="s">
         <v>104</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -9805,7 +9779,7 @@
       <c r="T39" t="s">
         <v>341</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -9837,10 +9811,10 @@
       <c r="O40" t="s">
         <v>101</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -9852,7 +9826,7 @@
       <c r="T40" t="s">
         <v>342</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -9890,10 +9864,10 @@
       <c r="O41" t="s">
         <v>96</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -9905,7 +9879,7 @@
       <c r="T41" t="s">
         <v>343</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -9943,10 +9917,10 @@
       <c r="O42" t="s">
         <v>83</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -9958,7 +9932,7 @@
       <c r="T42" t="s">
         <v>344</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -9996,10 +9970,10 @@
       <c r="O43" t="s">
         <v>85</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10011,7 +9985,7 @@
       <c r="T43" t="s">
         <v>345</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -10049,10 +10023,10 @@
       <c r="O44" t="s">
         <v>98</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10064,7 +10038,7 @@
       <c r="T44" t="s">
         <v>346</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -10102,10 +10076,10 @@
       <c r="O45" t="s">
         <v>82</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -10117,7 +10091,7 @@
       <c r="T45" t="s">
         <v>347</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -10155,10 +10129,10 @@
       <c r="O46" t="s">
         <v>89</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -10170,7 +10144,7 @@
       <c r="T46" t="s">
         <v>348</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -10185,25 +10159,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>349</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>350</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>351</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>352</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>353</v>
       </c>
     </row>
@@ -10865,22 +10839,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>355</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>356</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>357</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>358</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>359</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (08/09/2026 08:24)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1237,8 +1237,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1254,7 +1262,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1262,12 +1270,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1567,70 +1593,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1671,10 +1697,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>41754</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1686,7 +1712,7 @@
       <c r="T2" t="s">
         <v>149</v>
       </c>
-      <c r="U2" s="1">
+      <c r="U2" s="2">
         <v>46170</v>
       </c>
     </row>
@@ -1727,10 +1753,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>44709</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1777,10 +1803,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>44348</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1827,10 +1853,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>46059</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1842,7 +1868,7 @@
       <c r="T5" t="s">
         <v>150</v>
       </c>
-      <c r="U5" s="1">
+      <c r="U5" s="2">
         <v>46210</v>
       </c>
     </row>
@@ -1883,10 +1909,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>46149</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -1933,10 +1959,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>43731</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -1948,7 +1974,7 @@
       <c r="T7" t="s">
         <v>151</v>
       </c>
-      <c r="U7" s="1">
+      <c r="U7" s="2">
         <v>43507</v>
       </c>
     </row>
@@ -1989,10 +2015,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45511</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2039,10 +2065,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45716</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2054,7 +2080,7 @@
       <c r="T9" t="s">
         <v>152</v>
       </c>
-      <c r="U9" s="1">
+      <c r="U9" s="2">
         <v>44665</v>
       </c>
     </row>
@@ -2095,10 +2121,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>45064</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2139,10 +2165,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>46135</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2154,7 +2180,7 @@
       <c r="T11" t="s">
         <v>153</v>
       </c>
-      <c r="U11" s="1">
+      <c r="U11" s="2">
         <v>46227</v>
       </c>
     </row>
@@ -2195,7 +2221,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2239,10 +2265,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>46199</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2289,10 +2315,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45667</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2304,7 +2330,7 @@
       <c r="T14" t="s">
         <v>154</v>
       </c>
-      <c r="U14" s="1">
+      <c r="U14" s="2">
         <v>46072</v>
       </c>
     </row>
@@ -2345,10 +2371,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>46064</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2395,10 +2421,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>44285</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2410,7 +2436,7 @@
       <c r="T16" t="s">
         <v>155</v>
       </c>
-      <c r="U16" s="1">
+      <c r="U16" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2451,10 +2477,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45922</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2501,10 +2527,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>45930</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2516,7 +2542,7 @@
       <c r="T18" t="s">
         <v>156</v>
       </c>
-      <c r="U18" s="1">
+      <c r="U18" s="2">
         <v>46198</v>
       </c>
     </row>
@@ -2557,10 +2583,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45524</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2572,7 +2598,7 @@
       <c r="T19" t="s">
         <v>157</v>
       </c>
-      <c r="U19" s="1">
+      <c r="U19" s="2">
         <v>46258</v>
       </c>
     </row>
@@ -2613,10 +2639,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>45026</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2628,7 +2654,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="1">
+      <c r="U20" s="2">
         <v>46157</v>
       </c>
     </row>
@@ -2669,10 +2695,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>45159</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2684,7 +2710,7 @@
       <c r="T21" t="s">
         <v>125</v>
       </c>
-      <c r="U21" s="1">
+      <c r="U21" s="2">
         <v>46209</v>
       </c>
     </row>
@@ -2722,10 +2748,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2737,7 +2763,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="1">
+      <c r="U22" s="2">
         <v>45995</v>
       </c>
     </row>
@@ -2775,10 +2801,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>45713</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2787,7 +2813,7 @@
       <c r="S23" t="s">
         <v>148</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -2828,10 +2854,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>46062</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -2843,7 +2869,7 @@
       <c r="T24" t="s">
         <v>160</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>46253</v>
       </c>
     </row>
@@ -2884,10 +2910,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45079</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -2934,10 +2960,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>41346</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -2949,7 +2975,7 @@
       <c r="T26" t="s">
         <v>161</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>46150</v>
       </c>
     </row>
@@ -2990,10 +3016,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45579</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3040,10 +3066,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>46171</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3090,10 +3116,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44320</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3140,10 +3166,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="1">
+      <c r="P30" s="2">
         <v>42661</v>
       </c>
-      <c r="Q30" s="1">
+      <c r="Q30" s="2">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3155,7 +3181,7 @@
       <c r="T30" t="s">
         <v>162</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>45358</v>
       </c>
     </row>
@@ -3196,10 +3222,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="1">
+      <c r="P31" s="2">
         <v>46220</v>
       </c>
-      <c r="Q31" s="1">
+      <c r="Q31" s="2">
         <v>46253</v>
       </c>
       <c r="R31" t="s">
@@ -3211,7 +3237,7 @@
       <c r="T31" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46252</v>
       </c>
     </row>
@@ -3252,10 +3278,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="1">
+      <c r="P32" s="2">
         <v>43797</v>
       </c>
-      <c r="Q32" s="1">
+      <c r="Q32" s="2">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3302,10 +3328,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>42810</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3317,7 +3343,7 @@
       <c r="T33" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>43802</v>
       </c>
     </row>
@@ -3358,10 +3384,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>45070</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>46258</v>
       </c>
       <c r="R34" t="s">
@@ -3373,7 +3399,7 @@
       <c r="T34" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>46258</v>
       </c>
     </row>
@@ -3414,10 +3440,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>43250</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3464,10 +3490,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45841</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3514,10 +3540,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="1">
+      <c r="P37" s="2">
         <v>45105</v>
       </c>
-      <c r="Q37" s="1">
+      <c r="Q37" s="2">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3529,7 +3555,7 @@
       <c r="T37" t="s">
         <v>166</v>
       </c>
-      <c r="U37" s="1">
+      <c r="U37" s="2">
         <v>46184</v>
       </c>
     </row>
@@ -3570,10 +3596,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>45636</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3582,7 +3608,7 @@
       <c r="T38" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>45351</v>
       </c>
     </row>
@@ -3623,10 +3649,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>45831</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3670,10 +3696,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>44287</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3694,22 +3720,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>173</v>
       </c>
     </row>
@@ -7957,70 +7983,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -8058,10 +8084,10 @@
       <c r="O2" t="s">
         <v>103</v>
       </c>
-      <c r="P2" s="1">
+      <c r="P2" s="2">
         <v>45490</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -8105,10 +8131,10 @@
       <c r="O3" t="s">
         <v>82</v>
       </c>
-      <c r="P3" s="1">
+      <c r="P3" s="2">
         <v>45618</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -8152,10 +8178,10 @@
       <c r="O4" t="s">
         <v>98</v>
       </c>
-      <c r="P4" s="1">
+      <c r="P4" s="2">
         <v>45539</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -8199,10 +8225,10 @@
       <c r="O5" t="s">
         <v>99</v>
       </c>
-      <c r="P5" s="1">
+      <c r="P5" s="2">
         <v>45567</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -8246,10 +8272,10 @@
       <c r="O6" t="s">
         <v>96</v>
       </c>
-      <c r="P6" s="1">
+      <c r="P6" s="2">
         <v>45568</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -8293,10 +8319,10 @@
       <c r="O7" t="s">
         <v>84</v>
       </c>
-      <c r="P7" s="1">
+      <c r="P7" s="2">
         <v>45831</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -8340,10 +8366,10 @@
       <c r="O8" t="s">
         <v>104</v>
       </c>
-      <c r="P8" s="1">
+      <c r="P8" s="2">
         <v>45601</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -8387,10 +8413,10 @@
       <c r="O9" t="s">
         <v>93</v>
       </c>
-      <c r="P9" s="1">
+      <c r="P9" s="2">
         <v>45631</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -8434,10 +8460,10 @@
       <c r="O10" t="s">
         <v>90</v>
       </c>
-      <c r="P10" s="1">
+      <c r="P10" s="2">
         <v>43902</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -8481,10 +8507,10 @@
       <c r="O11" t="s">
         <v>100</v>
       </c>
-      <c r="P11" s="1">
+      <c r="P11" s="2">
         <v>44736</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -8528,10 +8554,10 @@
       <c r="O12" t="s">
         <v>83</v>
       </c>
-      <c r="P12" s="1">
+      <c r="P12" s="2">
         <v>45776</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -8575,10 +8601,10 @@
       <c r="O13" t="s">
         <v>81</v>
       </c>
-      <c r="P13" s="1">
+      <c r="P13" s="2">
         <v>45772</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -8622,10 +8648,10 @@
       <c r="O14" t="s">
         <v>101</v>
       </c>
-      <c r="P14" s="1">
+      <c r="P14" s="2">
         <v>45000</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -8669,7 +8695,7 @@
       <c r="O15" t="s">
         <v>95</v>
       </c>
-      <c r="P15" s="1">
+      <c r="P15" s="2">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -8710,7 +8736,7 @@
       <c r="O16" t="s">
         <v>91</v>
       </c>
-      <c r="P16" s="1">
+      <c r="P16" s="2">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -8751,10 +8777,10 @@
       <c r="O17" t="s">
         <v>94</v>
       </c>
-      <c r="P17" s="1">
+      <c r="P17" s="2">
         <v>45371</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -8798,10 +8824,10 @@
       <c r="O18" t="s">
         <v>92</v>
       </c>
-      <c r="P18" s="1">
+      <c r="P18" s="2">
         <v>46001</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -8845,10 +8871,10 @@
       <c r="O19" t="s">
         <v>105</v>
       </c>
-      <c r="P19" s="1">
+      <c r="P19" s="2">
         <v>45436</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -8892,10 +8918,10 @@
       <c r="O20" t="s">
         <v>97</v>
       </c>
-      <c r="P20" s="1">
+      <c r="P20" s="2">
         <v>44372</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -8939,10 +8965,10 @@
       <c r="O21" t="s">
         <v>106</v>
       </c>
-      <c r="P21" s="1">
+      <c r="P21" s="2">
         <v>44362</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -8986,10 +9012,10 @@
       <c r="O22" t="s">
         <v>87</v>
       </c>
-      <c r="P22" s="1">
+      <c r="P22" s="2">
         <v>45511</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9027,10 +9053,10 @@
       <c r="O23" t="s">
         <v>291</v>
       </c>
-      <c r="P23" s="1">
+      <c r="P23" s="2">
         <v>40044</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -9042,7 +9068,7 @@
       <c r="T23" t="s">
         <v>331</v>
       </c>
-      <c r="U23" s="1">
+      <c r="U23" s="2">
         <v>45775</v>
       </c>
     </row>
@@ -9080,10 +9106,10 @@
       <c r="O24" t="s">
         <v>81</v>
       </c>
-      <c r="P24" s="1">
+      <c r="P24" s="2">
         <v>43549</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -9095,7 +9121,7 @@
       <c r="T24" t="s">
         <v>332</v>
       </c>
-      <c r="U24" s="1">
+      <c r="U24" s="2">
         <v>45810</v>
       </c>
     </row>
@@ -9133,10 +9159,10 @@
       <c r="O25" t="s">
         <v>87</v>
       </c>
-      <c r="P25" s="1">
+      <c r="P25" s="2">
         <v>45447</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -9148,7 +9174,7 @@
       <c r="T25" t="s">
         <v>333</v>
       </c>
-      <c r="U25" s="1">
+      <c r="U25" s="2">
         <v>45937</v>
       </c>
     </row>
@@ -9186,10 +9212,10 @@
       <c r="O26" t="s">
         <v>101</v>
       </c>
-      <c r="P26" s="1">
+      <c r="P26" s="2">
         <v>44485</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -9201,7 +9227,7 @@
       <c r="T26" t="s">
         <v>334</v>
       </c>
-      <c r="U26" s="1">
+      <c r="U26" s="2">
         <v>45580</v>
       </c>
     </row>
@@ -9239,10 +9265,10 @@
       <c r="O27" t="s">
         <v>87</v>
       </c>
-      <c r="P27" s="1">
+      <c r="P27" s="2">
         <v>45420</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -9254,7 +9280,7 @@
       <c r="T27" t="s">
         <v>335</v>
       </c>
-      <c r="U27" s="1">
+      <c r="U27" s="2">
         <v>45588</v>
       </c>
     </row>
@@ -9292,10 +9318,10 @@
       <c r="O28" t="s">
         <v>102</v>
       </c>
-      <c r="P28" s="1">
+      <c r="P28" s="2">
         <v>44369</v>
       </c>
-      <c r="Q28" s="1">
+      <c r="Q28" s="2">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -9307,7 +9333,7 @@
       <c r="T28" t="s">
         <v>336</v>
       </c>
-      <c r="U28" s="1">
+      <c r="U28" s="2">
         <v>45831</v>
       </c>
     </row>
@@ -9345,10 +9371,10 @@
       <c r="O29" t="s">
         <v>99</v>
       </c>
-      <c r="P29" s="1">
+      <c r="P29" s="2">
         <v>44652</v>
       </c>
-      <c r="Q29" s="1">
+      <c r="Q29" s="2">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -9360,7 +9386,7 @@
       <c r="T29" t="s">
         <v>337</v>
       </c>
-      <c r="U29" s="1">
+      <c r="U29" s="2">
         <v>45734</v>
       </c>
     </row>
@@ -9392,7 +9418,7 @@
       <c r="T30" t="s">
         <v>338</v>
       </c>
-      <c r="U30" s="1">
+      <c r="U30" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -9424,7 +9450,7 @@
       <c r="T31" t="s">
         <v>339</v>
       </c>
-      <c r="U31" s="1">
+      <c r="U31" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -9456,7 +9482,7 @@
       <c r="T32" t="s">
         <v>340</v>
       </c>
-      <c r="U32" s="1">
+      <c r="U32" s="2">
         <v>46001</v>
       </c>
     </row>
@@ -9494,10 +9520,10 @@
       <c r="O33" t="s">
         <v>91</v>
       </c>
-      <c r="P33" s="1">
+      <c r="P33" s="2">
         <v>43762</v>
       </c>
-      <c r="Q33" s="1">
+      <c r="Q33" s="2">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -9509,7 +9535,7 @@
       <c r="T33" t="s">
         <v>319</v>
       </c>
-      <c r="U33" s="1">
+      <c r="U33" s="2">
         <v>46037</v>
       </c>
     </row>
@@ -9547,16 +9573,16 @@
       <c r="O34" t="s">
         <v>292</v>
       </c>
-      <c r="P34" s="1">
+      <c r="P34" s="2">
         <v>40071</v>
       </c>
-      <c r="Q34" s="1">
+      <c r="Q34" s="2">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>148</v>
       </c>
-      <c r="U34" s="1">
+      <c r="U34" s="2">
         <v>41023</v>
       </c>
     </row>
@@ -9588,10 +9614,10 @@
       <c r="O35" t="s">
         <v>88</v>
       </c>
-      <c r="P35" s="1">
+      <c r="P35" s="2">
         <v>44784</v>
       </c>
-      <c r="Q35" s="1">
+      <c r="Q35" s="2">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -9600,7 +9626,7 @@
       <c r="S35" t="s">
         <v>148</v>
       </c>
-      <c r="U35" s="1">
+      <c r="U35" s="2">
         <v>45259</v>
       </c>
     </row>
@@ -9638,10 +9664,10 @@
       <c r="O36" t="s">
         <v>92</v>
       </c>
-      <c r="P36" s="1">
+      <c r="P36" s="2">
         <v>45103</v>
       </c>
-      <c r="Q36" s="1">
+      <c r="Q36" s="2">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -9650,7 +9676,7 @@
       <c r="S36" t="s">
         <v>148</v>
       </c>
-      <c r="U36" s="1">
+      <c r="U36" s="2">
         <v>46000</v>
       </c>
     </row>
@@ -9714,10 +9740,10 @@
       <c r="O38" t="s">
         <v>97</v>
       </c>
-      <c r="P38" s="1">
+      <c r="P38" s="2">
         <v>38511</v>
       </c>
-      <c r="Q38" s="1">
+      <c r="Q38" s="2">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -9726,7 +9752,7 @@
       <c r="S38" t="s">
         <v>148</v>
       </c>
-      <c r="U38" s="1">
+      <c r="U38" s="2">
         <v>39068</v>
       </c>
     </row>
@@ -9764,10 +9790,10 @@
       <c r="O39" t="s">
         <v>104</v>
       </c>
-      <c r="P39" s="1">
+      <c r="P39" s="2">
         <v>39006</v>
       </c>
-      <c r="Q39" s="1">
+      <c r="Q39" s="2">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -9779,7 +9805,7 @@
       <c r="T39" t="s">
         <v>341</v>
       </c>
-      <c r="U39" s="1">
+      <c r="U39" s="2">
         <v>40568</v>
       </c>
     </row>
@@ -9811,10 +9837,10 @@
       <c r="O40" t="s">
         <v>101</v>
       </c>
-      <c r="P40" s="1">
+      <c r="P40" s="2">
         <v>40836</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="Q40" s="2">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -9826,7 +9852,7 @@
       <c r="T40" t="s">
         <v>342</v>
       </c>
-      <c r="U40" s="1">
+      <c r="U40" s="2">
         <v>42270</v>
       </c>
     </row>
@@ -9864,10 +9890,10 @@
       <c r="O41" t="s">
         <v>96</v>
       </c>
-      <c r="P41" s="1">
+      <c r="P41" s="2">
         <v>42940</v>
       </c>
-      <c r="Q41" s="1">
+      <c r="Q41" s="2">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -9879,7 +9905,7 @@
       <c r="T41" t="s">
         <v>343</v>
       </c>
-      <c r="U41" s="1">
+      <c r="U41" s="2">
         <v>44148</v>
       </c>
     </row>
@@ -9917,10 +9943,10 @@
       <c r="O42" t="s">
         <v>83</v>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="2">
         <v>43696</v>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="2">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -9932,7 +9958,7 @@
       <c r="T42" t="s">
         <v>344</v>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="2">
         <v>43185</v>
       </c>
     </row>
@@ -9970,10 +9996,10 @@
       <c r="O43" t="s">
         <v>85</v>
       </c>
-      <c r="P43" s="1">
+      <c r="P43" s="2">
         <v>43544</v>
       </c>
-      <c r="Q43" s="1">
+      <c r="Q43" s="2">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -9985,7 +10011,7 @@
       <c r="T43" t="s">
         <v>345</v>
       </c>
-      <c r="U43" s="1">
+      <c r="U43" s="2">
         <v>42850</v>
       </c>
     </row>
@@ -10023,10 +10049,10 @@
       <c r="O44" t="s">
         <v>98</v>
       </c>
-      <c r="P44" s="1">
+      <c r="P44" s="2">
         <v>45076</v>
       </c>
-      <c r="Q44" s="1">
+      <c r="Q44" s="2">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10038,7 +10064,7 @@
       <c r="T44" t="s">
         <v>346</v>
       </c>
-      <c r="U44" s="1">
+      <c r="U44" s="2">
         <v>44404</v>
       </c>
     </row>
@@ -10076,10 +10102,10 @@
       <c r="O45" t="s">
         <v>82</v>
       </c>
-      <c r="P45" s="1">
+      <c r="P45" s="2">
         <v>42963</v>
       </c>
-      <c r="Q45" s="1">
+      <c r="Q45" s="2">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -10091,7 +10117,7 @@
       <c r="T45" t="s">
         <v>347</v>
       </c>
-      <c r="U45" s="1">
+      <c r="U45" s="2">
         <v>42698</v>
       </c>
     </row>
@@ -10129,10 +10155,10 @@
       <c r="O46" t="s">
         <v>89</v>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="2">
         <v>45054</v>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="2">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -10144,7 +10170,7 @@
       <c r="T46" t="s">
         <v>348</v>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="2">
         <v>43941</v>
       </c>
     </row>
@@ -10159,25 +10185,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>353</v>
       </c>
     </row>
@@ -10839,22 +10865,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>359</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: motores (08/09/2026 12:05)
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_motores_tratada.xlsx
@@ -1237,16 +1237,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1262,7 +1254,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1270,30 +1262,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1593,70 +1567,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1697,10 +1671,10 @@
       <c r="O2">
         <v>4000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>41754</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>46134</v>
       </c>
       <c r="R2" t="s">
@@ -1712,7 +1686,7 @@
       <c r="T2" t="s">
         <v>149</v>
       </c>
-      <c r="U2" s="2">
+      <c r="U2" s="1">
         <v>46170</v>
       </c>
     </row>
@@ -1753,10 +1727,10 @@
       <c r="O3">
         <v>4000</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>44709</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>44652</v>
       </c>
       <c r="R3" t="s">
@@ -1803,10 +1777,10 @@
       <c r="O4">
         <v>4000</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>44348</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>44348</v>
       </c>
       <c r="R4" t="s">
@@ -1853,10 +1827,10 @@
       <c r="O5">
         <v>4000</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>46059</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>46203</v>
       </c>
       <c r="R5" t="s">
@@ -1868,7 +1842,7 @@
       <c r="T5" t="s">
         <v>150</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="1">
         <v>46210</v>
       </c>
     </row>
@@ -1909,10 +1883,10 @@
       <c r="O6">
         <v>4000</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>46149</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45510</v>
       </c>
       <c r="R6" t="s">
@@ -1959,10 +1933,10 @@
       <c r="O7">
         <v>4000</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>43731</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45301</v>
       </c>
       <c r="R7" t="s">
@@ -1974,7 +1948,7 @@
       <c r="T7" t="s">
         <v>151</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="1">
         <v>43507</v>
       </c>
     </row>
@@ -2015,10 +1989,10 @@
       <c r="O8">
         <v>4000</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45511</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>43725</v>
       </c>
       <c r="R8" t="s">
@@ -2065,10 +2039,10 @@
       <c r="O9">
         <v>4000</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45716</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45716</v>
       </c>
       <c r="R9" t="s">
@@ -2080,7 +2054,7 @@
       <c r="T9" t="s">
         <v>152</v>
       </c>
-      <c r="U9" s="2">
+      <c r="U9" s="1">
         <v>44665</v>
       </c>
     </row>
@@ -2121,10 +2095,10 @@
       <c r="O10">
         <v>4000</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>45064</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>45048</v>
       </c>
       <c r="R10" t="s">
@@ -2165,10 +2139,10 @@
       <c r="O11">
         <v>4000</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>46135</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>46169</v>
       </c>
       <c r="R11" t="s">
@@ -2180,7 +2154,7 @@
       <c r="T11" t="s">
         <v>153</v>
       </c>
-      <c r="U11" s="2">
+      <c r="U11" s="1">
         <v>46227</v>
       </c>
     </row>
@@ -2221,7 +2195,7 @@
       <c r="O12">
         <v>4000</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>46125</v>
       </c>
       <c r="S12" t="s">
@@ -2265,10 +2239,10 @@
       <c r="O13">
         <v>4000</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>46199</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>41861</v>
       </c>
       <c r="R13" t="s">
@@ -2315,10 +2289,10 @@
       <c r="O14">
         <v>4000</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45667</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>46059</v>
       </c>
       <c r="R14" t="s">
@@ -2330,7 +2304,7 @@
       <c r="T14" t="s">
         <v>154</v>
       </c>
-      <c r="U14" s="2">
+      <c r="U14" s="1">
         <v>46072</v>
       </c>
     </row>
@@ -2371,10 +2345,10 @@
       <c r="O15">
         <v>4000</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>46064</v>
       </c>
-      <c r="Q15" s="2">
+      <c r="Q15" s="1">
         <v>43592</v>
       </c>
       <c r="R15" t="s">
@@ -2421,10 +2395,10 @@
       <c r="O16">
         <v>4000</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>44285</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="1">
         <v>45524</v>
       </c>
       <c r="R16" t="s">
@@ -2436,7 +2410,7 @@
       <c r="T16" t="s">
         <v>155</v>
       </c>
-      <c r="U16" s="2">
+      <c r="U16" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2477,10 +2451,10 @@
       <c r="O17">
         <v>4000</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45922</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45061</v>
       </c>
       <c r="R17" t="s">
@@ -2527,10 +2501,10 @@
       <c r="O18">
         <v>4000</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>45930</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>46184</v>
       </c>
       <c r="R18" t="s">
@@ -2542,7 +2516,7 @@
       <c r="T18" t="s">
         <v>156</v>
       </c>
-      <c r="U18" s="2">
+      <c r="U18" s="1">
         <v>46198</v>
       </c>
     </row>
@@ -2583,10 +2557,10 @@
       <c r="O19">
         <v>4000</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45524</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>46014</v>
       </c>
       <c r="R19" t="s">
@@ -2598,7 +2572,7 @@
       <c r="T19" t="s">
         <v>157</v>
       </c>
-      <c r="U19" s="2">
+      <c r="U19" s="1">
         <v>46258</v>
       </c>
     </row>
@@ -2639,10 +2613,10 @@
       <c r="O20">
         <v>4000</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>45026</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>45446</v>
       </c>
       <c r="R20" t="s">
@@ -2654,7 +2628,7 @@
       <c r="T20" t="s">
         <v>158</v>
       </c>
-      <c r="U20" s="2">
+      <c r="U20" s="1">
         <v>46157</v>
       </c>
     </row>
@@ -2695,10 +2669,10 @@
       <c r="O21">
         <v>4000</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>45159</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>46199</v>
       </c>
       <c r="R21" t="s">
@@ -2710,7 +2684,7 @@
       <c r="T21" t="s">
         <v>125</v>
       </c>
-      <c r="U21" s="2">
+      <c r="U21" s="1">
         <v>46209</v>
       </c>
     </row>
@@ -2748,10 +2722,10 @@
       <c r="O22">
         <v>4000</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45922</v>
       </c>
       <c r="R22" t="s">
@@ -2763,7 +2737,7 @@
       <c r="T22" t="s">
         <v>159</v>
       </c>
-      <c r="U22" s="2">
+      <c r="U22" s="1">
         <v>45995</v>
       </c>
     </row>
@@ -2801,10 +2775,10 @@
       <c r="O23">
         <v>4000</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>45713</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>45810</v>
       </c>
       <c r="R23" t="s">
@@ -2813,7 +2787,7 @@
       <c r="S23" t="s">
         <v>148</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -2854,10 +2828,10 @@
       <c r="O24">
         <v>4000</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>46062</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>46220</v>
       </c>
       <c r="R24" t="s">
@@ -2869,7 +2843,7 @@
       <c r="T24" t="s">
         <v>160</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>46253</v>
       </c>
     </row>
@@ -2910,10 +2884,10 @@
       <c r="O25">
         <v>4000</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45079</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45062</v>
       </c>
       <c r="R25" t="s">
@@ -2960,10 +2934,10 @@
       <c r="O26">
         <v>4000</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>41346</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>45916</v>
       </c>
       <c r="R26" t="s">
@@ -2975,7 +2949,7 @@
       <c r="T26" t="s">
         <v>161</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>46150</v>
       </c>
     </row>
@@ -3016,10 +2990,10 @@
       <c r="O27">
         <v>4000</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45579</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45579</v>
       </c>
       <c r="R27" t="s">
@@ -3066,10 +3040,10 @@
       <c r="O28">
         <v>4000</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>46171</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>46149</v>
       </c>
       <c r="R28" t="s">
@@ -3116,10 +3090,10 @@
       <c r="O29">
         <v>4000</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44320</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>44320</v>
       </c>
       <c r="R29" t="s">
@@ -3166,10 +3140,10 @@
       <c r="O30">
         <v>4000</v>
       </c>
-      <c r="P30" s="2">
+      <c r="P30" s="1">
         <v>42661</v>
       </c>
-      <c r="Q30" s="2">
+      <c r="Q30" s="1">
         <v>45252</v>
       </c>
       <c r="R30" t="s">
@@ -3181,7 +3155,7 @@
       <c r="T30" t="s">
         <v>162</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>45358</v>
       </c>
     </row>
@@ -3222,10 +3196,10 @@
       <c r="O31">
         <v>4000</v>
       </c>
-      <c r="P31" s="2">
+      <c r="P31" s="1">
         <v>46220</v>
       </c>
-      <c r="Q31" s="2">
+      <c r="Q31" s="1">
         <v>46253</v>
       </c>
       <c r="R31" t="s">
@@ -3237,7 +3211,7 @@
       <c r="T31" t="s">
         <v>163</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46252</v>
       </c>
     </row>
@@ -3278,10 +3252,10 @@
       <c r="O32">
         <v>4000</v>
       </c>
-      <c r="P32" s="2">
+      <c r="P32" s="1">
         <v>43797</v>
       </c>
-      <c r="Q32" s="2">
+      <c r="Q32" s="1">
         <v>43725</v>
       </c>
       <c r="R32" t="s">
@@ -3328,10 +3302,10 @@
       <c r="O33">
         <v>4000</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>42810</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>43159</v>
       </c>
       <c r="R33" t="s">
@@ -3343,7 +3317,7 @@
       <c r="T33" t="s">
         <v>164</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>43802</v>
       </c>
     </row>
@@ -3384,10 +3358,10 @@
       <c r="O34">
         <v>4000</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>45070</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>46258</v>
       </c>
       <c r="R34" t="s">
@@ -3399,7 +3373,7 @@
       <c r="T34" t="s">
         <v>165</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>46258</v>
       </c>
     </row>
@@ -3440,10 +3414,10 @@
       <c r="O35">
         <v>4000</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>43250</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>41149</v>
       </c>
       <c r="R35" t="s">
@@ -3490,10 +3464,10 @@
       <c r="O36">
         <v>4000</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45841</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>45754</v>
       </c>
       <c r="R36" t="s">
@@ -3540,10 +3514,10 @@
       <c r="O37">
         <v>4000</v>
       </c>
-      <c r="P37" s="2">
+      <c r="P37" s="1">
         <v>45105</v>
       </c>
-      <c r="Q37" s="2">
+      <c r="Q37" s="1">
         <v>45509</v>
       </c>
       <c r="R37" t="s">
@@ -3555,7 +3529,7 @@
       <c r="T37" t="s">
         <v>166</v>
       </c>
-      <c r="U37" s="2">
+      <c r="U37" s="1">
         <v>46184</v>
       </c>
     </row>
@@ -3596,10 +3570,10 @@
       <c r="O38">
         <v>4000</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>45636</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>46219</v>
       </c>
       <c r="S38" t="s">
@@ -3608,7 +3582,7 @@
       <c r="T38" t="s">
         <v>167</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>45351</v>
       </c>
     </row>
@@ -3649,10 +3623,10 @@
       <c r="O39">
         <v>4000</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>45831</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>45740</v>
       </c>
       <c r="S39" t="s">
@@ -3696,10 +3670,10 @@
       <c r="O40">
         <v>4000</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>44287</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>44114</v>
       </c>
       <c r="R40" t="s">
@@ -3720,22 +3694,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>170</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>171</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>172</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>173</v>
       </c>
     </row>
@@ -7983,70 +7957,70 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -8084,10 +8058,10 @@
       <c r="O2" t="s">
         <v>103</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" s="1">
         <v>45490</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="Q2" s="1">
         <v>45015</v>
       </c>
       <c r="R2" t="s">
@@ -8131,10 +8105,10 @@
       <c r="O3" t="s">
         <v>82</v>
       </c>
-      <c r="P3" s="2">
+      <c r="P3" s="1">
         <v>45618</v>
       </c>
-      <c r="Q3" s="2">
+      <c r="Q3" s="1">
         <v>45614</v>
       </c>
       <c r="R3" t="s">
@@ -8178,10 +8152,10 @@
       <c r="O4" t="s">
         <v>98</v>
       </c>
-      <c r="P4" s="2">
+      <c r="P4" s="1">
         <v>45539</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="Q4" s="1">
         <v>45539</v>
       </c>
       <c r="R4" t="s">
@@ -8225,10 +8199,10 @@
       <c r="O5" t="s">
         <v>99</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="1">
         <v>45567</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="1">
         <v>45490</v>
       </c>
       <c r="R5" t="s">
@@ -8272,10 +8246,10 @@
       <c r="O6" t="s">
         <v>96</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="1">
         <v>45568</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="1">
         <v>45526</v>
       </c>
       <c r="R6" t="s">
@@ -8319,10 +8293,10 @@
       <c r="O7" t="s">
         <v>84</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="1">
         <v>45831</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="1">
         <v>45352</v>
       </c>
       <c r="R7" t="s">
@@ -8366,10 +8340,10 @@
       <c r="O8" t="s">
         <v>104</v>
       </c>
-      <c r="P8" s="2">
+      <c r="P8" s="1">
         <v>45601</v>
       </c>
-      <c r="Q8" s="2">
+      <c r="Q8" s="1">
         <v>44704</v>
       </c>
       <c r="R8" t="s">
@@ -8413,10 +8387,10 @@
       <c r="O9" t="s">
         <v>93</v>
       </c>
-      <c r="P9" s="2">
+      <c r="P9" s="1">
         <v>45631</v>
       </c>
-      <c r="Q9" s="2">
+      <c r="Q9" s="1">
         <v>45628</v>
       </c>
       <c r="R9" t="s">
@@ -8460,10 +8434,10 @@
       <c r="O10" t="s">
         <v>90</v>
       </c>
-      <c r="P10" s="2">
+      <c r="P10" s="1">
         <v>43902</v>
       </c>
-      <c r="Q10" s="2">
+      <c r="Q10" s="1">
         <v>43549</v>
       </c>
       <c r="R10" t="s">
@@ -8507,10 +8481,10 @@
       <c r="O11" t="s">
         <v>100</v>
       </c>
-      <c r="P11" s="2">
+      <c r="P11" s="1">
         <v>44736</v>
       </c>
-      <c r="Q11" s="2">
+      <c r="Q11" s="1">
         <v>44735</v>
       </c>
       <c r="R11" t="s">
@@ -8554,10 +8528,10 @@
       <c r="O12" t="s">
         <v>83</v>
       </c>
-      <c r="P12" s="2">
+      <c r="P12" s="1">
         <v>45776</v>
       </c>
-      <c r="Q12" s="2">
+      <c r="Q12" s="1">
         <v>45776</v>
       </c>
       <c r="R12" t="s">
@@ -8601,10 +8575,10 @@
       <c r="O13" t="s">
         <v>81</v>
       </c>
-      <c r="P13" s="2">
+      <c r="P13" s="1">
         <v>45772</v>
       </c>
-      <c r="Q13" s="2">
+      <c r="Q13" s="1">
         <v>45600</v>
       </c>
       <c r="R13" t="s">
@@ -8648,10 +8622,10 @@
       <c r="O14" t="s">
         <v>101</v>
       </c>
-      <c r="P14" s="2">
+      <c r="P14" s="1">
         <v>45000</v>
       </c>
-      <c r="Q14" s="2">
+      <c r="Q14" s="1">
         <v>44630</v>
       </c>
       <c r="R14" t="s">
@@ -8695,7 +8669,7 @@
       <c r="O15" t="s">
         <v>95</v>
       </c>
-      <c r="P15" s="2">
+      <c r="P15" s="1">
         <v>45930</v>
       </c>
       <c r="S15" t="s">
@@ -8736,7 +8710,7 @@
       <c r="O16" t="s">
         <v>91</v>
       </c>
-      <c r="P16" s="2">
+      <c r="P16" s="1">
         <v>46035</v>
       </c>
       <c r="S16" t="s">
@@ -8777,10 +8751,10 @@
       <c r="O17" t="s">
         <v>94</v>
       </c>
-      <c r="P17" s="2">
+      <c r="P17" s="1">
         <v>45371</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="1">
         <v>45026</v>
       </c>
       <c r="R17" t="s">
@@ -8824,10 +8798,10 @@
       <c r="O18" t="s">
         <v>92</v>
       </c>
-      <c r="P18" s="2">
+      <c r="P18" s="1">
         <v>46001</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="1">
         <v>45371</v>
       </c>
       <c r="R18" t="s">
@@ -8871,10 +8845,10 @@
       <c r="O19" t="s">
         <v>105</v>
       </c>
-      <c r="P19" s="2">
+      <c r="P19" s="1">
         <v>45436</v>
       </c>
-      <c r="Q19" s="2">
+      <c r="Q19" s="1">
         <v>45294</v>
       </c>
       <c r="R19" t="s">
@@ -8918,10 +8892,10 @@
       <c r="O20" t="s">
         <v>97</v>
       </c>
-      <c r="P20" s="2">
+      <c r="P20" s="1">
         <v>44372</v>
       </c>
-      <c r="Q20" s="2">
+      <c r="Q20" s="1">
         <v>44369</v>
       </c>
       <c r="R20" t="s">
@@ -8965,10 +8939,10 @@
       <c r="O21" t="s">
         <v>106</v>
       </c>
-      <c r="P21" s="2">
+      <c r="P21" s="1">
         <v>44362</v>
       </c>
-      <c r="Q21" s="2">
+      <c r="Q21" s="1">
         <v>43894</v>
       </c>
       <c r="R21" t="s">
@@ -9012,10 +8986,10 @@
       <c r="O22" t="s">
         <v>87</v>
       </c>
-      <c r="P22" s="2">
+      <c r="P22" s="1">
         <v>45511</v>
       </c>
-      <c r="Q22" s="2">
+      <c r="Q22" s="1">
         <v>45509</v>
       </c>
       <c r="R22" t="s">
@@ -9053,10 +9027,10 @@
       <c r="O23" t="s">
         <v>291</v>
       </c>
-      <c r="P23" s="2">
+      <c r="P23" s="1">
         <v>40044</v>
       </c>
-      <c r="Q23" s="2">
+      <c r="Q23" s="1">
         <v>40126</v>
       </c>
       <c r="R23" t="s">
@@ -9068,7 +9042,7 @@
       <c r="T23" t="s">
         <v>331</v>
       </c>
-      <c r="U23" s="2">
+      <c r="U23" s="1">
         <v>45775</v>
       </c>
     </row>
@@ -9106,10 +9080,10 @@
       <c r="O24" t="s">
         <v>81</v>
       </c>
-      <c r="P24" s="2">
+      <c r="P24" s="1">
         <v>43549</v>
       </c>
-      <c r="Q24" s="2">
+      <c r="Q24" s="1">
         <v>45772</v>
       </c>
       <c r="R24" t="s">
@@ -9121,7 +9095,7 @@
       <c r="T24" t="s">
         <v>332</v>
       </c>
-      <c r="U24" s="2">
+      <c r="U24" s="1">
         <v>45810</v>
       </c>
     </row>
@@ -9159,10 +9133,10 @@
       <c r="O25" t="s">
         <v>87</v>
       </c>
-      <c r="P25" s="2">
+      <c r="P25" s="1">
         <v>45447</v>
       </c>
-      <c r="Q25" s="2">
+      <c r="Q25" s="1">
         <v>45510</v>
       </c>
       <c r="R25" t="s">
@@ -9174,7 +9148,7 @@
       <c r="T25" t="s">
         <v>333</v>
       </c>
-      <c r="U25" s="2">
+      <c r="U25" s="1">
         <v>45937</v>
       </c>
     </row>
@@ -9212,10 +9186,10 @@
       <c r="O26" t="s">
         <v>101</v>
       </c>
-      <c r="P26" s="2">
+      <c r="P26" s="1">
         <v>44485</v>
       </c>
-      <c r="Q26" s="2">
+      <c r="Q26" s="1">
         <v>44959</v>
       </c>
       <c r="R26" t="s">
@@ -9227,7 +9201,7 @@
       <c r="T26" t="s">
         <v>334</v>
       </c>
-      <c r="U26" s="2">
+      <c r="U26" s="1">
         <v>45580</v>
       </c>
     </row>
@@ -9265,10 +9239,10 @@
       <c r="O27" t="s">
         <v>87</v>
       </c>
-      <c r="P27" s="2">
+      <c r="P27" s="1">
         <v>45420</v>
       </c>
-      <c r="Q27" s="2">
+      <c r="Q27" s="1">
         <v>45446</v>
       </c>
       <c r="R27" t="s">
@@ -9280,7 +9254,7 @@
       <c r="T27" t="s">
         <v>335</v>
       </c>
-      <c r="U27" s="2">
+      <c r="U27" s="1">
         <v>45588</v>
       </c>
     </row>
@@ -9318,10 +9292,10 @@
       <c r="O28" t="s">
         <v>102</v>
       </c>
-      <c r="P28" s="2">
+      <c r="P28" s="1">
         <v>44369</v>
       </c>
-      <c r="Q28" s="2">
+      <c r="Q28" s="1">
         <v>45824</v>
       </c>
       <c r="R28" t="s">
@@ -9333,7 +9307,7 @@
       <c r="T28" t="s">
         <v>336</v>
       </c>
-      <c r="U28" s="2">
+      <c r="U28" s="1">
         <v>45831</v>
       </c>
     </row>
@@ -9371,10 +9345,10 @@
       <c r="O29" t="s">
         <v>99</v>
       </c>
-      <c r="P29" s="2">
+      <c r="P29" s="1">
         <v>44652</v>
       </c>
-      <c r="Q29" s="2">
+      <c r="Q29" s="1">
         <v>45567</v>
       </c>
       <c r="R29" t="s">
@@ -9386,7 +9360,7 @@
       <c r="T29" t="s">
         <v>337</v>
       </c>
-      <c r="U29" s="2">
+      <c r="U29" s="1">
         <v>45734</v>
       </c>
     </row>
@@ -9418,7 +9392,7 @@
       <c r="T30" t="s">
         <v>338</v>
       </c>
-      <c r="U30" s="2">
+      <c r="U30" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -9450,7 +9424,7 @@
       <c r="T31" t="s">
         <v>339</v>
       </c>
-      <c r="U31" s="2">
+      <c r="U31" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -9482,7 +9456,7 @@
       <c r="T32" t="s">
         <v>340</v>
       </c>
-      <c r="U32" s="2">
+      <c r="U32" s="1">
         <v>46001</v>
       </c>
     </row>
@@ -9520,10 +9494,10 @@
       <c r="O33" t="s">
         <v>91</v>
       </c>
-      <c r="P33" s="2">
+      <c r="P33" s="1">
         <v>43762</v>
       </c>
-      <c r="Q33" s="2">
+      <c r="Q33" s="1">
         <v>46031</v>
       </c>
       <c r="R33" t="s">
@@ -9535,7 +9509,7 @@
       <c r="T33" t="s">
         <v>319</v>
       </c>
-      <c r="U33" s="2">
+      <c r="U33" s="1">
         <v>46037</v>
       </c>
     </row>
@@ -9573,16 +9547,16 @@
       <c r="O34" t="s">
         <v>292</v>
       </c>
-      <c r="P34" s="2">
+      <c r="P34" s="1">
         <v>40071</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="Q34" s="1">
         <v>41023</v>
       </c>
       <c r="S34" t="s">
         <v>148</v>
       </c>
-      <c r="U34" s="2">
+      <c r="U34" s="1">
         <v>41023</v>
       </c>
     </row>
@@ -9614,10 +9588,10 @@
       <c r="O35" t="s">
         <v>88</v>
       </c>
-      <c r="P35" s="2">
+      <c r="P35" s="1">
         <v>44784</v>
       </c>
-      <c r="Q35" s="2">
+      <c r="Q35" s="1">
         <v>45259</v>
       </c>
       <c r="R35" t="s">
@@ -9626,7 +9600,7 @@
       <c r="S35" t="s">
         <v>148</v>
       </c>
-      <c r="U35" s="2">
+      <c r="U35" s="1">
         <v>45259</v>
       </c>
     </row>
@@ -9664,10 +9638,10 @@
       <c r="O36" t="s">
         <v>92</v>
       </c>
-      <c r="P36" s="2">
+      <c r="P36" s="1">
         <v>45103</v>
       </c>
-      <c r="Q36" s="2">
+      <c r="Q36" s="1">
         <v>46000</v>
       </c>
       <c r="R36" t="s">
@@ -9676,7 +9650,7 @@
       <c r="S36" t="s">
         <v>148</v>
       </c>
-      <c r="U36" s="2">
+      <c r="U36" s="1">
         <v>46000</v>
       </c>
     </row>
@@ -9740,10 +9714,10 @@
       <c r="O38" t="s">
         <v>97</v>
       </c>
-      <c r="P38" s="2">
+      <c r="P38" s="1">
         <v>38511</v>
       </c>
-      <c r="Q38" s="2">
+      <c r="Q38" s="1">
         <v>39068</v>
       </c>
       <c r="R38" t="s">
@@ -9752,7 +9726,7 @@
       <c r="S38" t="s">
         <v>148</v>
       </c>
-      <c r="U38" s="2">
+      <c r="U38" s="1">
         <v>39068</v>
       </c>
     </row>
@@ -9790,10 +9764,10 @@
       <c r="O39" t="s">
         <v>104</v>
       </c>
-      <c r="P39" s="2">
+      <c r="P39" s="1">
         <v>39006</v>
       </c>
-      <c r="Q39" s="2">
+      <c r="Q39" s="1">
         <v>40568</v>
       </c>
       <c r="R39" t="s">
@@ -9805,7 +9779,7 @@
       <c r="T39" t="s">
         <v>341</v>
       </c>
-      <c r="U39" s="2">
+      <c r="U39" s="1">
         <v>40568</v>
       </c>
     </row>
@@ -9837,10 +9811,10 @@
       <c r="O40" t="s">
         <v>101</v>
       </c>
-      <c r="P40" s="2">
+      <c r="P40" s="1">
         <v>40836</v>
       </c>
-      <c r="Q40" s="2">
+      <c r="Q40" s="1">
         <v>42270</v>
       </c>
       <c r="R40" t="s">
@@ -9852,7 +9826,7 @@
       <c r="T40" t="s">
         <v>342</v>
       </c>
-      <c r="U40" s="2">
+      <c r="U40" s="1">
         <v>42270</v>
       </c>
     </row>
@@ -9890,10 +9864,10 @@
       <c r="O41" t="s">
         <v>96</v>
       </c>
-      <c r="P41" s="2">
+      <c r="P41" s="1">
         <v>42940</v>
       </c>
-      <c r="Q41" s="2">
+      <c r="Q41" s="1">
         <v>43494</v>
       </c>
       <c r="R41" t="s">
@@ -9905,7 +9879,7 @@
       <c r="T41" t="s">
         <v>343</v>
       </c>
-      <c r="U41" s="2">
+      <c r="U41" s="1">
         <v>44148</v>
       </c>
     </row>
@@ -9943,10 +9917,10 @@
       <c r="O42" t="s">
         <v>83</v>
       </c>
-      <c r="P42" s="2">
+      <c r="P42" s="1">
         <v>43696</v>
       </c>
-      <c r="Q42" s="2">
+      <c r="Q42" s="1">
         <v>45776</v>
       </c>
       <c r="R42" t="s">
@@ -9958,7 +9932,7 @@
       <c r="T42" t="s">
         <v>344</v>
       </c>
-      <c r="U42" s="2">
+      <c r="U42" s="1">
         <v>43185</v>
       </c>
     </row>
@@ -9996,10 +9970,10 @@
       <c r="O43" t="s">
         <v>85</v>
       </c>
-      <c r="P43" s="2">
+      <c r="P43" s="1">
         <v>43544</v>
       </c>
-      <c r="Q43" s="2">
+      <c r="Q43" s="1">
         <v>45916</v>
       </c>
       <c r="R43" t="s">
@@ -10011,7 +9985,7 @@
       <c r="T43" t="s">
         <v>345</v>
       </c>
-      <c r="U43" s="2">
+      <c r="U43" s="1">
         <v>42850</v>
       </c>
     </row>
@@ -10049,10 +10023,10 @@
       <c r="O44" t="s">
         <v>98</v>
       </c>
-      <c r="P44" s="2">
+      <c r="P44" s="1">
         <v>45076</v>
       </c>
-      <c r="Q44" s="2">
+      <c r="Q44" s="1">
         <v>45539</v>
       </c>
       <c r="R44" t="s">
@@ -10064,7 +10038,7 @@
       <c r="T44" t="s">
         <v>346</v>
       </c>
-      <c r="U44" s="2">
+      <c r="U44" s="1">
         <v>44404</v>
       </c>
     </row>
@@ -10102,10 +10076,10 @@
       <c r="O45" t="s">
         <v>82</v>
       </c>
-      <c r="P45" s="2">
+      <c r="P45" s="1">
         <v>42963</v>
       </c>
-      <c r="Q45" s="2">
+      <c r="Q45" s="1">
         <v>45239</v>
       </c>
       <c r="R45" t="s">
@@ -10117,7 +10091,7 @@
       <c r="T45" t="s">
         <v>347</v>
       </c>
-      <c r="U45" s="2">
+      <c r="U45" s="1">
         <v>42698</v>
       </c>
     </row>
@@ -10155,10 +10129,10 @@
       <c r="O46" t="s">
         <v>89</v>
       </c>
-      <c r="P46" s="2">
+      <c r="P46" s="1">
         <v>45054</v>
       </c>
-      <c r="Q46" s="2">
+      <c r="Q46" s="1">
         <v>45586</v>
       </c>
       <c r="R46" t="s">
@@ -10170,7 +10144,7 @@
       <c r="T46" t="s">
         <v>348</v>
       </c>
-      <c r="U46" s="2">
+      <c r="U46" s="1">
         <v>43941</v>
       </c>
     </row>
@@ -10185,25 +10159,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>168</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>169</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>349</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>350</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>351</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>352</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>353</v>
       </c>
     </row>
@@ -10865,22 +10839,22 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>355</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>356</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>357</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>358</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>359</v>
       </c>
     </row>

</xml_diff>